<commit_message>
Confirm 50mOhm M-wire shunt pitch and update PCB and BOM evidence
</commit_message>
<xml_diff>
--- a/projects/2026-electronics-contest/g-buck/rev-c2/downloads/GBUCK_RevC2_updated_BOM.xlsx
+++ b/projects/2026-electronics-contest/g-buck/rev-c2/downloads/GBUCK_RevC2_updated_BOM.xlsx
@@ -14,7 +14,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="重点变化与待确认" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'使用说明'!$A$1:$B$17</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'使用说明'!$A$1:$B$18</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'使用说明'!$1:$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'采购汇总'!$A$1:$J$47</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'采购汇总'!$1:$1</definedName>
@@ -457,7 +457,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:B17"/>
+  <dimension ref="A1:B18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="23" customWidth="1" min="1" max="1"/>
@@ -484,7 +484,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>当前Rev C2 PCB复核版（120×90mm，提交e4559eb）；不是只按旧Rev B参数表采购。</t>
+          <t>Rev C2 PCB复核版（120×90mm），已按新50mΩ商品图更新RS_IN/OUT机械证据；采购差额以用户确认的B3/Rev B中途补料后为基准。</t>
         </is>
       </c>
     </row>
@@ -568,7 +568,7 @@
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>U1须IR2184PbF，不能直接用已购IR2104；RS_L 25mΩ参数表明确未购齐。</t>
+          <t>U1须IR2184PbF，不能直接用IR2104；RS_L 25mΩ在B3清单中已包含，旧表记未购，现库存待核，不再自动假定库存为0。</t>
         </is>
       </c>
     </row>
@@ -599,77 +599,89 @@
     <row r="12" ht="46" customHeight="1">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>未确认封装</t>
+          <t>分流器新证据</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>分流器P10、双管夹中心距30及槽方向仍为占位；C_A3封装、D1实际封装、外壳固定仍需核对。</t>
+          <t>50mΩ商品图明确P10、线径0.8mm、图示体高12mm、额定5A，适用RS_IN/RS_OUT；不证明1%精度、连续功率或25mΩ的RS_L尺寸。</t>
         </is>
       </c>
     </row>
     <row r="13" ht="46" customHeight="1">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>电感</t>
+          <t>未确认封装</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>65125图示6A Max不是饱和电流保证；源设计仍要求Isat≥3A、Irms≥1.5A、DCR≤0.15Ω。</t>
+          <t>RS_L的P10、双管夹中心距30及槽方向仍为占位；RS_IN/OUT平面包络厚度、C_A3封装、D1实际封装及外壳固定仍需核对。</t>
         </is>
       </c>
     </row>
     <row r="14" ht="46" customHeight="1">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>当前制造状态</t>
+          <t>电感</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>PCB仍有未布连接，客户端打开、原生ERC/DRC未完成；清单提供采购核对依据，不是制板放行。</t>
+          <t>65125图示6A Max不是饱和电流保证；源设计仍要求Isat≥3A、Irms≥1.5A、DCR≤0.15Ω。</t>
         </is>
       </c>
     </row>
     <row r="15" ht="46" customHeight="1">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>本次原理图影响</t>
+          <t>当前制造状态</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>仅整理采购清单，不修改任何引脚、网络、阻容值或原理图文件。</t>
+          <t>PCB仍有未布连接，客户端打开、原生ERC/DRC未完成；清单提供采购核对依据，不是制板放行。</t>
         </is>
       </c>
     </row>
     <row r="16" ht="46" customHeight="1">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>本次器件/PCB影响</t>
+          <t>本次原理图影响</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>相对当前PCB复核版不新增/替换器件或改变封装；把已有变化、辅料和采购建议显式列出。</t>
+          <t>相对523113a，电气引脚、网络和阻容值保持；工程副本同步RS_IN/OUT专用封装关联和说明，原Rev C2源文件保留。</t>
         </is>
       </c>
     </row>
     <row r="17" ht="46" customHeight="1">
       <c r="A17" s="2" t="inlineStr">
         <is>
+          <t>本次器件/PCB影响</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>RS_IN/OUT由通用P10占位改为50mΩ M型专用封装关联，脚距10、孔1.1、焊盘2.6及位置/走线几何保持；未新增或替换实物。RS_L保持待确认。</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="46" customHeight="1">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
           <t>本次仿真/固件影响</t>
         </is>
       </c>
-      <c r="B17" s="2" t="inlineStr">
+      <c r="B18" s="2" t="inlineStr">
         <is>
           <t>没有修改或运行Multisim、ngspice及STM32固件，不据此重新宣称效率或保护实测通过。</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:B17"/>
+  <autoFilter ref="A1:B18"/>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" paperSize="8" fitToHeight="0" fitToWidth="1"/>
@@ -1144,12 +1156,12 @@
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>50mΩ，1%，≥1W</t>
+          <t>50mΩ，1%，≥1W（精度/功率仍待核）</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>直插；P10仅占位，实际脚距待确认</t>
+          <t>M型康铜丝直插；图示P10、线径0.8、体高12mm</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
@@ -1170,12 +1182,12 @@
       </c>
       <c r="I11" s="2" t="inlineStr">
         <is>
-          <t>已有购买记录；规格待核</t>
+          <t>脚距/线径已获商品图支持</t>
         </is>
       </c>
       <c r="J11" s="2" t="inlineStr">
         <is>
-          <t>两端式从器件两端独立Kelvin取样；不要按旧R2512直接采购</t>
+          <t>达科峰图标50mΩ/5A；已有备料可抵扣；连续功率、精度及平面厚度待核；独立Kelvin取样</t>
         </is>
       </c>
     </row>
@@ -1206,21 +1218,19 @@
       <c r="F12" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="G12" s="3" t="n">
-        <v>0</v>
-      </c>
+      <c r="G12" s="3" t="n"/>
       <c r="H12" s="2">
         <f>IF(G12="","",MAX(F12-G12,0))</f>
         <v/>
       </c>
       <c r="I12" s="2" t="inlineStr">
         <is>
-          <t>明确待补购</t>
+          <t>B3已列；现库存待核</t>
         </is>
       </c>
       <c r="J12" s="2" t="inlineStr">
         <is>
-          <t>参数表注明未购齐；选定料号后更新真实封装</t>
+          <t>旧参数表记未购；用户确认中途按B3补料，当前库存未知；50mΩ图不证明本件尺寸</t>
         </is>
       </c>
     </row>
@@ -3388,17 +3398,17 @@
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>SHUNT_TH_P10_TBD</t>
+          <t>SHUNT_M_50m_P10_D0p8</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>50mΩ，1%，≥1W</t>
+          <t>50mΩ，1%，≥1W（精度/功率仍待核）</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>直插；P10仅占位，实际脚距待确认</t>
+          <t>M型康铜丝直插；图示P10、线径0.8、体高12mm</t>
         </is>
       </c>
       <c r="F14" s="2" t="n">
@@ -3409,17 +3419,17 @@
       </c>
       <c r="H14" s="2" t="inlineStr">
         <is>
-          <t>已有购买记录；规格待核</t>
+          <t>脚距/线径已获商品图支持</t>
         </is>
       </c>
       <c r="I14" s="2" t="inlineStr">
         <is>
-          <t>两端式从器件两端独立Kelvin取样；不要按旧R2512直接采购</t>
+          <t>达科峰图标50mΩ/5A；已有备料可抵扣；连续功率、精度及平面厚度待核；独立Kelvin取样</t>
         </is>
       </c>
       <c r="J14" s="2" t="inlineStr">
         <is>
-          <t>已购类型改直插占位；P10仅假设，图片尚未确认本件脚距；高度12、线径0.8来自参数表；功率≥1W；Kelvin取样；RS_L25mΩ尚未购齐</t>
+          <t>用户商品图确认：达科峰M型康铜丝50mΩ、P10、线径0.8、图示体高12、额定5A；孔1.1/焊盘2.6为设计值；平面12×4包络仍为预留；1%精度和连续≥1W待核；Kelvin取样</t>
         </is>
       </c>
     </row>
@@ -3436,17 +3446,17 @@
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>SHUNT_TH_P10_TBD</t>
+          <t>SHUNT_M_50m_P10_D0p8</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>50mΩ，1%，≥1W</t>
+          <t>50mΩ，1%，≥1W（精度/功率仍待核）</t>
         </is>
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>直插；P10仅占位，实际脚距待确认</t>
+          <t>M型康铜丝直插；图示P10、线径0.8、体高12mm</t>
         </is>
       </c>
       <c r="F15" s="2" t="n">
@@ -3457,17 +3467,17 @@
       </c>
       <c r="H15" s="2" t="inlineStr">
         <is>
-          <t>已有购买记录；规格待核</t>
+          <t>脚距/线径已获商品图支持</t>
         </is>
       </c>
       <c r="I15" s="2" t="inlineStr">
         <is>
-          <t>两端式从器件两端独立Kelvin取样；不要按旧R2512直接采购</t>
+          <t>达科峰图标50mΩ/5A；已有备料可抵扣；连续功率、精度及平面厚度待核；独立Kelvin取样</t>
         </is>
       </c>
       <c r="J15" s="2" t="inlineStr">
         <is>
-          <t>已购类型改直插占位；P10仅假设，图片尚未确认本件脚距；高度12、线径0.8来自参数表；功率≥1W；Kelvin取样；RS_L25mΩ尚未购齐</t>
+          <t>用户商品图确认：达科峰M型康铜丝50mΩ、P10、线径0.8、图示体高12、额定5A；孔1.1/焊盘2.6为设计值；平面12×4包络仍为预留；1%精度和连续≥1W待核；Kelvin取样</t>
         </is>
       </c>
     </row>
@@ -3505,17 +3515,17 @@
       </c>
       <c r="H16" s="2" t="inlineStr">
         <is>
-          <t>明确待补购</t>
+          <t>B3已列；现库存待核</t>
         </is>
       </c>
       <c r="I16" s="2" t="inlineStr">
         <is>
-          <t>参数表注明未购齐；选定料号后更新真实封装；参数表明确未购齐</t>
+          <t>旧参数表记未购；用户确认中途按B3补料，当前库存未知；50mΩ图不证明本件尺寸</t>
         </is>
       </c>
       <c r="J16" s="2" t="inlineStr">
         <is>
-          <t>已购类型改直插占位；P10仅假设，图片尚未确认本件脚距；高度12、线径0.8来自参数表；功率≥1W；Kelvin取样；RS_L25mΩ尚未购齐</t>
+          <t>25mΩ已列B3补料清单；旧参数表记未购，现库存待核；本图仅50mΩ，不能套用到本件；P10仍占位；实际封装、1%与≥1W待核</t>
         </is>
       </c>
     </row>
@@ -8809,7 +8819,7 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>参数表注明未购</t>
+          <t>B3已列25mΩ；旧表记未购</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
@@ -8819,7 +8829,7 @@
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>补购并确认真实脚距/功率</t>
+          <t>现库存及真实尺寸待核；不按50mΩ图套用</t>
         </is>
       </c>
     </row>
@@ -8831,17 +8841,17 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>已购物料是直插；旧设计R2512</t>
+          <t>P10原为占位；原设计R2512</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>50mΩ、1%、≥1W；直插</t>
+          <t>50mΩ M型，商品图P10/线径0.8/体高12/额定5A</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>量两脚中心距，P10不是确认值</t>
+          <t>脚距已确认；精度、连续功率和包络厚度待核</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Set RS_L 25mOhm U-wire footprint to confirmed 5mm pitch
</commit_message>
<xml_diff>
--- a/projects/2026-electronics-contest/g-buck/rev-c2/downloads/GBUCK_RevC2_updated_BOM.xlsx
+++ b/projects/2026-electronics-contest/g-buck/rev-c2/downloads/GBUCK_RevC2_updated_BOM.xlsx
@@ -484,7 +484,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Rev C2 PCB复核版（120×90mm），已按新50mΩ商品图更新RS_IN/OUT机械证据；采购差额以用户确认的B3/Rev B中途补料后为基准。</t>
+          <t>Rev C2 PCB复核版（120×90mm），50mΩ P10与25mΩ P5已按用户商品图分别建封装；采购差额以B3/Rev B中途补料后为基准。</t>
         </is>
       </c>
     </row>
@@ -604,7 +604,7 @@
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>50mΩ商品图明确P10、线径0.8mm、图示体高12mm、额定5A，适用RS_IN/RS_OUT；不证明1%精度、连续功率或25mΩ的RS_L尺寸。</t>
+          <t>RS_IN/OUT：50mΩ P10、图示线径0.8、体高12、标称5A；RS_L：25mΩ P5、图示线径0.7、体高7。电阻体线径不自动证明焊接直脚径，精度/连续功率仍待核。</t>
         </is>
       </c>
     </row>
@@ -616,7 +616,7 @@
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>RS_L的P10、双管夹中心距30及槽方向仍为占位；RS_IN/OUT平面包络厚度、C_A3封装、D1实际封装及外壳固定仍需核对。</t>
+          <t>双管夹中心距30及槽方向仍为占位；分流器平面深度、焊脚径和完整包络、C_A3封装、D1实际封装及外壳固定仍需核对。</t>
         </is>
       </c>
     </row>
@@ -652,7 +652,7 @@
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>相对523113a，电气引脚、网络和阻容值保持；工程副本同步RS_IN/OUT专用封装关联和说明，原Rev C2源文件保留。</t>
+          <t>相对9de6ebe，电气引脚、网络和25mΩ数值保持；工程副本更新RS_L专用封装关联和说明，原Rev C2源文件保留。</t>
         </is>
       </c>
     </row>
@@ -664,7 +664,7 @@
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>RS_IN/OUT由通用P10占位改为50mΩ M型专用封装关联，脚距10、孔1.1、焊盘2.6及位置/走线几何保持；未新增或替换实物。RS_L保持待确认。</t>
+          <t>RS_L由P10占位改为用户25mΩ图的U型P5，两个孔/焊盘各向中心移动2.5mm；孔1.1、焊盘2.6、器件中心与其他器件保持。未确认库存、精度或功率。</t>
         </is>
       </c>
     </row>
@@ -1199,12 +1199,12 @@
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>25mΩ，1%，≥1W</t>
+          <t>25mΩ，1%，≥1W（精度/功率仍待核）</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>直插；封装/脚距待选型</t>
+          <t>U型直插；图示P5、线径0.7、体高7mm</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
@@ -1225,12 +1225,12 @@
       </c>
       <c r="I12" s="2" t="inlineStr">
         <is>
-          <t>B3已列；现库存待核</t>
+          <t>25mΩ商品图已给尺寸；库存待核</t>
         </is>
       </c>
       <c r="J12" s="2" t="inlineStr">
         <is>
-          <t>旧参数表记未购；用户确认中途按B3补料，当前库存未知；50mΩ图不证明本件尺寸</t>
+          <t>DILIN迪林商品图；P10占位改P5；图未给精度/功率及实际焊脚径/深度；B3已列，库存未知</t>
         </is>
       </c>
     </row>
@@ -3494,17 +3494,17 @@
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>SHUNT_TH_P10_TBD</t>
+          <t>SHUNT_U_25m_P5_D0p7</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>25mΩ，1%，≥1W</t>
+          <t>25mΩ，1%，≥1W（精度/功率仍待核）</t>
         </is>
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>直插；封装/脚距待选型</t>
+          <t>U型直插；图示P5、线径0.7、体高7mm</t>
         </is>
       </c>
       <c r="F16" s="2" t="n">
@@ -3515,17 +3515,17 @@
       </c>
       <c r="H16" s="2" t="inlineStr">
         <is>
-          <t>B3已列；现库存待核</t>
+          <t>25mΩ商品图已给尺寸；库存待核</t>
         </is>
       </c>
       <c r="I16" s="2" t="inlineStr">
         <is>
-          <t>旧参数表记未购；用户确认中途按B3补料，当前库存未知；50mΩ图不证明本件尺寸</t>
+          <t>DILIN迪林商品图；P10占位改P5；图未给精度/功率及实际焊脚径/深度；B3已列，库存未知</t>
         </is>
       </c>
       <c r="J16" s="2" t="inlineStr">
         <is>
-          <t>25mΩ已列B3补料清单；旧参数表记未购，现库存待核；本图仅50mΩ，不能套用到本件；P10仍占位；实际封装、1%与≥1W待核</t>
+          <t>用户DILIN迪林图确认25mΩ、U型、P5、图示线径0.7、体高7；从P10占位改P5；孔1.1/焊盘2.6及12×4包络为保守设计预留；实际焊脚径、深度、1%精度与连续≥1W待核；库存未知</t>
         </is>
       </c>
     </row>
@@ -8819,17 +8819,17 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>B3已列25mΩ；旧表记未购</t>
+          <t>旧P10占位；库存未知</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>25mΩ、1%、≥1W</t>
+          <t>25mΩ U型；P5、图示线径0.7、体高7</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>现库存及真实尺寸待核；不按50mΩ图套用</t>
+          <t>PCB改P5；精度、连续功率及实际焊脚径/深度仍待核</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Use 5x20 fast fuse clips with confirmed 5.66mm pin pitch
</commit_message>
<xml_diff>
--- a/projects/2026-electronics-contest/g-buck/rev-c2/downloads/GBUCK_RevC2_updated_BOM.xlsx
+++ b/projects/2026-electronics-contest/g-buck/rev-c2/downloads/GBUCK_RevC2_updated_BOM.xlsx
@@ -14,7 +14,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="重点变化与待确认" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'使用说明'!$A$1:$B$18</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'使用说明'!$A$1:$B$19</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'使用说明'!$1:$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'采购汇总'!$A$1:$J$47</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'采购汇总'!$1:$1</definedName>
@@ -457,7 +457,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:B18"/>
+  <dimension ref="A1:B19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="23" customWidth="1" min="1" max="1"/>
@@ -484,7 +484,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Rev C2 PCB复核版（120×90mm），50mΩ P10与25mΩ P5已按用户商品图分别建封装；采购差额以B3/Rev B中途补料后为基准。</t>
+          <t>Rev C2 PCB复核版（120×90mm）；分流器按商品图建库，F1按最新5×20/2A快断和单夹P5.66确认更新；采购差额以B3/Rev B中途补料后为基准。</t>
         </is>
       </c>
     </row>
@@ -611,77 +611,89 @@
     <row r="13" ht="46" customHeight="1">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>未确认封装</t>
+          <t>保险夹确认</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>双管夹中心距30及槽方向仍为占位；分流器平面深度、焊脚径和完整包络、C_A3封装、D1实际封装及外壳固定仍需核对。</t>
+          <t>用户明确单夹脚中心距5.66mm；脚宽1.1/材料厚0.5。槽0.9×1.5及双夹中心距15mm是设计选择，装入5×20实物核对端帽接触/止挡后方可冻结；不能使用旧6×30/7.7尺寸。</t>
         </is>
       </c>
     </row>
     <row r="14" ht="46" customHeight="1">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>电感</t>
+          <t>未确认封装</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>65125图示6A Max不是饱和电流保证；源设计仍要求Isat≥3A、Irms≥1.5A、DCR≤0.15Ω。</t>
+          <t>F1组合间距/方向试装、分流器平面深度及焊脚径/完整包络、C_A3封装、D1实际封装和外壳固定仍需核对。</t>
         </is>
       </c>
     </row>
     <row r="15" ht="46" customHeight="1">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>当前制造状态</t>
+          <t>电感</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>PCB仍有未布连接，客户端打开、原生ERC/DRC未完成；清单提供采购核对依据，不是制板放行。</t>
+          <t>65125图示6A Max不是饱和电流保证；源设计仍要求Isat≥3A、Irms≥1.5A、DCR≤0.15Ω。</t>
         </is>
       </c>
     </row>
     <row r="16" ht="46" customHeight="1">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>本次原理图影响</t>
+          <t>当前制造状态</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>相对9de6ebe，电气引脚、网络和25mΩ数值保持；工程副本更新RS_L专用封装关联和说明，原Rev C2源文件保留。</t>
+          <t>PCB仍有未布连接，客户端打开、原生ERC/DRC未完成；清单提供采购核对依据，不是制板放行。</t>
         </is>
       </c>
     </row>
     <row r="17" ht="46" customHeight="1">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>本次器件/PCB影响</t>
+          <t>本次原理图影响</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>RS_L由P10占位改为用户25mΩ图的U型P5，两个孔/焊盘各向中心移动2.5mm；孔1.1、焊盘2.6、器件中心与其他器件保持。未确认库存、精度或功率。</t>
+          <t>相对6135e14，电气网络/脚号、2A熔断额定及阻容值保持；F1由6×30标注改为5×20 FAST，封装关联/说明同步，源文件保留。</t>
         </is>
       </c>
     </row>
     <row r="18" ht="46" customHeight="1">
       <c r="A18" s="2" t="inlineStr">
         <is>
+          <t>本次器件/PCB影响</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>F1改用最新5×20快断管及P5.66管夹，四孔位置/槽尺寸改变；双夹15mm只作试装初值。分流器和其他器件保持；仿真/固件未改。</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="46" customHeight="1">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
           <t>本次仿真/固件影响</t>
         </is>
       </c>
-      <c r="B18" s="2" t="inlineStr">
+      <c r="B19" s="2" t="inlineStr">
         <is>
           <t>没有修改或运行Multisim、ngspice及STM32固件，不据此重新宣称效率或保护实测通过。</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:B18"/>
+  <autoFilter ref="A1:B19"/>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" paperSize="8" fitToHeight="0" fitToWidth="1"/>
@@ -2532,12 +2544,12 @@
       </c>
       <c r="B43" s="2" t="inlineStr">
         <is>
-          <t>2A保险管，6×30mm</t>
+          <t>2A快断保险管，5×20mm，商品标250V</t>
         </is>
       </c>
       <c r="C43" s="2" t="inlineStr">
         <is>
-          <t>配6×30mm管夹</t>
+          <t>配5×20mm管夹</t>
         </is>
       </c>
       <c r="D43" s="2" t="inlineStr">
@@ -2558,12 +2570,12 @@
       </c>
       <c r="I43" s="2" t="inlineStr">
         <is>
-          <t>快慢断/完整型号待定</t>
+          <t>尺寸/快断已给资料；实际电气性能待核</t>
         </is>
       </c>
       <c r="J43" s="2" t="inlineStr">
         <is>
-          <t>管夹额定10A不等于保险管10A；还需另购2只管夹，见辅料表</t>
+          <t>商品BXG16519；250V未注明AC/DC分断条件，启动不误熔断与故障分断待验证；管夹另列2只</t>
         </is>
       </c>
     </row>
@@ -7297,22 +7309,22 @@
       </c>
       <c r="B100" s="2" t="inlineStr">
         <is>
-          <t>2A / 6x30</t>
+          <t>2A / 5x20 FAST</t>
         </is>
       </c>
       <c r="C100" s="2" t="inlineStr">
         <is>
-          <t>FUSE_6X30_4SLOT_TBD</t>
+          <t>FUSE_5X20_CLIP_P5p66_ASM15_TBD</t>
         </is>
       </c>
       <c r="D100" s="2" t="inlineStr">
         <is>
-          <t>2A保险管，6×30mm</t>
+          <t>2A快断保险管，5×20mm，商品标250V</t>
         </is>
       </c>
       <c r="E100" s="2" t="inlineStr">
         <is>
-          <t>配6×30mm管夹</t>
+          <t>配5×20mm管夹</t>
         </is>
       </c>
       <c r="F100" s="2" t="n">
@@ -7323,17 +7335,17 @@
       </c>
       <c r="H100" s="2" t="inlineStr">
         <is>
-          <t>快慢断/完整型号待定</t>
+          <t>尺寸/快断已给资料；实际电气性能待核</t>
         </is>
       </c>
       <c r="I100" s="2" t="inlineStr">
         <is>
-          <t>管夹额定10A不等于保险管10A；还需另购2只管夹，见辅料表</t>
+          <t>商品BXG16519；250V未注明AC/DC分断条件，启动不误熔断与故障分断待验证；管夹另列2只</t>
         </is>
       </c>
       <c r="J100" s="2" t="inlineStr">
         <is>
-          <t>改用6×30mm管夹；仍需2A保险管；双夹中心距与7.7mm脚距轴向待量；当前4槽为占位，禁止制板</t>
+          <t>最新选型5×20mm、2A快断保险管（商品标250V）；5×20黄铜镀镍夹2只，脚宽1.1/厚0.5/用户确认单夹P5.66；槽0.9×1.5为设计值；两夹中心距15仅试装初值，需验证端帽接触和止挡；旧6×30/7.7作废，禁止直接制板</t>
         </is>
       </c>
     </row>
@@ -8523,7 +8535,7 @@
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>适配6×30mm保险管的管夹，单夹脚距7.7mm</t>
+          <t>5×20mm黄铜镀镍管夹；单夹脚中心距5.66mm</t>
         </is>
       </c>
       <c r="D6" s="2" t="n">
@@ -8536,7 +8548,7 @@
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>配1只F1保险管；图示脚宽1.4、材料厚0.5；两夹中心距/方向待实装核对</t>
+          <t>用户确认5.66是中心距；脚宽1.1/厚0.5；槽0.9×1.5设计值；双夹中心距15仅试装初值，旧6×30尺寸作废</t>
         </is>
       </c>
     </row>
@@ -8863,17 +8875,17 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>旧5×20占位</t>
+          <t>中间采用6×30/7.7，现作废</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>2A、6×30保险管+2只管夹</t>
+          <t>5×20mm、2A快断；配2只P5.66夹</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>7.7mm为单夹脚距；双夹装配间距/方向待核</t>
+          <t>脚宽1.1/厚0.5；四槽更新；双夹15mm试装初值必须实物核对</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Record two SR560 SMD selections and keep diode footprints pending
</commit_message>
<xml_diff>
--- a/projects/2026-electronics-contest/g-buck/rev-c2/downloads/GBUCK_RevC2_updated_BOM.xlsx
+++ b/projects/2026-electronics-contest/g-buck/rev-c2/downloads/GBUCK_RevC2_updated_BOM.xlsx
@@ -14,7 +14,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="重点变化与待确认" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'使用说明'!$A$1:$B$19</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'使用说明'!$A$1:$B$20</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'使用说明'!$1:$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'采购汇总'!$A$1:$J$47</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'采购汇总'!$1:$1</definedName>
@@ -457,7 +457,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:B19"/>
+  <dimension ref="A1:B20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="23" customWidth="1" min="1" max="1"/>
@@ -484,7 +484,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Rev C2 PCB复核版（120×90mm）；分流器按商品图建库，F1按最新5×20/2A快断和单夹P5.66确认更新；采购差额以B3/Rev B中途补料后为基准。</t>
+          <t>当前有效PCB为6f9da6a；用户确认电感立式、D1和D_FREE均选SR560贴片。直插推断已撤回；两只贴片的完整料号/封装仍待核，采购差额以B3补料后为基准。</t>
         </is>
       </c>
     </row>
@@ -623,77 +623,89 @@
     <row r="14" ht="46" customHeight="1">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>未确认封装</t>
+          <t>二极管确认</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>F1组合间距/方向试装、分流器平面深度及焊脚径/完整包络、C_A3封装、D1实际封装和外壳固定仍需核对。</t>
+          <t>D1/D_FREE均按用户SR560贴片意图记录；此前目录SR560是DO-201AD轴向系列，与贴片描述不一致。保留原SMB占位并标待核，未改直插孔或确定SMA/SMB/SMC尺寸。</t>
         </is>
       </c>
     </row>
     <row r="15" ht="46" customHeight="1">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>电感</t>
+          <t>未确认封装</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>65125图示6A Max不是饱和电流保证；源设计仍要求Isat≥3A、Irms≥1.5A、DCR≤0.15Ω。</t>
+          <t>D1/D_FREE真实贴片料号/封装、F1组合试装、分流器完整包络、C_A3封装及外壳固定仍需核对。</t>
         </is>
       </c>
     </row>
     <row r="16" ht="46" customHeight="1">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>当前制造状态</t>
+          <t>电感</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>PCB仍有未布连接，客户端打开、原生ERC/DRC未完成；清单提供采购核对依据，不是制板放行。</t>
+          <t>65125图示6A Max不是饱和电流保证；源设计仍要求Isat≥3A、Irms≥1.5A、DCR≤0.15Ω。</t>
         </is>
       </c>
     </row>
     <row r="17" ht="46" customHeight="1">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>本次原理图影响</t>
+          <t>当前制造状态</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>相对6135e14，电气网络/脚号、2A熔断额定及阻容值保持；F1由6×30标注改为5×20 FAST，封装关联/说明同步，源文件保留。</t>
+          <t>PCB仍有未布连接，客户端打开、原生ERC/DRC未完成；清单提供采购核对依据，不是制板放行。</t>
         </is>
       </c>
     </row>
     <row r="18" ht="46" customHeight="1">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>本次器件/PCB影响</t>
+          <t>本次原理图影响</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>F1改用最新5×20快断管及P5.66管夹，四孔位置/槽尺寸改变；双夹15mm只作试装初值。分流器和其他器件保持；仿真/固件未改。</t>
+          <t>相对6f9da6a，未修改原理图文件、网络或数值；工程内原SS56标注仍为未冻结的占位，采购表另列用户两只SR560贴片选型意图。</t>
         </is>
       </c>
     </row>
     <row r="19" ht="46" customHeight="1">
       <c r="A19" s="2" t="inlineStr">
         <is>
+          <t>本次器件/PCB影响</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>已撤回未提交的D1轴向直插改版，PCB文件恢复为6f9da6a，未更改焊盘/孔位/位置。SR560贴片与原SMB的兼容性未确认，完整料号/尺寸到位后再同步实际封装。</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="46" customHeight="1">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
           <t>本次仿真/固件影响</t>
         </is>
       </c>
-      <c r="B19" s="2" t="inlineStr">
+      <c r="B20" s="2" t="inlineStr">
         <is>
           <t>没有修改或运行Multisim、ngspice及STM32固件，不据此重新宣称效率或保护实测通过。</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:B19"/>
+  <autoFilter ref="A1:B20"/>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" paperSize="8" fitToHeight="0" fitToWidth="1"/>
@@ -1151,12 +1163,12 @@
       </c>
       <c r="I10" s="2" t="inlineStr">
         <is>
-          <t>电气额定待核</t>
+          <t>用户已确认立式；电气额定待核</t>
         </is>
       </c>
       <c r="J10" s="2" t="inlineStr">
         <is>
-          <t>图示220μH/6A Max/DCR≤55mΩ，6A Max不是Isat证明；卧式需换布局</t>
+          <t>沿用当前立式布局；图示6A Max不是Isat证明</t>
         </is>
       </c>
     </row>
@@ -2372,12 +2384,12 @@
       </c>
       <c r="B39" s="2" t="inlineStr">
         <is>
-          <t>SS56，≥60V/≥5A</t>
+          <t>SR560贴片（用户选型）；目标≥60V/≥5A待核</t>
         </is>
       </c>
       <c r="C39" s="2" t="inlineStr">
         <is>
-          <t>SMB / DO-214AA</t>
+          <t>贴片外形待核；原工程SMB仅占位</t>
         </is>
       </c>
       <c r="D39" s="2" t="inlineStr">
@@ -2398,12 +2410,12 @@
       </c>
       <c r="I39" s="2" t="inlineStr">
         <is>
-          <t>D1实际封装待核</t>
+          <t>用户明确两只贴片；厂家完整料号/封装待核</t>
         </is>
       </c>
       <c r="J39" s="2" t="inlineStr">
         <is>
-          <t>共2只；工程定义1=K、2=A；销售商名称不代替完整型号</t>
+          <t>共2只；用户最新明确两个都是SR560贴片。所发DO-201AD轴向表不作为贴片建库依据；需实物丝印/具体订单选项/尺寸图；原工程SS56/SMB不视为兼容性确认</t>
         </is>
       </c>
     </row>
@@ -3383,12 +3395,12 @@
       </c>
       <c r="H13" s="2" t="inlineStr">
         <is>
-          <t>电气额定待核</t>
+          <t>用户已确认立式；电气额定待核</t>
         </is>
       </c>
       <c r="I13" s="2" t="inlineStr">
         <is>
-          <t>图示220μH/6A Max/DCR≤55mΩ，6A Max不是Isat证明；卧式需换布局</t>
+          <t>沿用当前立式布局；图示6A Max不是Isat证明</t>
         </is>
       </c>
       <c r="J13" s="2" t="inlineStr">
@@ -6843,12 +6855,12 @@
       </c>
       <c r="D90" s="2" t="inlineStr">
         <is>
-          <t>SS56，≥60V/≥5A</t>
+          <t>SR560贴片（用户选型）；目标≥60V/≥5A待核</t>
         </is>
       </c>
       <c r="E90" s="2" t="inlineStr">
         <is>
-          <t>SMB / DO-214AA</t>
+          <t>贴片外形待核；原工程SMB仅占位</t>
         </is>
       </c>
       <c r="F90" s="2" t="n">
@@ -6859,12 +6871,12 @@
       </c>
       <c r="H90" s="2" t="inlineStr">
         <is>
-          <t>D1实际封装待核</t>
+          <t>用户明确两只贴片；厂家完整料号/封装待核</t>
         </is>
       </c>
       <c r="I90" s="2" t="inlineStr">
         <is>
-          <t>共2只；工程定义1=K、2=A；销售商名称不代替完整型号</t>
+          <t>共2只；用户最新明确两个都是SR560贴片。所发DO-201AD轴向表不作为贴片建库依据；需实物丝印/具体订单选项/尺寸图；原工程SS56/SMB不视为兼容性确认</t>
         </is>
       </c>
       <c r="J90" s="2" t="inlineStr"/>
@@ -6887,12 +6899,12 @@
       </c>
       <c r="D91" s="2" t="inlineStr">
         <is>
-          <t>SS56，≥60V/≥5A</t>
+          <t>SR560贴片（用户选型）；目标≥60V/≥5A待核</t>
         </is>
       </c>
       <c r="E91" s="2" t="inlineStr">
         <is>
-          <t>SMB / DO-214AA</t>
+          <t>贴片外形待核；原工程SMB仅占位</t>
         </is>
       </c>
       <c r="F91" s="2" t="n">
@@ -6903,12 +6915,12 @@
       </c>
       <c r="H91" s="2" t="inlineStr">
         <is>
-          <t>D1实际封装待核</t>
+          <t>用户明确两只贴片；厂家完整料号/封装待核</t>
         </is>
       </c>
       <c r="I91" s="2" t="inlineStr">
         <is>
-          <t>共2只；工程定义1=K、2=A；销售商名称不代替完整型号</t>
+          <t>共2只；用户最新明确两个都是SR560贴片。所发DO-201AD轴向表不作为贴片建库依据；需实物丝印/具体订单选项/尺寸图；原工程SS56/SMB不视为兼容性确认</t>
         </is>
       </c>
       <c r="J91" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Confirm both SR560 diodes as SMB and synchronize native BOM labels
</commit_message>
<xml_diff>
--- a/projects/2026-electronics-contest/g-buck/rev-c2/downloads/GBUCK_RevC2_updated_BOM.xlsx
+++ b/projects/2026-electronics-contest/g-buck/rev-c2/downloads/GBUCK_RevC2_updated_BOM.xlsx
@@ -484,7 +484,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>当前有效PCB为6f9da6a；用户确认电感立式、D1和D_FREE均选SR560贴片。直插推断已撤回；两只贴片的完整料号/封装仍待核，采购差额以B3补料后为基准。</t>
+          <t>本次比较11bce99；用户已确认电感立式、D1/D_FREE均SR560贴片且为SMB。物料标注与工程同步，焊盘/位置保持；采购差额以B3补料后为基准。</t>
         </is>
       </c>
     </row>
@@ -628,7 +628,7 @@
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>D1/D_FREE均按用户SR560贴片意图记录；此前目录SR560是DO-201AD轴向系列，与贴片描述不一致。保留原SMB占位并标待核，未改直插孔或确定SMA/SMB/SMC尺寸。</t>
+          <t>两只SR560/SMB已由用户明确；沿用现有SMB标准几何，1=K/2=A。DO-201AD图不用于贴片建库，厂家完整电气手册/推荐焊盘最终复核仍需归档。</t>
         </is>
       </c>
     </row>
@@ -640,7 +640,7 @@
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>D1/D_FREE真实贴片料号/封装、F1组合试装、分流器完整包络、C_A3封装及外壳固定仍需核对。</t>
+          <t>F1组合试装、分流器完整包络、C_A3封装及外壳固定仍待核；D1/D_FREE封装类别SMB已确认，真实厂家资料待最终复核。</t>
         </is>
       </c>
     </row>
@@ -676,7 +676,7 @@
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>相对6f9da6a，未修改原理图文件、网络或数值；工程内原SS56标注仍为未冻结的占位，采购表另列用户两只SR560贴片选型意图。</t>
+          <t>相对11bce99，D1/D_FREE物料型号由原SS56标注同步为用户SR560/SMB，网络/电气脚号及阻容值保持；原Rev C2源文件保留。</t>
         </is>
       </c>
     </row>
@@ -688,7 +688,7 @@
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>已撤回未提交的D1轴向直插改版，PCB文件恢复为6f9da6a，未更改焊盘/孔位/位置。SR560贴片与原SMB的兼容性未确认，完整料号/尺寸到位后再同步实际封装。</t>
+          <t>两只二极管的型号/说明更新，沿用SMB焊盘、位置及现有走线；电感立式仅确认原布局。标准封装类别确认不等于厂家数据/实测已通过。</t>
         </is>
       </c>
     </row>
@@ -700,7 +700,7 @@
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>没有修改或运行Multisim、ngspice及STM32固件，不据此重新宣称效率或保护实测通过。</t>
+          <t>未修改或运行Multisim/ngspice/STM32固件，旧器件/功能等效模型未同步为SR560厂家模型，不证明新选型压降、温升、效率或保护实测通过。</t>
         </is>
       </c>
     </row>
@@ -2384,12 +2384,12 @@
       </c>
       <c r="B39" s="2" t="inlineStr">
         <is>
-          <t>SR560贴片（用户选型）；目标≥60V/≥5A待核</t>
+          <t>SR560，目标60V/5A（用户选型）</t>
         </is>
       </c>
       <c r="C39" s="2" t="inlineStr">
         <is>
-          <t>贴片外形待核；原工程SMB仅占位</t>
+          <t>SMB / DO-214AA，贴片</t>
         </is>
       </c>
       <c r="D39" s="2" t="inlineStr">
@@ -2410,12 +2410,12 @@
       </c>
       <c r="I39" s="2" t="inlineStr">
         <is>
-          <t>用户明确两只贴片；厂家完整料号/封装待核</t>
+          <t>用户已确认SMB；厂家资料待最终复核</t>
         </is>
       </c>
       <c r="J39" s="2" t="inlineStr">
         <is>
-          <t>共2只；用户最新明确两个都是SR560贴片。所发DO-201AD轴向表不作为贴片建库依据；需实物丝印/具体订单选项/尺寸图；原工程SS56/SMB不视为兼容性确认</t>
+          <t>共2只；1=K色条端、2=A。沿用原SMB焊盘；SR560为用户确认选型，原轴向目录不作为SMB厂家尺寸/电气手册；完整订货型号/额定条件/推荐焊盘待归档</t>
         </is>
       </c>
     </row>
@@ -3405,7 +3405,7 @@
       </c>
       <c r="J13" s="2" t="inlineStr">
         <is>
-          <t>65125 220μH±10%；DCR≤55mΩ；卖家6A Max≠Isat；立式20×10投影、P10、线径0.75；孔1.1为设计值</t>
+          <t>用户已确认立式；65125 220μH±10%；DCR≤55mΩ；卖家6A Max≠Isat；20×10投影、P10、线径0.75；孔1.1为设计值</t>
         </is>
       </c>
     </row>
@@ -6845,7 +6845,7 @@
       </c>
       <c r="B90" s="2" t="inlineStr">
         <is>
-          <t>SS56</t>
+          <t>SR560 / 60V / 5A</t>
         </is>
       </c>
       <c r="C90" s="2" t="inlineStr">
@@ -6855,12 +6855,12 @@
       </c>
       <c r="D90" s="2" t="inlineStr">
         <is>
-          <t>SR560贴片（用户选型）；目标≥60V/≥5A待核</t>
+          <t>SR560，目标60V/5A（用户选型）</t>
         </is>
       </c>
       <c r="E90" s="2" t="inlineStr">
         <is>
-          <t>贴片外形待核；原工程SMB仅占位</t>
+          <t>SMB / DO-214AA，贴片</t>
         </is>
       </c>
       <c r="F90" s="2" t="n">
@@ -6871,15 +6871,19 @@
       </c>
       <c r="H90" s="2" t="inlineStr">
         <is>
-          <t>用户明确两只贴片；厂家完整料号/封装待核</t>
+          <t>用户已确认SMB；厂家资料待最终复核</t>
         </is>
       </c>
       <c r="I90" s="2" t="inlineStr">
         <is>
-          <t>共2只；用户最新明确两个都是SR560贴片。所发DO-201AD轴向表不作为贴片建库依据；需实物丝印/具体订单选项/尺寸图；原工程SS56/SMB不视为兼容性确认</t>
-        </is>
-      </c>
-      <c r="J90" s="2" t="inlineStr"/>
+          <t>共2只；1=K色条端、2=A。沿用原SMB焊盘；SR560为用户确认选型，原轴向目录不作为SMB厂家尺寸/电气手册；完整订货型号/额定条件/推荐焊盘待归档</t>
+        </is>
+      </c>
+      <c r="J90" s="2" t="inlineStr">
+        <is>
+          <t>用户明确SR560贴片、SMB（DO-214AA）；沿用现有SMB焊盘和位置；1=K色条端接V_SHUNT_IN、2=A接IN_PRE；厂家完整料号、额定条件及推荐焊盘最终复核待归档，不采用DO-201AD轴向目录尺寸</t>
+        </is>
+      </c>
     </row>
     <row r="91" ht="58" customHeight="1">
       <c r="A91" s="2" t="inlineStr">
@@ -6889,7 +6893,7 @@
       </c>
       <c r="B91" s="2" t="inlineStr">
         <is>
-          <t>SS56 / 60V / 5A</t>
+          <t>SR560 / 60V / 5A</t>
         </is>
       </c>
       <c r="C91" s="2" t="inlineStr">
@@ -6899,12 +6903,12 @@
       </c>
       <c r="D91" s="2" t="inlineStr">
         <is>
-          <t>SR560贴片（用户选型）；目标≥60V/≥5A待核</t>
+          <t>SR560，目标60V/5A（用户选型）</t>
         </is>
       </c>
       <c r="E91" s="2" t="inlineStr">
         <is>
-          <t>贴片外形待核；原工程SMB仅占位</t>
+          <t>SMB / DO-214AA，贴片</t>
         </is>
       </c>
       <c r="F91" s="2" t="n">
@@ -6915,17 +6919,17 @@
       </c>
       <c r="H91" s="2" t="inlineStr">
         <is>
-          <t>用户明确两只贴片；厂家完整料号/封装待核</t>
+          <t>用户已确认SMB；厂家资料待最终复核</t>
         </is>
       </c>
       <c r="I91" s="2" t="inlineStr">
         <is>
-          <t>共2只；用户最新明确两个都是SR560贴片。所发DO-201AD轴向表不作为贴片建库依据；需实物丝印/具体订单选项/尺寸图；原工程SS56/SMB不视为兼容性确认</t>
+          <t>共2只；1=K色条端、2=A。沿用原SMB焊盘；SR560为用户确认选型，原轴向目录不作为SMB厂家尺寸/电气手册；完整订货型号/额定条件/推荐焊盘待归档</t>
         </is>
       </c>
       <c r="J91" s="2" t="inlineStr">
         <is>
-          <t>阴极1接SW，阳极2接GND；紧贴QL；不可承诺消除全部Qrr</t>
+          <t>用户明确与D1均SR560贴片、SMB（DO-214AA）；沿用现有SMB焊盘和位置；1=K色条端接SW、2=A接GND；厂家电气/热条件及推荐焊盘最终复核待归档</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Confirm C_A3 as 0805 and preserve reviewed component placements
</commit_message>
<xml_diff>
--- a/projects/2026-electronics-contest/g-buck/rev-c2/downloads/GBUCK_RevC2_updated_BOM.xlsx
+++ b/projects/2026-electronics-contest/g-buck/rev-c2/downloads/GBUCK_RevC2_updated_BOM.xlsx
@@ -16,7 +16,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'使用说明'!$A$1:$B$20</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'使用说明'!$1:$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'采购汇总'!$A$1:$J$47</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'采购汇总'!$A$1:$J$46</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'采购汇总'!$1:$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'逐位号_120项'!$A$1:$J$121</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="2">'逐位号_120项'!$1:$1</definedName>
@@ -484,7 +484,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>本次比较11bce99；用户已确认电感立式、D1/D_FREE均SR560贴片且为SMB。物料标注与工程同步，焊盘/位置保持；采购差额以B3补料后为基准。</t>
+          <t>本次比较c3892ab；用户确认C_A3为0805，由原1206占位改0805，10μF/25V保持；采购差额继续以B3补料后为基准。</t>
         </is>
       </c>
     </row>
@@ -640,7 +640,7 @@
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>F1组合试装、分流器完整包络、C_A3封装及外壳固定仍待核；D1/D_FREE封装类别SMB已确认，真实厂家资料待最终复核。</t>
+          <t>C_A3的0805类别已确认；F1组合试装、分流器完整包络及外壳固定仍待核。C_A3完整料号/介质/偏压有效容量、二极管厂家数据待最终复核。</t>
         </is>
       </c>
     </row>
@@ -676,7 +676,7 @@
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>相对11bce99，D1/D_FREE物料型号由原SS56标注同步为用户SR560/SMB，网络/电气脚号及阻容值保持；原Rev C2源文件保留。</t>
+          <t>相对c3892ab，C_A3仅改封装关联/说明，10μF/25V及全部电气网络和脚号保持；原Rev C2源文件保留。</t>
         </is>
       </c>
     </row>
@@ -688,7 +688,7 @@
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>两只二极管的型号/说明更新，沿用SMB焊盘、位置及现有走线；电感立式仅确认原布局。标准封装类别确认不等于厂家数据/实测已通过。</t>
+          <t>C_A3由C1206改C0805，铜焊盘尺寸及中心距改变；保留全部器件中心/角度。C6/C_A3采购合并为同规格2只，45项合并行、120位号，不重复计料。</t>
         </is>
       </c>
     </row>
@@ -718,7 +718,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:J47"/>
+  <dimension ref="A1:J46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -1534,14 +1534,14 @@
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t>C6</t>
+          <t>C6、C_A3</t>
         </is>
       </c>
       <c r="E19" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F19" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G19" s="3" t="n"/>
       <c r="H19" s="2">
@@ -1550,12 +1550,12 @@
       </c>
       <c r="I19" s="2" t="inlineStr">
         <is>
-          <t>核对实物料号</t>
+          <t>两只0805已确认；完整料号/介质待核</t>
         </is>
       </c>
       <c r="J19" s="2" t="inlineStr">
         <is>
-          <t>按参数表2×1.25mm改0805；介质和有效容量待核</t>
+          <t>共2只；C6来自原参数表，C_A3本轮由用户明确0805并替换原1206占位；实际介质与偏压后容量待核，库存另填</t>
         </is>
       </c>
     </row>
@@ -1567,24 +1567,24 @@
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>10μF/25V，建议X7R</t>
+          <t>100nF/50V，X7R（统一采购建议）</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>1206，暂保留</t>
+          <t>0805</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t>C_A3</t>
+          <t>C5、C_U2、C_U3、C_U4、C_A2、C_REF_POS、C_REF_NEG、C_REF_OV、C_U5、C_U9、C11、C_U6、C_U7、C_U8、C_REF_IOUT、C_IOUT_PROT</t>
         </is>
       </c>
       <c r="E20" s="2" t="n">
-        <v>1</v>
+        <v>16</v>
       </c>
       <c r="F20" s="2" t="n">
-        <v>1</v>
+        <v>16</v>
       </c>
       <c r="G20" s="3" t="n"/>
       <c r="H20" s="2">
@@ -1593,12 +1593,12 @@
       </c>
       <c r="I20" s="2" t="inlineStr">
         <is>
-          <t>封装待确认</t>
+          <t>料号需纠错</t>
         </is>
       </c>
       <c r="J20" s="2" t="inlineStr">
         <is>
-          <t>参数表未填写本件；不能从C6推断为0805</t>
+          <t>合计16只；C_IOUT_PROT源要求25V，其余按原参数表50V统一采购；472是4.7nF，不能代用100nF</t>
         </is>
       </c>
     </row>
@@ -1610,7 +1610,7 @@
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>100nF/50V，X7R（统一采购建议）</t>
+          <t>4.7nF/50V，建议统一C0G/NP0</t>
         </is>
       </c>
       <c r="C21" s="2" t="inlineStr">
@@ -1620,14 +1620,14 @@
       </c>
       <c r="D21" s="2" t="inlineStr">
         <is>
-          <t>C5、C_U2、C_U3、C_U4、C_A2、C_REF_POS、C_REF_NEG、C_REF_OV、C_U5、C_U9、C11、C_U6、C_U7、C_U8、C_REF_IOUT、C_IOUT_PROT</t>
+          <t>C7、C8、C9、C10、C_VINP_ADC</t>
         </is>
       </c>
       <c r="E21" s="2" t="n">
-        <v>16</v>
+        <v>5</v>
       </c>
       <c r="F21" s="2" t="n">
-        <v>16</v>
+        <v>5</v>
       </c>
       <c r="G21" s="3" t="n"/>
       <c r="H21" s="2">
@@ -1636,12 +1636,12 @@
       </c>
       <c r="I21" s="2" t="inlineStr">
         <is>
-          <t>料号需纠错</t>
+          <t>核对已购物料</t>
         </is>
       </c>
       <c r="J21" s="2" t="inlineStr">
         <is>
-          <t>合计16只；C_IOUT_PROT源要求25V，其余按原参数表50V统一采购；472是4.7nF，不能代用100nF</t>
+          <t>共5只；C_VINP_ADC明确C0G，其余按源要求可选相容介质；不把它们当100nF</t>
         </is>
       </c>
     </row>
@@ -1653,7 +1653,7 @@
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>4.7nF/50V，建议统一C0G/NP0</t>
+          <t>1nF/50V，建议C0G/NP0</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
@@ -1663,14 +1663,14 @@
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t>C7、C8、C9、C10、C_VINP_ADC</t>
+          <t>C_IL_ADC、C_IL_PROT</t>
         </is>
       </c>
       <c r="E22" s="2" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="F22" s="2" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="G22" s="3" t="n"/>
       <c r="H22" s="2">
@@ -1684,7 +1684,7 @@
       </c>
       <c r="J22" s="2" t="inlineStr">
         <is>
-          <t>共5只；C_VINP_ADC明确C0G，其余按源要求可选相容介质；不把它们当100nF</t>
+          <t>正常装配2只；C_IL_PROT明确C0G</t>
         </is>
       </c>
     </row>
@@ -1696,7 +1696,7 @@
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>1nF/50V，建议C0G/NP0</t>
+          <t>1nF/100V，C0G/NP0，DNP</t>
         </is>
       </c>
       <c r="C23" s="2" t="inlineStr">
@@ -1706,14 +1706,14 @@
       </c>
       <c r="D23" s="2" t="inlineStr">
         <is>
-          <t>C_IL_ADC、C_IL_PROT</t>
+          <t>C_SN</t>
         </is>
       </c>
       <c r="E23" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F23" s="2" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G23" s="3" t="n"/>
       <c r="H23" s="2">
@@ -1722,24 +1722,24 @@
       </c>
       <c r="I23" s="2" t="inlineStr">
         <is>
-          <t>核对已购物料</t>
+          <t>DNP，默认不装</t>
         </is>
       </c>
       <c r="J23" s="2" t="inlineStr">
         <is>
-          <t>正常装配2只；C_IL_PROT明确C0G</t>
+          <t>吸收电路预留，实测振铃后决定是否装配及调值</t>
         </is>
       </c>
     </row>
     <row r="24" ht="58" customHeight="1">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>贴片电容</t>
+          <t>普通电阻</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>1nF/100V，C0G/NP0，DNP</t>
+          <t>4.7Ω，建议1%、≥0.125W</t>
         </is>
       </c>
       <c r="C24" s="2" t="inlineStr">
@@ -1749,14 +1749,14 @@
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>C_SN</t>
+          <t>RG_H、RG_L</t>
         </is>
       </c>
       <c r="E24" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F24" s="2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G24" s="3" t="n"/>
       <c r="H24" s="2">
@@ -1765,12 +1765,12 @@
       </c>
       <c r="I24" s="2" t="inlineStr">
         <is>
-          <t>DNP，默认不装</t>
+          <t>核对已购物料</t>
         </is>
       </c>
       <c r="J24" s="2" t="inlineStr">
         <is>
-          <t>吸收电路预留，实测振铃后决定是否装配及调值</t>
+          <t>不要沿用Rev B中的旧栅极电阻值</t>
         </is>
       </c>
     </row>
@@ -1782,7 +1782,7 @@
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>4.7Ω，建议1%、≥0.125W</t>
+          <t>1Ω，建议1%、≥0.125W</t>
         </is>
       </c>
       <c r="C25" s="2" t="inlineStr">
@@ -1792,14 +1792,14 @@
       </c>
       <c r="D25" s="2" t="inlineStr">
         <is>
-          <t>RG_H、RG_L</t>
+          <t>R_VDDA</t>
         </is>
       </c>
       <c r="E25" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F25" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G25" s="3" t="n"/>
       <c r="H25" s="2">
@@ -1813,7 +1813,7 @@
       </c>
       <c r="J25" s="2" t="inlineStr">
         <is>
-          <t>不要沿用Rev B中的旧栅极电阻值</t>
+          <t>模拟电源串联电阻，不能错装成0Ω</t>
         </is>
       </c>
     </row>
@@ -1825,7 +1825,7 @@
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>1Ω，建议1%、≥0.125W</t>
+          <t>100Ω，建议1%、≥0.125W</t>
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr">
@@ -1835,7 +1835,7 @@
       </c>
       <c r="D26" s="2" t="inlineStr">
         <is>
-          <t>R_VDDA</t>
+          <t>R_PWM</t>
         </is>
       </c>
       <c r="E26" s="2" t="n">
@@ -1856,7 +1856,7 @@
       </c>
       <c r="J26" s="2" t="inlineStr">
         <is>
-          <t>模拟电源串联电阻，不能错装成0Ω</t>
+          <t>与100Ω/0.1%精密电阻分开采购</t>
         </is>
       </c>
     </row>
@@ -1868,7 +1868,7 @@
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>100Ω，建议1%、≥0.125W</t>
+          <t>1kΩ，1%、≥0.125W（统一采购建议）</t>
         </is>
       </c>
       <c r="C27" s="2" t="inlineStr">
@@ -1878,14 +1878,14 @@
       </c>
       <c r="D27" s="2" t="inlineStr">
         <is>
-          <t>R_PWM</t>
+          <t>R3、R6、R7、R8、R_IL_ADC、R_VINP_ADC、R_IL_PROT、R_IOUT_PROT</t>
         </is>
       </c>
       <c r="E27" s="2" t="n">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="F27" s="2" t="n">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="G27" s="3" t="n"/>
       <c r="H27" s="2">
@@ -1899,7 +1899,7 @@
       </c>
       <c r="J27" s="2" t="inlineStr">
         <is>
-          <t>与100Ω/0.1%精密电阻分开采购</t>
+          <t>共8只；两项保护电阻明确要求1%；原图其余未明确精度，建议统一1%</t>
         </is>
       </c>
     </row>
@@ -1911,7 +1911,7 @@
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>1kΩ，1%、≥0.125W（统一采购建议）</t>
+          <t>10kΩ，建议1%、≥0.125W</t>
         </is>
       </c>
       <c r="C28" s="2" t="inlineStr">
@@ -1921,14 +1921,14 @@
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t>R3、R6、R7、R8、R_IL_ADC、R_VINP_ADC、R_IL_PROT、R_IOUT_PROT</t>
+          <t>R_GSH、R_GSL、R_IN_PD、R_SD_PD、R12、R13、R14、R_EN_PD、R_ARM_PD、R_IOUT_PU</t>
         </is>
       </c>
       <c r="E28" s="2" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="F28" s="2" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="G28" s="3" t="n"/>
       <c r="H28" s="2">
@@ -1942,7 +1942,7 @@
       </c>
       <c r="J28" s="2" t="inlineStr">
         <is>
-          <t>共8只；两项保护电阻明确要求1%；原图其余未明确精度，建议统一1%</t>
+          <t>普通10kΩ共10只；不替代0.1%分压/参考电阻</t>
         </is>
       </c>
     </row>
@@ -1954,7 +1954,7 @@
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>10kΩ，建议1%、≥0.125W</t>
+          <t>23kΩ，建议1%、≥0.125W</t>
         </is>
       </c>
       <c r="C29" s="2" t="inlineStr">
@@ -1964,14 +1964,14 @@
       </c>
       <c r="D29" s="2" t="inlineStr">
         <is>
-          <t>R_GSH、R_GSL、R_IN_PD、R_SD_PD、R12、R13、R14、R_EN_PD、R_ARM_PD、R_IOUT_PU</t>
+          <t>R11</t>
         </is>
       </c>
       <c r="E29" s="2" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="F29" s="2" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="G29" s="3" t="n"/>
       <c r="H29" s="2">
@@ -1985,19 +1985,19 @@
       </c>
       <c r="J29" s="2" t="inlineStr">
         <is>
-          <t>普通10kΩ共10只；不替代0.1%分压/参考电阻</t>
+          <t>按23kΩ采购；不直接换成22kΩ</t>
         </is>
       </c>
     </row>
     <row r="30" ht="58" customHeight="1">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>普通电阻</t>
+          <t>精密电阻</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>23kΩ，建议1%、≥0.125W</t>
+          <t>100kΩ，0.1%，≥0.125W</t>
         </is>
       </c>
       <c r="C30" s="2" t="inlineStr">
@@ -2007,14 +2007,14 @@
       </c>
       <c r="D30" s="2" t="inlineStr">
         <is>
-          <t>R11</t>
+          <t>R1、R_VINP_TOP</t>
         </is>
       </c>
       <c r="E30" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F30" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G30" s="3" t="n"/>
       <c r="H30" s="2">
@@ -2023,12 +2023,12 @@
       </c>
       <c r="I30" s="2" t="inlineStr">
         <is>
-          <t>核对已购物料</t>
+          <t>精度/料号待核</t>
         </is>
       </c>
       <c r="J30" s="2" t="inlineStr">
         <is>
-          <t>按23kΩ采购；不直接换成22kΩ</t>
+          <t>温漂未在源图固定；按实购物料记录，不虚构已确认参数</t>
         </is>
       </c>
     </row>
@@ -2040,7 +2040,7 @@
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>100kΩ，0.1%，≥0.125W</t>
+          <t>10kΩ，0.1%，≥0.125W</t>
         </is>
       </c>
       <c r="C31" s="2" t="inlineStr">
@@ -2050,14 +2050,14 @@
       </c>
       <c r="D31" s="2" t="inlineStr">
         <is>
-          <t>R1、R_VINP_TOP</t>
+          <t>R2、R4、R9、R16、R_IOUT_BOT、R_VINP_BOT</t>
         </is>
       </c>
       <c r="E31" s="2" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="F31" s="2" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="G31" s="3" t="n"/>
       <c r="H31" s="2">
@@ -2071,7 +2071,7 @@
       </c>
       <c r="J31" s="2" t="inlineStr">
         <is>
-          <t>温漂未在源图固定；按实购物料记录，不虚构已确认参数</t>
+          <t>共6只，与普通10kΩ区分</t>
         </is>
       </c>
     </row>
@@ -2083,7 +2083,7 @@
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>10kΩ，0.1%，≥0.125W</t>
+          <t>1kΩ，0.1%，≥0.125W</t>
         </is>
       </c>
       <c r="C32" s="2" t="inlineStr">
@@ -2093,14 +2093,14 @@
       </c>
       <c r="D32" s="2" t="inlineStr">
         <is>
-          <t>R2、R4、R9、R16、R_IOUT_BOT、R_VINP_BOT</t>
+          <t>R5</t>
         </is>
       </c>
       <c r="E32" s="2" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="F32" s="2" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="G32" s="3" t="n"/>
       <c r="H32" s="2">
@@ -2114,7 +2114,7 @@
       </c>
       <c r="J32" s="2" t="inlineStr">
         <is>
-          <t>共6只，与普通10kΩ区分</t>
+          <t>与普通1kΩ区分</t>
         </is>
       </c>
     </row>
@@ -2126,7 +2126,7 @@
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>1kΩ，0.1%，≥0.125W</t>
+          <t>49.9kΩ，0.1%，≥0.125W</t>
         </is>
       </c>
       <c r="C33" s="2" t="inlineStr">
@@ -2136,14 +2136,14 @@
       </c>
       <c r="D33" s="2" t="inlineStr">
         <is>
-          <t>R5</t>
+          <t>R10A、R15A</t>
         </is>
       </c>
       <c r="E33" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F33" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G33" s="3" t="n"/>
       <c r="H33" s="2">
@@ -2157,7 +2157,7 @@
       </c>
       <c r="J33" s="2" t="inlineStr">
         <is>
-          <t>与普通1kΩ区分</t>
+          <t>保留49.9kΩ，不用近似值替代</t>
         </is>
       </c>
     </row>
@@ -2169,7 +2169,7 @@
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>49.9kΩ，0.1%，≥0.125W</t>
+          <t>100Ω，0.1%，≥0.125W</t>
         </is>
       </c>
       <c r="C34" s="2" t="inlineStr">
@@ -2179,7 +2179,7 @@
       </c>
       <c r="D34" s="2" t="inlineStr">
         <is>
-          <t>R10A、R15A</t>
+          <t>R10B、R15B</t>
         </is>
       </c>
       <c r="E34" s="2" t="n">
@@ -2200,7 +2200,7 @@
       </c>
       <c r="J34" s="2" t="inlineStr">
         <is>
-          <t>保留49.9kΩ，不用近似值替代</t>
+          <t>共2只，与R_PWM分开</t>
         </is>
       </c>
     </row>
@@ -2212,7 +2212,7 @@
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t>100Ω，0.1%，≥0.125W</t>
+          <t>20kΩ，0.1%，≥0.125W</t>
         </is>
       </c>
       <c r="C35" s="2" t="inlineStr">
@@ -2222,14 +2222,14 @@
       </c>
       <c r="D35" s="2" t="inlineStr">
         <is>
-          <t>R10B、R15B</t>
+          <t>R_IOUT_TOP</t>
         </is>
       </c>
       <c r="E35" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F35" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G35" s="3" t="n"/>
       <c r="H35" s="2">
@@ -2243,29 +2243,29 @@
       </c>
       <c r="J35" s="2" t="inlineStr">
         <is>
-          <t>共2只，与R_PWM分开</t>
+          <t>输出告警参考上臂</t>
         </is>
       </c>
     </row>
     <row r="36" ht="58" customHeight="1">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>精密电阻</t>
+          <t>功率电阻</t>
         </is>
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>20kΩ，0.1%，≥0.125W</t>
+          <t>2.2kΩ，≥0.25W</t>
         </is>
       </c>
       <c r="C36" s="2" t="inlineStr">
         <is>
-          <t>0805</t>
+          <t>1206</t>
         </is>
       </c>
       <c r="D36" s="2" t="inlineStr">
         <is>
-          <t>R_IOUT_TOP</t>
+          <t>R_BL</t>
         </is>
       </c>
       <c r="E36" s="2" t="n">
@@ -2281,12 +2281,12 @@
       </c>
       <c r="I36" s="2" t="inlineStr">
         <is>
-          <t>精度/料号待核</t>
+          <t>功率/料号待核</t>
         </is>
       </c>
       <c r="J36" s="2" t="inlineStr">
         <is>
-          <t>输出告警参考上臂</t>
+          <t>确认实物额定功率，不能买成普通0805</t>
         </is>
       </c>
     </row>
@@ -2298,7 +2298,7 @@
       </c>
       <c r="B37" s="2" t="inlineStr">
         <is>
-          <t>2.2kΩ，≥0.25W</t>
+          <t>10Ω，≥0.25W，DNP</t>
         </is>
       </c>
       <c r="C37" s="2" t="inlineStr">
@@ -2308,14 +2308,14 @@
       </c>
       <c r="D37" s="2" t="inlineStr">
         <is>
-          <t>R_BL</t>
+          <t>R_SN</t>
         </is>
       </c>
       <c r="E37" s="2" t="n">
         <v>1</v>
       </c>
       <c r="F37" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G37" s="3" t="n"/>
       <c r="H37" s="2">
@@ -2324,41 +2324,41 @@
       </c>
       <c r="I37" s="2" t="inlineStr">
         <is>
-          <t>功率/料号待核</t>
+          <t>DNP，默认不装</t>
         </is>
       </c>
       <c r="J37" s="2" t="inlineStr">
         <is>
-          <t>确认实物额定功率，不能买成普通0805</t>
+          <t>与C_SN配套；由旧0805占位改1206</t>
         </is>
       </c>
     </row>
     <row r="38" ht="58" customHeight="1">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>功率电阻</t>
+          <t>二极管</t>
         </is>
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>10Ω，≥0.25W，DNP</t>
+          <t>SR560，目标60V/5A（用户选型）</t>
         </is>
       </c>
       <c r="C38" s="2" t="inlineStr">
         <is>
-          <t>1206</t>
+          <t>SMB / DO-214AA，贴片</t>
         </is>
       </c>
       <c r="D38" s="2" t="inlineStr">
         <is>
-          <t>R_SN</t>
+          <t>D1、D_FREE</t>
         </is>
       </c>
       <c r="E38" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F38" s="2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G38" s="3" t="n"/>
       <c r="H38" s="2">
@@ -2367,12 +2367,12 @@
       </c>
       <c r="I38" s="2" t="inlineStr">
         <is>
-          <t>DNP，默认不装</t>
+          <t>用户已确认SMB；厂家资料待最终复核</t>
         </is>
       </c>
       <c r="J38" s="2" t="inlineStr">
         <is>
-          <t>与C_SN配套；由旧0805占位改1206</t>
+          <t>共2只；1=K色条端、2=A。沿用原SMB焊盘；SR560为用户确认选型，原轴向目录不作为SMB厂家尺寸/电气手册；完整订货型号/额定条件/推荐焊盘待归档</t>
         </is>
       </c>
     </row>
@@ -2384,24 +2384,24 @@
       </c>
       <c r="B39" s="2" t="inlineStr">
         <is>
-          <t>SR560，目标60V/5A（用户选型）</t>
+          <t>UF4007，快恢复</t>
         </is>
       </c>
       <c r="C39" s="2" t="inlineStr">
         <is>
-          <t>SMB / DO-214AA，贴片</t>
+          <t>DO-41，成型P10.16待核</t>
         </is>
       </c>
       <c r="D39" s="2" t="inlineStr">
         <is>
-          <t>D1、D_FREE</t>
+          <t>D_BOOT</t>
         </is>
       </c>
       <c r="E39" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F39" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G39" s="3" t="n"/>
       <c r="H39" s="2">
@@ -2410,12 +2410,12 @@
       </c>
       <c r="I39" s="2" t="inlineStr">
         <is>
-          <t>用户已确认SMB；厂家资料待最终复核</t>
+          <t>成型脚距待核</t>
         </is>
       </c>
       <c r="J39" s="2" t="inlineStr">
         <is>
-          <t>共2只；1=K色条端、2=A。沿用原SMB焊盘；SR560为用户确认选型，原轴向目录不作为SMB厂家尺寸/电气手册；完整订货型号/额定条件/推荐焊盘待归档</t>
+          <t>工程定义1=A、2=K；不是普通1N4007</t>
         </is>
       </c>
     </row>
@@ -2427,24 +2427,24 @@
       </c>
       <c r="B40" s="2" t="inlineStr">
         <is>
-          <t>UF4007，快恢复</t>
+          <t>BAT54S，串联双肖特基</t>
         </is>
       </c>
       <c r="C40" s="2" t="inlineStr">
         <is>
-          <t>DO-41，成型P10.16待核</t>
+          <t>SOT-23</t>
         </is>
       </c>
       <c r="D40" s="2" t="inlineStr">
         <is>
-          <t>D_BOOT</t>
+          <t>D_ADC1、D_ADC2、D_ADC3、D_ADC4、D_ADC5、D_ADC6</t>
         </is>
       </c>
       <c r="E40" s="2" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="F40" s="2" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="G40" s="3" t="n"/>
       <c r="H40" s="2">
@@ -2453,12 +2453,12 @@
       </c>
       <c r="I40" s="2" t="inlineStr">
         <is>
-          <t>成型脚距待核</t>
+          <t>核对已购物料</t>
         </is>
       </c>
       <c r="J40" s="2" t="inlineStr">
         <is>
-          <t>工程定义1=A、2=K；不是普通1N4007</t>
+          <t>共6只；1=A1、2=K2、3=K1/A2；不能装BAT54/BAT54C</t>
         </is>
       </c>
     </row>
@@ -2470,7 +2470,7 @@
       </c>
       <c r="B41" s="2" t="inlineStr">
         <is>
-          <t>BAT54S，串联双肖特基</t>
+          <t>BAT54，单肖特基</t>
         </is>
       </c>
       <c r="C41" s="2" t="inlineStr">
@@ -2480,14 +2480,14 @@
       </c>
       <c r="D41" s="2" t="inlineStr">
         <is>
-          <t>D_ADC1、D_ADC2、D_ADC3、D_ADC4、D_ADC5、D_ADC6</t>
+          <t>D_POR</t>
         </is>
       </c>
       <c r="E41" s="2" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="F41" s="2" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="G41" s="3" t="n"/>
       <c r="H41" s="2">
@@ -2501,29 +2501,29 @@
       </c>
       <c r="J41" s="2" t="inlineStr">
         <is>
-          <t>共6只；1=A1、2=K2、3=K1/A2；不能装BAT54/BAT54C</t>
+          <t>1=A、3=K、2=NC；不能与BAT54S混装</t>
         </is>
       </c>
     </row>
     <row r="42" ht="58" customHeight="1">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>二极管</t>
+          <t>保险</t>
         </is>
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t>BAT54，单肖特基</t>
+          <t>2A快断保险管，5×20mm，商品标250V</t>
         </is>
       </c>
       <c r="C42" s="2" t="inlineStr">
         <is>
-          <t>SOT-23</t>
+          <t>配5×20mm管夹</t>
         </is>
       </c>
       <c r="D42" s="2" t="inlineStr">
         <is>
-          <t>D_POR</t>
+          <t>F1</t>
         </is>
       </c>
       <c r="E42" s="2" t="n">
@@ -2539,41 +2539,41 @@
       </c>
       <c r="I42" s="2" t="inlineStr">
         <is>
-          <t>核对已购物料</t>
+          <t>尺寸/快断已给资料；实际电气性能待核</t>
         </is>
       </c>
       <c r="J42" s="2" t="inlineStr">
         <is>
-          <t>1=A、3=K、2=NC；不能与BAT54S混装</t>
+          <t>商品BXG16519；250V未注明AC/DC分断条件，启动不误熔断与故障分断待验证；管夹另列2只</t>
         </is>
       </c>
     </row>
     <row r="43" ht="58" customHeight="1">
       <c r="A43" s="2" t="inlineStr">
         <is>
-          <t>保险</t>
+          <t>连接器</t>
         </is>
       </c>
       <c r="B43" s="2" t="inlineStr">
         <is>
-          <t>2A快断保险管，5×20mm，商品标250V</t>
+          <t>2P接线端子，P2.54，≥3A</t>
         </is>
       </c>
       <c r="C43" s="2" t="inlineStr">
         <is>
-          <t>配5×20mm管夹</t>
+          <t>图示5.48×6.30×8.80mm；孔1.30</t>
         </is>
       </c>
       <c r="D43" s="2" t="inlineStr">
         <is>
-          <t>F1</t>
+          <t>J1、J2、J_BYP、J_MON</t>
         </is>
       </c>
       <c r="E43" s="2" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="F43" s="2" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="G43" s="3" t="n"/>
       <c r="H43" s="2">
@@ -2582,12 +2582,12 @@
       </c>
       <c r="I43" s="2" t="inlineStr">
         <is>
-          <t>尺寸/快断已给资料；实际电气性能待核</t>
+          <t>完整型号/朝向待核</t>
         </is>
       </c>
       <c r="J43" s="2" t="inlineStr">
         <is>
-          <t>商品BXG16519；250V未注明AC/DC分断条件，启动不误熔断与故障分断待验证；管夹另列2只</t>
+          <t>共4只；照片标称6A/150V；J_BYP是接口，不包含外接开关</t>
         </is>
       </c>
     </row>
@@ -2599,24 +2599,24 @@
       </c>
       <c r="B44" s="2" t="inlineStr">
         <is>
-          <t>2P接线端子，P2.54，≥3A</t>
+          <t>1×4直排针，P2.54</t>
         </is>
       </c>
       <c r="C44" s="2" t="inlineStr">
         <is>
-          <t>图示5.48×6.30×8.80mm；孔1.30</t>
+          <t>直插，针长/塑高待核</t>
         </is>
       </c>
       <c r="D44" s="2" t="inlineStr">
         <is>
-          <t>J1、J2、J_BYP、J_MON</t>
+          <t>J_AUX12、J_AUX5</t>
         </is>
       </c>
       <c r="E44" s="2" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="F44" s="2" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="G44" s="3" t="n"/>
       <c r="H44" s="2">
@@ -2625,12 +2625,12 @@
       </c>
       <c r="I44" s="2" t="inlineStr">
         <is>
-          <t>完整型号/朝向待核</t>
+          <t>配对件待核</t>
         </is>
       </c>
       <c r="J44" s="2" t="inlineStr">
         <is>
-          <t>共4只；照片标称6A/150V；J_BYP是接口，不包含外接开关</t>
+          <t>共2只；与LM2596HV通过排线相接，不直接按四角焊盘插装</t>
         </is>
       </c>
     </row>
@@ -2642,24 +2642,24 @@
       </c>
       <c r="B45" s="2" t="inlineStr">
         <is>
-          <t>1×4直排针，P2.54</t>
+          <t>2×8排针，P2.54</t>
         </is>
       </c>
       <c r="C45" s="2" t="inlineStr">
         <is>
-          <t>直插，针长/塑高待核</t>
+          <t>直插；配对高度待核</t>
         </is>
       </c>
       <c r="D45" s="2" t="inlineStr">
         <is>
-          <t>J_AUX12、J_AUX5</t>
+          <t>J_CTL</t>
         </is>
       </c>
       <c r="E45" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F45" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G45" s="3" t="n"/>
       <c r="H45" s="2">
@@ -2673,36 +2673,36 @@
       </c>
       <c r="J45" s="2" t="inlineStr">
         <is>
-          <t>共2只；与LM2596HV通过排线相接，不直接按四角焊盘插装</t>
+          <t>1只，16针；PA6监测走独立J_MON，不占此16针</t>
         </is>
       </c>
     </row>
     <row r="46" ht="58" customHeight="1">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>连接器</t>
+          <t>测试点</t>
         </is>
       </c>
       <c r="B46" s="2" t="inlineStr">
         <is>
-          <t>2×8排针，P2.54</t>
+          <t>裸铜测试焊盘，直径1.5mm</t>
         </is>
       </c>
       <c r="C46" s="2" t="inlineStr">
         <is>
-          <t>直插；配对高度待核</t>
+          <t>PCB焊盘；默认不买测试柱</t>
         </is>
       </c>
       <c r="D46" s="2" t="inlineStr">
         <is>
-          <t>J_CTL</t>
+          <t>TP1、TP2、TP3、TP4、TP5、TP6、TP7、TP8、TP9、TP10、TP11、TP12、TP13、TP14</t>
         </is>
       </c>
       <c r="E46" s="2" t="n">
-        <v>1</v>
+        <v>14</v>
       </c>
       <c r="F46" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G46" s="3" t="n"/>
       <c r="H46" s="2">
@@ -2711,62 +2711,19 @@
       </c>
       <c r="I46" s="2" t="inlineStr">
         <is>
-          <t>配对件待核</t>
+          <t>默认无需采购</t>
         </is>
       </c>
       <c r="J46" s="2" t="inlineStr">
         <is>
-          <t>1只，16针；PA6监测走独立J_MON，不占此16针</t>
-        </is>
-      </c>
-    </row>
-    <row r="47" ht="58" customHeight="1">
-      <c r="A47" s="2" t="inlineStr">
-        <is>
-          <t>测试点</t>
-        </is>
-      </c>
-      <c r="B47" s="2" t="inlineStr">
-        <is>
-          <t>裸铜测试焊盘，直径1.5mm</t>
-        </is>
-      </c>
-      <c r="C47" s="2" t="inlineStr">
-        <is>
-          <t>PCB焊盘；默认不买测试柱</t>
-        </is>
-      </c>
-      <c r="D47" s="2" t="inlineStr">
-        <is>
-          <t>TP1、TP2、TP3、TP4、TP5、TP6、TP7、TP8、TP9、TP10、TP11、TP12、TP13、TP14</t>
-        </is>
-      </c>
-      <c r="E47" s="2" t="n">
-        <v>14</v>
-      </c>
-      <c r="F47" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="G47" s="3" t="n"/>
-      <c r="H47" s="2">
-        <f>IF(G47="","",MAX(F47-G47,0))</f>
-        <v/>
-      </c>
-      <c r="I47" s="2" t="inlineStr">
-        <is>
-          <t>默认无需采购</t>
-        </is>
-      </c>
-      <c r="J47" s="2" t="inlineStr">
-        <is>
           <t>14个设计测试点，实物采购数量为0；若改测试柱需同步封装</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:J47"/>
+  <autoFilter ref="A1:J46"/>
   <dataValidations count="1">
-    <dataValidation sqref="G2:G47" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="请输入非负整数" error="库存数量应为0或正整数" type="whole" operator="greaterThanOrEqual">
+    <dataValidation sqref="G2:G46" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="请输入非负整数" error="库存数量应为0或正整数" type="whole" operator="greaterThanOrEqual">
       <formula1>0</formula1>
     </dataValidation>
   </dataValidations>
@@ -3967,12 +3924,12 @@
       </c>
       <c r="H25" s="2" t="inlineStr">
         <is>
-          <t>核对实物料号</t>
+          <t>两只0805已确认；完整料号/介质待核</t>
         </is>
       </c>
       <c r="I25" s="2" t="inlineStr">
         <is>
-          <t>按参数表2×1.25mm改0805；介质和有效容量待核</t>
+          <t>共2只；C6来自原参数表，C_A3本轮由用户明确0805并替换原1206占位；实际介质与偏压后容量待核，库存另填</t>
         </is>
       </c>
       <c r="J25" s="2" t="inlineStr">
@@ -3994,7 +3951,7 @@
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>C1206</t>
+          <t>C0805</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr">
@@ -4004,7 +3961,7 @@
       </c>
       <c r="E26" s="2" t="inlineStr">
         <is>
-          <t>1206，暂保留</t>
+          <t>0805</t>
         </is>
       </c>
       <c r="F26" s="2" t="n">
@@ -4015,17 +3972,17 @@
       </c>
       <c r="H26" s="2" t="inlineStr">
         <is>
-          <t>封装待确认</t>
+          <t>两只0805已确认；完整料号/介质待核</t>
         </is>
       </c>
       <c r="I26" s="2" t="inlineStr">
         <is>
-          <t>参数表未填写本件；不能从C6推断为0805</t>
+          <t>共2只；C6来自原参数表，C_A3本轮由用户明确0805并替换原1206占位；实际介质与偏压后容量待核，库存另填</t>
         </is>
       </c>
       <c r="J26" s="2" t="inlineStr">
         <is>
-          <t>资料未填写，暂保留C1206；不能从C6推定本件也为0805</t>
+          <t>用户明确0805；10μF/25V保持，原1206暂定封装改C0805；中心(92,25)mm/90°保持，焊盘缩小并各向中心移动0.5mm；实际介质/完整料号及偏压容量待归档</t>
         </is>
       </c>
     </row>
@@ -8952,22 +8909,22 @@
     <row r="8" ht="58" customHeight="1">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>C2/C4/C6</t>
+          <t>C2/C4/C6/C_A3</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>旧C1206占位</t>
+          <t>原C1206占位</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>0805；C4为10μF/50V</t>
+          <t>现均0805；C4为10μF/50V</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>C_A3仍暂留1206，不跟随改动</t>
+          <t>C_A3本轮由用户单独确认0805，10μF/25V保持</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Record user confirmation of U1 IR2184 through-hole package
</commit_message>
<xml_diff>
--- a/projects/2026-electronics-contest/g-buck/rev-c2/downloads/GBUCK_RevC2_updated_BOM.xlsx
+++ b/projects/2026-electronics-contest/g-buck/rev-c2/downloads/GBUCK_RevC2_updated_BOM.xlsx
@@ -484,7 +484,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>本次比较c3892ab；用户确认C_A3为0805，由原1206占位改0805，10μF/25V保持；采购差额继续以B3补料后为基准。</t>
+          <t>本次比较61b2872；用户确认U1为IR2184直插，与既有DIP-8一致，本轮仅更新确认状态；C_A3已在上一版改0805；采购差额仍扣除B3后库存。</t>
         </is>
       </c>
     </row>
@@ -568,7 +568,7 @@
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>U1须IR2184PbF，不能直接用IR2104；RS_L 25mΩ在B3清单中已包含，旧表记未购，现库存待核，不再自动假定库存为0。</t>
+          <t>U1型号家族/直插类别已确认；保留IR2184PbF设计标注，不再列为型号封装待确认或默认补购；库存数量另填，IR2104不可代装。RS_L 25mΩ在B3清单中已包含，旧表记未购，现库存待核，不再自动假定库存为0。</t>
         </is>
       </c>
     </row>
@@ -676,7 +676,7 @@
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>相对c3892ab，C_A3仅改封装关联/说明，10μF/25V及全部电气网络和脚号保持；原Rev C2源文件保留。</t>
+          <t>相对61b2872，仅更新U1确认记录；原理图与PCB原生文件未改，网络、脚号和参数保持；回读U1八脚与DIP8_300一致。</t>
         </is>
       </c>
     </row>
@@ -688,7 +688,7 @@
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>C_A3由C1206改C0805，铜焊盘尺寸及中心距改变；保留全部器件中心/角度。C6/C_A3采购合并为同规格2只，45项合并行、120位号，不重复计料。</t>
+          <t>U1仍为设计IR2184PbF/DIP-8、每套1只；用户确认IR2184直插，撤销待确认标签，不新增或默认补购。型号、数量、封装和全部PCB几何保持，45项合并行/120位号保持。</t>
         </is>
       </c>
     </row>
@@ -819,12 +819,12 @@
       </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
-          <t>重点补购/核对</t>
+          <t>用户已确认IR2184直插</t>
         </is>
       </c>
       <c r="J2" s="2" t="inlineStr">
         <is>
-          <t>Rev C2要求；IR2104不可直接代装</t>
+          <t>与既有DIP8_300一致；保留设计PbF标注，不把家族确认当成完整订货号/厂家确认；库存数量另填；IR2104不可代装</t>
         </is>
       </c>
     </row>
@@ -2840,12 +2840,12 @@
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t>重点补购/核对</t>
+          <t>用户已确认IR2184直插</t>
         </is>
       </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
-          <t>Rev C2要求；IR2104不可直接代装</t>
+          <t>与既有DIP8_300一致；保留设计PbF标注，不把家族确认当成完整订货号/厂家确认；库存数量另填；IR2104不可代装</t>
         </is>
       </c>
       <c r="J2" s="2" t="inlineStr">
@@ -8787,12 +8787,12 @@
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>IR2184PbF，DIP8</t>
+          <t>设计IR2184PbF，DIP8</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>按Rev C2；不可直接代装</t>
+          <t>用户已确认IR2184直插；无需本轮改板，不默认补购；完整订货号/库存数量另记</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Classify confirmed 4.7nF batch separately from 100nF requirements
</commit_message>
<xml_diff>
--- a/projects/2026-electronics-contest/g-buck/rev-c2/downloads/GBUCK_RevC2_updated_BOM.xlsx
+++ b/projects/2026-electronics-contest/g-buck/rev-c2/downloads/GBUCK_RevC2_updated_BOM.xlsx
@@ -484,7 +484,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>本次比较61b2872；用户确认U1为IR2184直插，与既有DIP-8一致，本轮仅更新确认状态；C_A3已在上一版改0805；采购差额仍扣除B3后库存。</t>
+          <t>本次比较a50761f；用户确认原100nF询问所对应批次实际为4.7nF，改按4.7nF物料登记，不修改设计电容值；实际可用库存仍须核对。</t>
         </is>
       </c>
     </row>
@@ -592,7 +592,7 @@
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>参数表填在100nF项的CL21B472JBANNNC含472，通常对应4.7nF；100nF需按实际正确料号核对，不能批量错装。</t>
+          <t>用户已明确这批实际4.7nF，与CL21B472JBANNNC中的472一致；该批不能计作100nF。100nF/104的单独库存未确认，不直接认定需补16只。4.7nF数量/耐压/介质另核。</t>
         </is>
       </c>
     </row>
@@ -676,7 +676,7 @@
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>相对61b2872，仅更新U1确认记录；原理图与PCB原生文件未改，网络、脚号和参数保持；回读U1八脚与DIP8_300一致。</t>
+          <t>相对a50761f，仅纠正实购物料分类；原理图和PCB原生文件保持，100nF设计仍16只、4.7nF仍5只，不把去耦电容改为4.7nF。</t>
         </is>
       </c>
     </row>
@@ -688,7 +688,7 @@
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>U1仍为设计IR2184PbF/DIP-8、每套1只；用户确认IR2184直插，撤销待确认标签，不新增或默认补购。型号、数量、封装和全部PCB几何保持，45项合并行/120位号保持。</t>
+          <t>已确认批次归4.7nF，不抵扣100nF可用库存；是否另有100nF/104及4.7nF数量/介质仍待核。采购需求/45行/120位号及全部PCB几何保持；不自动填写库存0或缺货16只。</t>
         </is>
       </c>
     </row>
@@ -1593,12 +1593,12 @@
       </c>
       <c r="I20" s="2" t="inlineStr">
         <is>
-          <t>料号需纠错</t>
+          <t>该批实物已确认为4.7nF；100nF另核库存</t>
         </is>
       </c>
       <c r="J20" s="2" t="inlineStr">
         <is>
-          <t>合计16只；C_IOUT_PROT源要求25V，其余按原参数表50V统一采购；472是4.7nF，不能代用100nF</t>
+          <t>100nF仍需16只；C_IOUT_PROT源要求25V，其余按原参数表50V统一采购；已确认472批次不抵扣100nF库存，另有100nF数量待核，不默认缺16只</t>
         </is>
       </c>
     </row>
@@ -1636,12 +1636,12 @@
       </c>
       <c r="I21" s="2" t="inlineStr">
         <is>
-          <t>核对已购物料</t>
+          <t>用户已确认该批容量4.7nF；数量/介质另核</t>
         </is>
       </c>
       <c r="J21" s="2" t="inlineStr">
         <is>
-          <t>共5只；C_VINP_ADC明确C0G，其余按源要求可选相容介质；不把它们当100nF</t>
+          <t>设计共5只；参数表CL21B472JBANNNC与本轮确认容量一致，不计入100nF。容量确认不证明耐压/介质相容；C_VINP_ADC明确C0G，不能凭容量直接抵扣可用库存</t>
         </is>
       </c>
     </row>
@@ -4020,12 +4020,12 @@
       </c>
       <c r="H27" s="2" t="inlineStr">
         <is>
-          <t>料号需纠错</t>
+          <t>该批实物已确认为4.7nF；100nF另核库存</t>
         </is>
       </c>
       <c r="I27" s="2" t="inlineStr">
         <is>
-          <t>合计16只；C_IOUT_PROT源要求25V，其余按原参数表50V统一采购；472是4.7nF，不能代用100nF</t>
+          <t>100nF仍需16只；C_IOUT_PROT源要求25V，其余按原参数表50V统一采购；已确认472批次不抵扣100nF库存，另有100nF数量待核，不默认缺16只</t>
         </is>
       </c>
       <c r="J27" s="2" t="inlineStr"/>
@@ -4064,12 +4064,12 @@
       </c>
       <c r="H28" s="2" t="inlineStr">
         <is>
-          <t>料号需纠错</t>
+          <t>该批实物已确认为4.7nF；100nF另核库存</t>
         </is>
       </c>
       <c r="I28" s="2" t="inlineStr">
         <is>
-          <t>合计16只；C_IOUT_PROT源要求25V，其余按原参数表50V统一采购；472是4.7nF，不能代用100nF</t>
+          <t>100nF仍需16只；C_IOUT_PROT源要求25V，其余按原参数表50V统一采购；已确认472批次不抵扣100nF库存，另有100nF数量待核，不默认缺16只</t>
         </is>
       </c>
       <c r="J28" s="2" t="inlineStr"/>
@@ -4108,12 +4108,12 @@
       </c>
       <c r="H29" s="2" t="inlineStr">
         <is>
-          <t>料号需纠错</t>
+          <t>该批实物已确认为4.7nF；100nF另核库存</t>
         </is>
       </c>
       <c r="I29" s="2" t="inlineStr">
         <is>
-          <t>合计16只；C_IOUT_PROT源要求25V，其余按原参数表50V统一采购；472是4.7nF，不能代用100nF</t>
+          <t>100nF仍需16只；C_IOUT_PROT源要求25V，其余按原参数表50V统一采购；已确认472批次不抵扣100nF库存，另有100nF数量待核，不默认缺16只</t>
         </is>
       </c>
       <c r="J29" s="2" t="inlineStr"/>
@@ -4152,12 +4152,12 @@
       </c>
       <c r="H30" s="2" t="inlineStr">
         <is>
-          <t>料号需纠错</t>
+          <t>该批实物已确认为4.7nF；100nF另核库存</t>
         </is>
       </c>
       <c r="I30" s="2" t="inlineStr">
         <is>
-          <t>合计16只；C_IOUT_PROT源要求25V，其余按原参数表50V统一采购；472是4.7nF，不能代用100nF</t>
+          <t>100nF仍需16只；C_IOUT_PROT源要求25V，其余按原参数表50V统一采购；已确认472批次不抵扣100nF库存，另有100nF数量待核，不默认缺16只</t>
         </is>
       </c>
       <c r="J30" s="2" t="inlineStr"/>
@@ -4196,12 +4196,12 @@
       </c>
       <c r="H31" s="2" t="inlineStr">
         <is>
-          <t>料号需纠错</t>
+          <t>该批实物已确认为4.7nF；100nF另核库存</t>
         </is>
       </c>
       <c r="I31" s="2" t="inlineStr">
         <is>
-          <t>合计16只；C_IOUT_PROT源要求25V，其余按原参数表50V统一采购；472是4.7nF，不能代用100nF</t>
+          <t>100nF仍需16只；C_IOUT_PROT源要求25V，其余按原参数表50V统一采购；已确认472批次不抵扣100nF库存，另有100nF数量待核，不默认缺16只</t>
         </is>
       </c>
       <c r="J31" s="2" t="inlineStr"/>
@@ -4240,12 +4240,12 @@
       </c>
       <c r="H32" s="2" t="inlineStr">
         <is>
-          <t>料号需纠错</t>
+          <t>该批实物已确认为4.7nF；100nF另核库存</t>
         </is>
       </c>
       <c r="I32" s="2" t="inlineStr">
         <is>
-          <t>合计16只；C_IOUT_PROT源要求25V，其余按原参数表50V统一采购；472是4.7nF，不能代用100nF</t>
+          <t>100nF仍需16只；C_IOUT_PROT源要求25V，其余按原参数表50V统一采购；已确认472批次不抵扣100nF库存，另有100nF数量待核，不默认缺16只</t>
         </is>
       </c>
       <c r="J32" s="2" t="inlineStr"/>
@@ -4284,12 +4284,12 @@
       </c>
       <c r="H33" s="2" t="inlineStr">
         <is>
-          <t>料号需纠错</t>
+          <t>该批实物已确认为4.7nF；100nF另核库存</t>
         </is>
       </c>
       <c r="I33" s="2" t="inlineStr">
         <is>
-          <t>合计16只；C_IOUT_PROT源要求25V，其余按原参数表50V统一采购；472是4.7nF，不能代用100nF</t>
+          <t>100nF仍需16只；C_IOUT_PROT源要求25V，其余按原参数表50V统一采购；已确认472批次不抵扣100nF库存，另有100nF数量待核，不默认缺16只</t>
         </is>
       </c>
       <c r="J33" s="2" t="inlineStr"/>
@@ -4328,12 +4328,12 @@
       </c>
       <c r="H34" s="2" t="inlineStr">
         <is>
-          <t>料号需纠错</t>
+          <t>该批实物已确认为4.7nF；100nF另核库存</t>
         </is>
       </c>
       <c r="I34" s="2" t="inlineStr">
         <is>
-          <t>合计16只；C_IOUT_PROT源要求25V，其余按原参数表50V统一采购；472是4.7nF，不能代用100nF</t>
+          <t>100nF仍需16只；C_IOUT_PROT源要求25V，其余按原参数表50V统一采购；已确认472批次不抵扣100nF库存，另有100nF数量待核，不默认缺16只</t>
         </is>
       </c>
       <c r="J34" s="2" t="inlineStr"/>
@@ -4372,12 +4372,12 @@
       </c>
       <c r="H35" s="2" t="inlineStr">
         <is>
-          <t>料号需纠错</t>
+          <t>该批实物已确认为4.7nF；100nF另核库存</t>
         </is>
       </c>
       <c r="I35" s="2" t="inlineStr">
         <is>
-          <t>合计16只；C_IOUT_PROT源要求25V，其余按原参数表50V统一采购；472是4.7nF，不能代用100nF</t>
+          <t>100nF仍需16只；C_IOUT_PROT源要求25V，其余按原参数表50V统一采购；已确认472批次不抵扣100nF库存，另有100nF数量待核，不默认缺16只</t>
         </is>
       </c>
       <c r="J35" s="2" t="inlineStr"/>
@@ -4416,12 +4416,12 @@
       </c>
       <c r="H36" s="2" t="inlineStr">
         <is>
-          <t>料号需纠错</t>
+          <t>该批实物已确认为4.7nF；100nF另核库存</t>
         </is>
       </c>
       <c r="I36" s="2" t="inlineStr">
         <is>
-          <t>合计16只；C_IOUT_PROT源要求25V，其余按原参数表50V统一采购；472是4.7nF，不能代用100nF</t>
+          <t>100nF仍需16只；C_IOUT_PROT源要求25V，其余按原参数表50V统一采购；已确认472批次不抵扣100nF库存，另有100nF数量待核，不默认缺16只</t>
         </is>
       </c>
       <c r="J36" s="2" t="inlineStr"/>
@@ -4460,12 +4460,12 @@
       </c>
       <c r="H37" s="2" t="inlineStr">
         <is>
-          <t>料号需纠错</t>
+          <t>该批实物已确认为4.7nF；100nF另核库存</t>
         </is>
       </c>
       <c r="I37" s="2" t="inlineStr">
         <is>
-          <t>合计16只；C_IOUT_PROT源要求25V，其余按原参数表50V统一采购；472是4.7nF，不能代用100nF</t>
+          <t>100nF仍需16只；C_IOUT_PROT源要求25V，其余按原参数表50V统一采购；已确认472批次不抵扣100nF库存，另有100nF数量待核，不默认缺16只</t>
         </is>
       </c>
       <c r="J37" s="2" t="inlineStr"/>
@@ -4504,12 +4504,12 @@
       </c>
       <c r="H38" s="2" t="inlineStr">
         <is>
-          <t>料号需纠错</t>
+          <t>该批实物已确认为4.7nF；100nF另核库存</t>
         </is>
       </c>
       <c r="I38" s="2" t="inlineStr">
         <is>
-          <t>合计16只；C_IOUT_PROT源要求25V，其余按原参数表50V统一采购；472是4.7nF，不能代用100nF</t>
+          <t>100nF仍需16只；C_IOUT_PROT源要求25V，其余按原参数表50V统一采购；已确认472批次不抵扣100nF库存，另有100nF数量待核，不默认缺16只</t>
         </is>
       </c>
       <c r="J38" s="2" t="inlineStr"/>
@@ -4548,12 +4548,12 @@
       </c>
       <c r="H39" s="2" t="inlineStr">
         <is>
-          <t>料号需纠错</t>
+          <t>该批实物已确认为4.7nF；100nF另核库存</t>
         </is>
       </c>
       <c r="I39" s="2" t="inlineStr">
         <is>
-          <t>合计16只；C_IOUT_PROT源要求25V，其余按原参数表50V统一采购；472是4.7nF，不能代用100nF</t>
+          <t>100nF仍需16只；C_IOUT_PROT源要求25V，其余按原参数表50V统一采购；已确认472批次不抵扣100nF库存，另有100nF数量待核，不默认缺16只</t>
         </is>
       </c>
       <c r="J39" s="2" t="inlineStr"/>
@@ -4592,12 +4592,12 @@
       </c>
       <c r="H40" s="2" t="inlineStr">
         <is>
-          <t>料号需纠错</t>
+          <t>该批实物已确认为4.7nF；100nF另核库存</t>
         </is>
       </c>
       <c r="I40" s="2" t="inlineStr">
         <is>
-          <t>合计16只；C_IOUT_PROT源要求25V，其余按原参数表50V统一采购；472是4.7nF，不能代用100nF</t>
+          <t>100nF仍需16只；C_IOUT_PROT源要求25V，其余按原参数表50V统一采购；已确认472批次不抵扣100nF库存，另有100nF数量待核，不默认缺16只</t>
         </is>
       </c>
       <c r="J40" s="2" t="inlineStr"/>
@@ -4636,12 +4636,12 @@
       </c>
       <c r="H41" s="2" t="inlineStr">
         <is>
-          <t>料号需纠错</t>
+          <t>该批实物已确认为4.7nF；100nF另核库存</t>
         </is>
       </c>
       <c r="I41" s="2" t="inlineStr">
         <is>
-          <t>合计16只；C_IOUT_PROT源要求25V，其余按原参数表50V统一采购；472是4.7nF，不能代用100nF</t>
+          <t>100nF仍需16只；C_IOUT_PROT源要求25V，其余按原参数表50V统一采购；已确认472批次不抵扣100nF库存，另有100nF数量待核，不默认缺16只</t>
         </is>
       </c>
       <c r="J41" s="2" t="inlineStr"/>
@@ -4680,12 +4680,12 @@
       </c>
       <c r="H42" s="2" t="inlineStr">
         <is>
-          <t>料号需纠错</t>
+          <t>该批实物已确认为4.7nF；100nF另核库存</t>
         </is>
       </c>
       <c r="I42" s="2" t="inlineStr">
         <is>
-          <t>合计16只；C_IOUT_PROT源要求25V，其余按原参数表50V统一采购；472是4.7nF，不能代用100nF</t>
+          <t>100nF仍需16只；C_IOUT_PROT源要求25V，其余按原参数表50V统一采购；已确认472批次不抵扣100nF库存，另有100nF数量待核，不默认缺16只</t>
         </is>
       </c>
       <c r="J42" s="2" t="inlineStr">
@@ -4728,12 +4728,12 @@
       </c>
       <c r="H43" s="2" t="inlineStr">
         <is>
-          <t>核对已购物料</t>
+          <t>用户已确认该批容量4.7nF；数量/介质另核</t>
         </is>
       </c>
       <c r="I43" s="2" t="inlineStr">
         <is>
-          <t>共5只；C_VINP_ADC明确C0G，其余按源要求可选相容介质；不把它们当100nF</t>
+          <t>设计共5只；参数表CL21B472JBANNNC与本轮确认容量一致，不计入100nF。容量确认不证明耐压/介质相容；C_VINP_ADC明确C0G，不能凭容量直接抵扣可用库存</t>
         </is>
       </c>
       <c r="J43" s="2" t="inlineStr"/>
@@ -4772,12 +4772,12 @@
       </c>
       <c r="H44" s="2" t="inlineStr">
         <is>
-          <t>核对已购物料</t>
+          <t>用户已确认该批容量4.7nF；数量/介质另核</t>
         </is>
       </c>
       <c r="I44" s="2" t="inlineStr">
         <is>
-          <t>共5只；C_VINP_ADC明确C0G，其余按源要求可选相容介质；不把它们当100nF</t>
+          <t>设计共5只；参数表CL21B472JBANNNC与本轮确认容量一致，不计入100nF。容量确认不证明耐压/介质相容；C_VINP_ADC明确C0G，不能凭容量直接抵扣可用库存</t>
         </is>
       </c>
       <c r="J44" s="2" t="inlineStr"/>
@@ -4816,12 +4816,12 @@
       </c>
       <c r="H45" s="2" t="inlineStr">
         <is>
-          <t>核对已购物料</t>
+          <t>用户已确认该批容量4.7nF；数量/介质另核</t>
         </is>
       </c>
       <c r="I45" s="2" t="inlineStr">
         <is>
-          <t>共5只；C_VINP_ADC明确C0G，其余按源要求可选相容介质；不把它们当100nF</t>
+          <t>设计共5只；参数表CL21B472JBANNNC与本轮确认容量一致，不计入100nF。容量确认不证明耐压/介质相容；C_VINP_ADC明确C0G，不能凭容量直接抵扣可用库存</t>
         </is>
       </c>
       <c r="J45" s="2" t="inlineStr"/>
@@ -4860,12 +4860,12 @@
       </c>
       <c r="H46" s="2" t="inlineStr">
         <is>
-          <t>核对已购物料</t>
+          <t>用户已确认该批容量4.7nF；数量/介质另核</t>
         </is>
       </c>
       <c r="I46" s="2" t="inlineStr">
         <is>
-          <t>共5只；C_VINP_ADC明确C0G，其余按源要求可选相容介质；不把它们当100nF</t>
+          <t>设计共5只；参数表CL21B472JBANNNC与本轮确认容量一致，不计入100nF。容量确认不证明耐压/介质相容；C_VINP_ADC明确C0G，不能凭容量直接抵扣可用库存</t>
         </is>
       </c>
       <c r="J46" s="2" t="inlineStr"/>
@@ -4904,12 +4904,12 @@
       </c>
       <c r="H47" s="2" t="inlineStr">
         <is>
-          <t>核对已购物料</t>
+          <t>用户已确认该批容量4.7nF；数量/介质另核</t>
         </is>
       </c>
       <c r="I47" s="2" t="inlineStr">
         <is>
-          <t>共5只；C_VINP_ADC明确C0G，其余按源要求可选相容介质；不把它们当100nF</t>
+          <t>设计共5只；参数表CL21B472JBANNNC与本轮确认容量一致，不计入100nF。容量确认不证明耐压/介质相容；C_VINP_ADC明确C0G，不能凭容量直接抵扣可用库存</t>
         </is>
       </c>
       <c r="J47" s="2" t="inlineStr">
@@ -8936,17 +8936,17 @@
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>旧参数表14只，填了含472的料号</t>
+          <t>旧参数表误填472料号；用户确认该批4.7nF</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>Rev C2合计16只</t>
+          <t>Rev C2仍需100nF共16只</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>纠正容量料号；不要把4.7nF当100nF</t>
+          <t>该批不作100nF库存；是否另有100nF/104及数量待核，不默认缺16只</t>
         </is>
       </c>
     </row>
@@ -8958,7 +8958,7 @@
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>旧表5只但不含最新位号说明</t>
+          <t>用户确认所询问批次实际4.7nF</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
@@ -8968,7 +8968,7 @@
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>保持VIN_POST滤波器件</t>
+          <t>容量确认；可用数量/耐压/介质另核，C_VINP_ADC要求C0G，不凭容量认定相容</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Record separate 100nF 0805 purchase without assuming ratings or quantity
</commit_message>
<xml_diff>
--- a/projects/2026-electronics-contest/g-buck/rev-c2/downloads/GBUCK_RevC2_updated_BOM.xlsx
+++ b/projects/2026-electronics-contest/g-buck/rev-c2/downloads/GBUCK_RevC2_updated_BOM.xlsx
@@ -484,7 +484,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>本次比较a50761f；用户确认原100nF询问所对应批次实际为4.7nF，改按4.7nF物料登记，不修改设计电容值；实际可用库存仍须核对。</t>
+          <t>本次比较1404d80；用户确认另外买了100nF、0805，更新已购状态；实际数量/耐压/介质待核。4.7nF为独立批次，设计电容值/数量及PCB保持。</t>
         </is>
       </c>
     </row>
@@ -592,7 +592,7 @@
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>用户已明确这批实际4.7nF，与CL21B472JBANNNC中的472一致；该批不能计作100nF。100nF/104的单独库存未确认，不直接认定需补16只。4.7nF数量/耐压/介质另核。</t>
+          <t>472批次已确认4.7nF；随后用户确认另外买了100nF/0805，两批分开记录。100nF/0805不再列未购，但实际数量/耐压/介质待核，不自动填16只库存或缺16只；4.7nF数量/额定也另核。</t>
         </is>
       </c>
     </row>
@@ -676,7 +676,7 @@
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>相对a50761f，仅纠正实购物料分类；原理图和PCB原生文件保持，100nF设计仍16只、4.7nF仍5只，不把去耦电容改为4.7nF。</t>
+          <t>相对1404d80，仅记录另购100nF/0805已获用户确认；原理图和PCB原生文件未改，网络/脚号/参数保持，100nF设计仍16只、4.7nF仍5只。</t>
         </is>
       </c>
     </row>
@@ -688,7 +688,7 @@
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>已确认批次归4.7nF，不抵扣100nF可用库存；是否另有100nF/104及4.7nF数量/介质仍待核。采购需求/45行/120位号及全部PCB几何保持；不自动填写库存0或缺货16只。</t>
+          <t>100nF/0805改为已购；数量/耐压/介质待核，库存数量与补购数量保持未填，不认定已经足量。设计需求、45行采购记录/120位号和全部PCB几何保持，无本轮新增器件或封装变更。</t>
         </is>
       </c>
     </row>
@@ -1593,12 +1593,12 @@
       </c>
       <c r="I20" s="2" t="inlineStr">
         <is>
-          <t>该批实物已确认为4.7nF；100nF另核库存</t>
+          <t>用户已确认另购100nF/0805；数量/耐压/介质待核</t>
         </is>
       </c>
       <c r="J20" s="2" t="inlineStr">
         <is>
-          <t>100nF仍需16只；C_IOUT_PROT源要求25V，其余按原参数表50V统一采购；已确认472批次不抵扣100nF库存，另有100nF数量待核，不默认缺16只</t>
+          <t>每板设计16只，用户回复买了0805，确认另有100nF备料；不将16只需求填作库存。50V/X7R仍为统一采购建议，实际料号/耐压/介质待核；472批次独立记4.7nF</t>
         </is>
       </c>
     </row>
@@ -4020,12 +4020,12 @@
       </c>
       <c r="H27" s="2" t="inlineStr">
         <is>
-          <t>该批实物已确认为4.7nF；100nF另核库存</t>
+          <t>用户已确认另购100nF/0805；数量/耐压/介质待核</t>
         </is>
       </c>
       <c r="I27" s="2" t="inlineStr">
         <is>
-          <t>100nF仍需16只；C_IOUT_PROT源要求25V，其余按原参数表50V统一采购；已确认472批次不抵扣100nF库存，另有100nF数量待核，不默认缺16只</t>
+          <t>每板设计16只，用户回复买了0805，确认另有100nF备料；不将16只需求填作库存。50V/X7R仍为统一采购建议，实际料号/耐压/介质待核；472批次独立记4.7nF</t>
         </is>
       </c>
       <c r="J27" s="2" t="inlineStr"/>
@@ -4064,12 +4064,12 @@
       </c>
       <c r="H28" s="2" t="inlineStr">
         <is>
-          <t>该批实物已确认为4.7nF；100nF另核库存</t>
+          <t>用户已确认另购100nF/0805；数量/耐压/介质待核</t>
         </is>
       </c>
       <c r="I28" s="2" t="inlineStr">
         <is>
-          <t>100nF仍需16只；C_IOUT_PROT源要求25V，其余按原参数表50V统一采购；已确认472批次不抵扣100nF库存，另有100nF数量待核，不默认缺16只</t>
+          <t>每板设计16只，用户回复买了0805，确认另有100nF备料；不将16只需求填作库存。50V/X7R仍为统一采购建议，实际料号/耐压/介质待核；472批次独立记4.7nF</t>
         </is>
       </c>
       <c r="J28" s="2" t="inlineStr"/>
@@ -4108,12 +4108,12 @@
       </c>
       <c r="H29" s="2" t="inlineStr">
         <is>
-          <t>该批实物已确认为4.7nF；100nF另核库存</t>
+          <t>用户已确认另购100nF/0805；数量/耐压/介质待核</t>
         </is>
       </c>
       <c r="I29" s="2" t="inlineStr">
         <is>
-          <t>100nF仍需16只；C_IOUT_PROT源要求25V，其余按原参数表50V统一采购；已确认472批次不抵扣100nF库存，另有100nF数量待核，不默认缺16只</t>
+          <t>每板设计16只，用户回复买了0805，确认另有100nF备料；不将16只需求填作库存。50V/X7R仍为统一采购建议，实际料号/耐压/介质待核；472批次独立记4.7nF</t>
         </is>
       </c>
       <c r="J29" s="2" t="inlineStr"/>
@@ -4152,12 +4152,12 @@
       </c>
       <c r="H30" s="2" t="inlineStr">
         <is>
-          <t>该批实物已确认为4.7nF；100nF另核库存</t>
+          <t>用户已确认另购100nF/0805；数量/耐压/介质待核</t>
         </is>
       </c>
       <c r="I30" s="2" t="inlineStr">
         <is>
-          <t>100nF仍需16只；C_IOUT_PROT源要求25V，其余按原参数表50V统一采购；已确认472批次不抵扣100nF库存，另有100nF数量待核，不默认缺16只</t>
+          <t>每板设计16只，用户回复买了0805，确认另有100nF备料；不将16只需求填作库存。50V/X7R仍为统一采购建议，实际料号/耐压/介质待核；472批次独立记4.7nF</t>
         </is>
       </c>
       <c r="J30" s="2" t="inlineStr"/>
@@ -4196,12 +4196,12 @@
       </c>
       <c r="H31" s="2" t="inlineStr">
         <is>
-          <t>该批实物已确认为4.7nF；100nF另核库存</t>
+          <t>用户已确认另购100nF/0805；数量/耐压/介质待核</t>
         </is>
       </c>
       <c r="I31" s="2" t="inlineStr">
         <is>
-          <t>100nF仍需16只；C_IOUT_PROT源要求25V，其余按原参数表50V统一采购；已确认472批次不抵扣100nF库存，另有100nF数量待核，不默认缺16只</t>
+          <t>每板设计16只，用户回复买了0805，确认另有100nF备料；不将16只需求填作库存。50V/X7R仍为统一采购建议，实际料号/耐压/介质待核；472批次独立记4.7nF</t>
         </is>
       </c>
       <c r="J31" s="2" t="inlineStr"/>
@@ -4240,12 +4240,12 @@
       </c>
       <c r="H32" s="2" t="inlineStr">
         <is>
-          <t>该批实物已确认为4.7nF；100nF另核库存</t>
+          <t>用户已确认另购100nF/0805；数量/耐压/介质待核</t>
         </is>
       </c>
       <c r="I32" s="2" t="inlineStr">
         <is>
-          <t>100nF仍需16只；C_IOUT_PROT源要求25V，其余按原参数表50V统一采购；已确认472批次不抵扣100nF库存，另有100nF数量待核，不默认缺16只</t>
+          <t>每板设计16只，用户回复买了0805，确认另有100nF备料；不将16只需求填作库存。50V/X7R仍为统一采购建议，实际料号/耐压/介质待核；472批次独立记4.7nF</t>
         </is>
       </c>
       <c r="J32" s="2" t="inlineStr"/>
@@ -4284,12 +4284,12 @@
       </c>
       <c r="H33" s="2" t="inlineStr">
         <is>
-          <t>该批实物已确认为4.7nF；100nF另核库存</t>
+          <t>用户已确认另购100nF/0805；数量/耐压/介质待核</t>
         </is>
       </c>
       <c r="I33" s="2" t="inlineStr">
         <is>
-          <t>100nF仍需16只；C_IOUT_PROT源要求25V，其余按原参数表50V统一采购；已确认472批次不抵扣100nF库存，另有100nF数量待核，不默认缺16只</t>
+          <t>每板设计16只，用户回复买了0805，确认另有100nF备料；不将16只需求填作库存。50V/X7R仍为统一采购建议，实际料号/耐压/介质待核；472批次独立记4.7nF</t>
         </is>
       </c>
       <c r="J33" s="2" t="inlineStr"/>
@@ -4328,12 +4328,12 @@
       </c>
       <c r="H34" s="2" t="inlineStr">
         <is>
-          <t>该批实物已确认为4.7nF；100nF另核库存</t>
+          <t>用户已确认另购100nF/0805；数量/耐压/介质待核</t>
         </is>
       </c>
       <c r="I34" s="2" t="inlineStr">
         <is>
-          <t>100nF仍需16只；C_IOUT_PROT源要求25V，其余按原参数表50V统一采购；已确认472批次不抵扣100nF库存，另有100nF数量待核，不默认缺16只</t>
+          <t>每板设计16只，用户回复买了0805，确认另有100nF备料；不将16只需求填作库存。50V/X7R仍为统一采购建议，实际料号/耐压/介质待核；472批次独立记4.7nF</t>
         </is>
       </c>
       <c r="J34" s="2" t="inlineStr"/>
@@ -4372,12 +4372,12 @@
       </c>
       <c r="H35" s="2" t="inlineStr">
         <is>
-          <t>该批实物已确认为4.7nF；100nF另核库存</t>
+          <t>用户已确认另购100nF/0805；数量/耐压/介质待核</t>
         </is>
       </c>
       <c r="I35" s="2" t="inlineStr">
         <is>
-          <t>100nF仍需16只；C_IOUT_PROT源要求25V，其余按原参数表50V统一采购；已确认472批次不抵扣100nF库存，另有100nF数量待核，不默认缺16只</t>
+          <t>每板设计16只，用户回复买了0805，确认另有100nF备料；不将16只需求填作库存。50V/X7R仍为统一采购建议，实际料号/耐压/介质待核；472批次独立记4.7nF</t>
         </is>
       </c>
       <c r="J35" s="2" t="inlineStr"/>
@@ -4416,12 +4416,12 @@
       </c>
       <c r="H36" s="2" t="inlineStr">
         <is>
-          <t>该批实物已确认为4.7nF；100nF另核库存</t>
+          <t>用户已确认另购100nF/0805；数量/耐压/介质待核</t>
         </is>
       </c>
       <c r="I36" s="2" t="inlineStr">
         <is>
-          <t>100nF仍需16只；C_IOUT_PROT源要求25V，其余按原参数表50V统一采购；已确认472批次不抵扣100nF库存，另有100nF数量待核，不默认缺16只</t>
+          <t>每板设计16只，用户回复买了0805，确认另有100nF备料；不将16只需求填作库存。50V/X7R仍为统一采购建议，实际料号/耐压/介质待核；472批次独立记4.7nF</t>
         </is>
       </c>
       <c r="J36" s="2" t="inlineStr"/>
@@ -4460,12 +4460,12 @@
       </c>
       <c r="H37" s="2" t="inlineStr">
         <is>
-          <t>该批实物已确认为4.7nF；100nF另核库存</t>
+          <t>用户已确认另购100nF/0805；数量/耐压/介质待核</t>
         </is>
       </c>
       <c r="I37" s="2" t="inlineStr">
         <is>
-          <t>100nF仍需16只；C_IOUT_PROT源要求25V，其余按原参数表50V统一采购；已确认472批次不抵扣100nF库存，另有100nF数量待核，不默认缺16只</t>
+          <t>每板设计16只，用户回复买了0805，确认另有100nF备料；不将16只需求填作库存。50V/X7R仍为统一采购建议，实际料号/耐压/介质待核；472批次独立记4.7nF</t>
         </is>
       </c>
       <c r="J37" s="2" t="inlineStr"/>
@@ -4504,12 +4504,12 @@
       </c>
       <c r="H38" s="2" t="inlineStr">
         <is>
-          <t>该批实物已确认为4.7nF；100nF另核库存</t>
+          <t>用户已确认另购100nF/0805；数量/耐压/介质待核</t>
         </is>
       </c>
       <c r="I38" s="2" t="inlineStr">
         <is>
-          <t>100nF仍需16只；C_IOUT_PROT源要求25V，其余按原参数表50V统一采购；已确认472批次不抵扣100nF库存，另有100nF数量待核，不默认缺16只</t>
+          <t>每板设计16只，用户回复买了0805，确认另有100nF备料；不将16只需求填作库存。50V/X7R仍为统一采购建议，实际料号/耐压/介质待核；472批次独立记4.7nF</t>
         </is>
       </c>
       <c r="J38" s="2" t="inlineStr"/>
@@ -4548,12 +4548,12 @@
       </c>
       <c r="H39" s="2" t="inlineStr">
         <is>
-          <t>该批实物已确认为4.7nF；100nF另核库存</t>
+          <t>用户已确认另购100nF/0805；数量/耐压/介质待核</t>
         </is>
       </c>
       <c r="I39" s="2" t="inlineStr">
         <is>
-          <t>100nF仍需16只；C_IOUT_PROT源要求25V，其余按原参数表50V统一采购；已确认472批次不抵扣100nF库存，另有100nF数量待核，不默认缺16只</t>
+          <t>每板设计16只，用户回复买了0805，确认另有100nF备料；不将16只需求填作库存。50V/X7R仍为统一采购建议，实际料号/耐压/介质待核；472批次独立记4.7nF</t>
         </is>
       </c>
       <c r="J39" s="2" t="inlineStr"/>
@@ -4592,12 +4592,12 @@
       </c>
       <c r="H40" s="2" t="inlineStr">
         <is>
-          <t>该批实物已确认为4.7nF；100nF另核库存</t>
+          <t>用户已确认另购100nF/0805；数量/耐压/介质待核</t>
         </is>
       </c>
       <c r="I40" s="2" t="inlineStr">
         <is>
-          <t>100nF仍需16只；C_IOUT_PROT源要求25V，其余按原参数表50V统一采购；已确认472批次不抵扣100nF库存，另有100nF数量待核，不默认缺16只</t>
+          <t>每板设计16只，用户回复买了0805，确认另有100nF备料；不将16只需求填作库存。50V/X7R仍为统一采购建议，实际料号/耐压/介质待核；472批次独立记4.7nF</t>
         </is>
       </c>
       <c r="J40" s="2" t="inlineStr"/>
@@ -4636,12 +4636,12 @@
       </c>
       <c r="H41" s="2" t="inlineStr">
         <is>
-          <t>该批实物已确认为4.7nF；100nF另核库存</t>
+          <t>用户已确认另购100nF/0805；数量/耐压/介质待核</t>
         </is>
       </c>
       <c r="I41" s="2" t="inlineStr">
         <is>
-          <t>100nF仍需16只；C_IOUT_PROT源要求25V，其余按原参数表50V统一采购；已确认472批次不抵扣100nF库存，另有100nF数量待核，不默认缺16只</t>
+          <t>每板设计16只，用户回复买了0805，确认另有100nF备料；不将16只需求填作库存。50V/X7R仍为统一采购建议，实际料号/耐压/介质待核；472批次独立记4.7nF</t>
         </is>
       </c>
       <c r="J41" s="2" t="inlineStr"/>
@@ -4680,12 +4680,12 @@
       </c>
       <c r="H42" s="2" t="inlineStr">
         <is>
-          <t>该批实物已确认为4.7nF；100nF另核库存</t>
+          <t>用户已确认另购100nF/0805；数量/耐压/介质待核</t>
         </is>
       </c>
       <c r="I42" s="2" t="inlineStr">
         <is>
-          <t>100nF仍需16只；C_IOUT_PROT源要求25V，其余按原参数表50V统一采购；已确认472批次不抵扣100nF库存，另有100nF数量待核，不默认缺16只</t>
+          <t>每板设计16只，用户回复买了0805，确认另有100nF备料；不将16只需求填作库存。50V/X7R仍为统一采购建议，实际料号/耐压/介质待核；472批次独立记4.7nF</t>
         </is>
       </c>
       <c r="J42" s="2" t="inlineStr">
@@ -8936,7 +8936,7 @@
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>旧参数表误填472料号；用户确认该批4.7nF</t>
+          <t>原472批次实际4.7nF；现确认另购100nF/0805</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
@@ -8946,7 +8946,7 @@
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>该批不作100nF库存；是否另有100nF/104及数量待核，不默认缺16只</t>
+          <t>已购状态确认，数量/耐压/介质待核；不默认库存16只或已经足量</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Confirm purchased 100nF 0805 capacitors are rated 50V
</commit_message>
<xml_diff>
--- a/projects/2026-electronics-contest/g-buck/rev-c2/downloads/GBUCK_RevC2_updated_BOM.xlsx
+++ b/projects/2026-electronics-contest/g-buck/rev-c2/downloads/GBUCK_RevC2_updated_BOM.xlsx
@@ -484,7 +484,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>本次比较1404d80；用户确认另外买了100nF、0805，更新已购状态；实际数量/耐压/介质待核。4.7nF为独立批次，设计电容值/数量及PCB保持。</t>
+          <t>本次比较3384d1c；用户确认已购100nF/0805的额定耐压50V，更新物料记录；实际数量/介质/完整料号待核。设计参数、用量与PCB保持。</t>
         </is>
       </c>
     </row>
@@ -592,7 +592,7 @@
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>472批次已确认4.7nF；随后用户确认另外买了100nF/0805，两批分开记录。100nF/0805不再列未购，但实际数量/耐压/介质待核，不自动填16只库存或缺16只；4.7nF数量/额定也另核。</t>
+          <t>472批次已确认4.7nF；随后用户确认另外买了100nF/0805，两批分开记录。100nF/0805已购且50V已确认，实际数量/介质/完整料号待核，不自动填16只库存或缺16只；4.7nF数量/额定也另核。</t>
         </is>
       </c>
     </row>
@@ -676,7 +676,7 @@
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>相对1404d80，仅记录另购100nF/0805已获用户确认；原理图和PCB原生文件未改，网络/脚号/参数保持，100nF设计仍16只、4.7nF仍5只。</t>
+          <t>相对3384d1c，仅补记已购100nF/0805的50V额定；原理图和PCB原生文件未改，网络/脚号/参数与数量保持；100nF设计仍16只。</t>
         </is>
       </c>
     </row>
@@ -688,7 +688,7 @@
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>100nF/0805改为已购；数量/耐压/介质待核，库存数量与补购数量保持未填，不认定已经足量。设计需求、45行采购记录/120位号和全部PCB几何保持，无本轮新增器件或封装变更。</t>
+          <t>100nF/50V/0805已获用户确认，符合现有统一采购耐压；仅撤销该批耐压待核标签。数量/介质/完整料号待核，不自动填写库存或补购数量。设计需求、45采购行/120位号及全部PCB几何保持，无新增器件或替换要求。</t>
         </is>
       </c>
     </row>
@@ -1567,7 +1567,7 @@
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>100nF/50V，X7R（统一采购建议）</t>
+          <t>100nF/50V，建议X7R</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
@@ -1593,12 +1593,12 @@
       </c>
       <c r="I20" s="2" t="inlineStr">
         <is>
-          <t>用户已确认另购100nF/0805；数量/耐压/介质待核</t>
+          <t>已购100nF/50V/0805已确认；数量/介质待核</t>
         </is>
       </c>
       <c r="J20" s="2" t="inlineStr">
         <is>
-          <t>每板设计16只，用户回复买了0805，确认另有100nF备料；不将16只需求填作库存。50V/X7R仍为统一采购建议，实际料号/耐压/介质待核；472批次独立记4.7nF</t>
+          <t>用户补充50v，确认这批额定50V，符合当前统一采购耐压；每板设计16只，实际数量/介质/完整料号待核。X7R仍为建议，不将需求16只自动填作库存；472批次独立记4.7nF</t>
         </is>
       </c>
     </row>
@@ -4004,7 +4004,7 @@
       </c>
       <c r="D27" s="2" t="inlineStr">
         <is>
-          <t>100nF/50V，X7R（统一采购建议）</t>
+          <t>100nF/50V，建议X7R</t>
         </is>
       </c>
       <c r="E27" s="2" t="inlineStr">
@@ -4020,12 +4020,12 @@
       </c>
       <c r="H27" s="2" t="inlineStr">
         <is>
-          <t>用户已确认另购100nF/0805；数量/耐压/介质待核</t>
+          <t>已购100nF/50V/0805已确认；数量/介质待核</t>
         </is>
       </c>
       <c r="I27" s="2" t="inlineStr">
         <is>
-          <t>每板设计16只，用户回复买了0805，确认另有100nF备料；不将16只需求填作库存。50V/X7R仍为统一采购建议，实际料号/耐压/介质待核；472批次独立记4.7nF</t>
+          <t>用户补充50v，确认这批额定50V，符合当前统一采购耐压；每板设计16只，实际数量/介质/完整料号待核。X7R仍为建议，不将需求16只自动填作库存；472批次独立记4.7nF</t>
         </is>
       </c>
       <c r="J27" s="2" t="inlineStr"/>
@@ -4048,7 +4048,7 @@
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t>100nF/50V，X7R（统一采购建议）</t>
+          <t>100nF/50V，建议X7R</t>
         </is>
       </c>
       <c r="E28" s="2" t="inlineStr">
@@ -4064,12 +4064,12 @@
       </c>
       <c r="H28" s="2" t="inlineStr">
         <is>
-          <t>用户已确认另购100nF/0805；数量/耐压/介质待核</t>
+          <t>已购100nF/50V/0805已确认；数量/介质待核</t>
         </is>
       </c>
       <c r="I28" s="2" t="inlineStr">
         <is>
-          <t>每板设计16只，用户回复买了0805，确认另有100nF备料；不将16只需求填作库存。50V/X7R仍为统一采购建议，实际料号/耐压/介质待核；472批次独立记4.7nF</t>
+          <t>用户补充50v，确认这批额定50V，符合当前统一采购耐压；每板设计16只，实际数量/介质/完整料号待核。X7R仍为建议，不将需求16只自动填作库存；472批次独立记4.7nF</t>
         </is>
       </c>
       <c r="J28" s="2" t="inlineStr"/>
@@ -4092,7 +4092,7 @@
       </c>
       <c r="D29" s="2" t="inlineStr">
         <is>
-          <t>100nF/50V，X7R（统一采购建议）</t>
+          <t>100nF/50V，建议X7R</t>
         </is>
       </c>
       <c r="E29" s="2" t="inlineStr">
@@ -4108,12 +4108,12 @@
       </c>
       <c r="H29" s="2" t="inlineStr">
         <is>
-          <t>用户已确认另购100nF/0805；数量/耐压/介质待核</t>
+          <t>已购100nF/50V/0805已确认；数量/介质待核</t>
         </is>
       </c>
       <c r="I29" s="2" t="inlineStr">
         <is>
-          <t>每板设计16只，用户回复买了0805，确认另有100nF备料；不将16只需求填作库存。50V/X7R仍为统一采购建议，实际料号/耐压/介质待核；472批次独立记4.7nF</t>
+          <t>用户补充50v，确认这批额定50V，符合当前统一采购耐压；每板设计16只，实际数量/介质/完整料号待核。X7R仍为建议，不将需求16只自动填作库存；472批次独立记4.7nF</t>
         </is>
       </c>
       <c r="J29" s="2" t="inlineStr"/>
@@ -4136,7 +4136,7 @@
       </c>
       <c r="D30" s="2" t="inlineStr">
         <is>
-          <t>100nF/50V，X7R（统一采购建议）</t>
+          <t>100nF/50V，建议X7R</t>
         </is>
       </c>
       <c r="E30" s="2" t="inlineStr">
@@ -4152,12 +4152,12 @@
       </c>
       <c r="H30" s="2" t="inlineStr">
         <is>
-          <t>用户已确认另购100nF/0805；数量/耐压/介质待核</t>
+          <t>已购100nF/50V/0805已确认；数量/介质待核</t>
         </is>
       </c>
       <c r="I30" s="2" t="inlineStr">
         <is>
-          <t>每板设计16只，用户回复买了0805，确认另有100nF备料；不将16只需求填作库存。50V/X7R仍为统一采购建议，实际料号/耐压/介质待核；472批次独立记4.7nF</t>
+          <t>用户补充50v，确认这批额定50V，符合当前统一采购耐压；每板设计16只，实际数量/介质/完整料号待核。X7R仍为建议，不将需求16只自动填作库存；472批次独立记4.7nF</t>
         </is>
       </c>
       <c r="J30" s="2" t="inlineStr"/>
@@ -4180,7 +4180,7 @@
       </c>
       <c r="D31" s="2" t="inlineStr">
         <is>
-          <t>100nF/50V，X7R（统一采购建议）</t>
+          <t>100nF/50V，建议X7R</t>
         </is>
       </c>
       <c r="E31" s="2" t="inlineStr">
@@ -4196,12 +4196,12 @@
       </c>
       <c r="H31" s="2" t="inlineStr">
         <is>
-          <t>用户已确认另购100nF/0805；数量/耐压/介质待核</t>
+          <t>已购100nF/50V/0805已确认；数量/介质待核</t>
         </is>
       </c>
       <c r="I31" s="2" t="inlineStr">
         <is>
-          <t>每板设计16只，用户回复买了0805，确认另有100nF备料；不将16只需求填作库存。50V/X7R仍为统一采购建议，实际料号/耐压/介质待核；472批次独立记4.7nF</t>
+          <t>用户补充50v，确认这批额定50V，符合当前统一采购耐压；每板设计16只，实际数量/介质/完整料号待核。X7R仍为建议，不将需求16只自动填作库存；472批次独立记4.7nF</t>
         </is>
       </c>
       <c r="J31" s="2" t="inlineStr"/>
@@ -4224,7 +4224,7 @@
       </c>
       <c r="D32" s="2" t="inlineStr">
         <is>
-          <t>100nF/50V，X7R（统一采购建议）</t>
+          <t>100nF/50V，建议X7R</t>
         </is>
       </c>
       <c r="E32" s="2" t="inlineStr">
@@ -4240,12 +4240,12 @@
       </c>
       <c r="H32" s="2" t="inlineStr">
         <is>
-          <t>用户已确认另购100nF/0805；数量/耐压/介质待核</t>
+          <t>已购100nF/50V/0805已确认；数量/介质待核</t>
         </is>
       </c>
       <c r="I32" s="2" t="inlineStr">
         <is>
-          <t>每板设计16只，用户回复买了0805，确认另有100nF备料；不将16只需求填作库存。50V/X7R仍为统一采购建议，实际料号/耐压/介质待核；472批次独立记4.7nF</t>
+          <t>用户补充50v，确认这批额定50V，符合当前统一采购耐压；每板设计16只，实际数量/介质/完整料号待核。X7R仍为建议，不将需求16只自动填作库存；472批次独立记4.7nF</t>
         </is>
       </c>
       <c r="J32" s="2" t="inlineStr"/>
@@ -4268,7 +4268,7 @@
       </c>
       <c r="D33" s="2" t="inlineStr">
         <is>
-          <t>100nF/50V，X7R（统一采购建议）</t>
+          <t>100nF/50V，建议X7R</t>
         </is>
       </c>
       <c r="E33" s="2" t="inlineStr">
@@ -4284,12 +4284,12 @@
       </c>
       <c r="H33" s="2" t="inlineStr">
         <is>
-          <t>用户已确认另购100nF/0805；数量/耐压/介质待核</t>
+          <t>已购100nF/50V/0805已确认；数量/介质待核</t>
         </is>
       </c>
       <c r="I33" s="2" t="inlineStr">
         <is>
-          <t>每板设计16只，用户回复买了0805，确认另有100nF备料；不将16只需求填作库存。50V/X7R仍为统一采购建议，实际料号/耐压/介质待核；472批次独立记4.7nF</t>
+          <t>用户补充50v，确认这批额定50V，符合当前统一采购耐压；每板设计16只，实际数量/介质/完整料号待核。X7R仍为建议，不将需求16只自动填作库存；472批次独立记4.7nF</t>
         </is>
       </c>
       <c r="J33" s="2" t="inlineStr"/>
@@ -4312,7 +4312,7 @@
       </c>
       <c r="D34" s="2" t="inlineStr">
         <is>
-          <t>100nF/50V，X7R（统一采购建议）</t>
+          <t>100nF/50V，建议X7R</t>
         </is>
       </c>
       <c r="E34" s="2" t="inlineStr">
@@ -4328,12 +4328,12 @@
       </c>
       <c r="H34" s="2" t="inlineStr">
         <is>
-          <t>用户已确认另购100nF/0805；数量/耐压/介质待核</t>
+          <t>已购100nF/50V/0805已确认；数量/介质待核</t>
         </is>
       </c>
       <c r="I34" s="2" t="inlineStr">
         <is>
-          <t>每板设计16只，用户回复买了0805，确认另有100nF备料；不将16只需求填作库存。50V/X7R仍为统一采购建议，实际料号/耐压/介质待核；472批次独立记4.7nF</t>
+          <t>用户补充50v，确认这批额定50V，符合当前统一采购耐压；每板设计16只，实际数量/介质/完整料号待核。X7R仍为建议，不将需求16只自动填作库存；472批次独立记4.7nF</t>
         </is>
       </c>
       <c r="J34" s="2" t="inlineStr"/>
@@ -4356,7 +4356,7 @@
       </c>
       <c r="D35" s="2" t="inlineStr">
         <is>
-          <t>100nF/50V，X7R（统一采购建议）</t>
+          <t>100nF/50V，建议X7R</t>
         </is>
       </c>
       <c r="E35" s="2" t="inlineStr">
@@ -4372,12 +4372,12 @@
       </c>
       <c r="H35" s="2" t="inlineStr">
         <is>
-          <t>用户已确认另购100nF/0805；数量/耐压/介质待核</t>
+          <t>已购100nF/50V/0805已确认；数量/介质待核</t>
         </is>
       </c>
       <c r="I35" s="2" t="inlineStr">
         <is>
-          <t>每板设计16只，用户回复买了0805，确认另有100nF备料；不将16只需求填作库存。50V/X7R仍为统一采购建议，实际料号/耐压/介质待核；472批次独立记4.7nF</t>
+          <t>用户补充50v，确认这批额定50V，符合当前统一采购耐压；每板设计16只，实际数量/介质/完整料号待核。X7R仍为建议，不将需求16只自动填作库存；472批次独立记4.7nF</t>
         </is>
       </c>
       <c r="J35" s="2" t="inlineStr"/>
@@ -4400,7 +4400,7 @@
       </c>
       <c r="D36" s="2" t="inlineStr">
         <is>
-          <t>100nF/50V，X7R（统一采购建议）</t>
+          <t>100nF/50V，建议X7R</t>
         </is>
       </c>
       <c r="E36" s="2" t="inlineStr">
@@ -4416,12 +4416,12 @@
       </c>
       <c r="H36" s="2" t="inlineStr">
         <is>
-          <t>用户已确认另购100nF/0805；数量/耐压/介质待核</t>
+          <t>已购100nF/50V/0805已确认；数量/介质待核</t>
         </is>
       </c>
       <c r="I36" s="2" t="inlineStr">
         <is>
-          <t>每板设计16只，用户回复买了0805，确认另有100nF备料；不将16只需求填作库存。50V/X7R仍为统一采购建议，实际料号/耐压/介质待核；472批次独立记4.7nF</t>
+          <t>用户补充50v，确认这批额定50V，符合当前统一采购耐压；每板设计16只，实际数量/介质/完整料号待核。X7R仍为建议，不将需求16只自动填作库存；472批次独立记4.7nF</t>
         </is>
       </c>
       <c r="J36" s="2" t="inlineStr"/>
@@ -4444,7 +4444,7 @@
       </c>
       <c r="D37" s="2" t="inlineStr">
         <is>
-          <t>100nF/50V，X7R（统一采购建议）</t>
+          <t>100nF/50V，建议X7R</t>
         </is>
       </c>
       <c r="E37" s="2" t="inlineStr">
@@ -4460,12 +4460,12 @@
       </c>
       <c r="H37" s="2" t="inlineStr">
         <is>
-          <t>用户已确认另购100nF/0805；数量/耐压/介质待核</t>
+          <t>已购100nF/50V/0805已确认；数量/介质待核</t>
         </is>
       </c>
       <c r="I37" s="2" t="inlineStr">
         <is>
-          <t>每板设计16只，用户回复买了0805，确认另有100nF备料；不将16只需求填作库存。50V/X7R仍为统一采购建议，实际料号/耐压/介质待核；472批次独立记4.7nF</t>
+          <t>用户补充50v，确认这批额定50V，符合当前统一采购耐压；每板设计16只，实际数量/介质/完整料号待核。X7R仍为建议，不将需求16只自动填作库存；472批次独立记4.7nF</t>
         </is>
       </c>
       <c r="J37" s="2" t="inlineStr"/>
@@ -4488,7 +4488,7 @@
       </c>
       <c r="D38" s="2" t="inlineStr">
         <is>
-          <t>100nF/50V，X7R（统一采购建议）</t>
+          <t>100nF/50V，建议X7R</t>
         </is>
       </c>
       <c r="E38" s="2" t="inlineStr">
@@ -4504,12 +4504,12 @@
       </c>
       <c r="H38" s="2" t="inlineStr">
         <is>
-          <t>用户已确认另购100nF/0805；数量/耐压/介质待核</t>
+          <t>已购100nF/50V/0805已确认；数量/介质待核</t>
         </is>
       </c>
       <c r="I38" s="2" t="inlineStr">
         <is>
-          <t>每板设计16只，用户回复买了0805，确认另有100nF备料；不将16只需求填作库存。50V/X7R仍为统一采购建议，实际料号/耐压/介质待核；472批次独立记4.7nF</t>
+          <t>用户补充50v，确认这批额定50V，符合当前统一采购耐压；每板设计16只，实际数量/介质/完整料号待核。X7R仍为建议，不将需求16只自动填作库存；472批次独立记4.7nF</t>
         </is>
       </c>
       <c r="J38" s="2" t="inlineStr"/>
@@ -4532,7 +4532,7 @@
       </c>
       <c r="D39" s="2" t="inlineStr">
         <is>
-          <t>100nF/50V，X7R（统一采购建议）</t>
+          <t>100nF/50V，建议X7R</t>
         </is>
       </c>
       <c r="E39" s="2" t="inlineStr">
@@ -4548,12 +4548,12 @@
       </c>
       <c r="H39" s="2" t="inlineStr">
         <is>
-          <t>用户已确认另购100nF/0805；数量/耐压/介质待核</t>
+          <t>已购100nF/50V/0805已确认；数量/介质待核</t>
         </is>
       </c>
       <c r="I39" s="2" t="inlineStr">
         <is>
-          <t>每板设计16只，用户回复买了0805，确认另有100nF备料；不将16只需求填作库存。50V/X7R仍为统一采购建议，实际料号/耐压/介质待核；472批次独立记4.7nF</t>
+          <t>用户补充50v，确认这批额定50V，符合当前统一采购耐压；每板设计16只，实际数量/介质/完整料号待核。X7R仍为建议，不将需求16只自动填作库存；472批次独立记4.7nF</t>
         </is>
       </c>
       <c r="J39" s="2" t="inlineStr"/>
@@ -4576,7 +4576,7 @@
       </c>
       <c r="D40" s="2" t="inlineStr">
         <is>
-          <t>100nF/50V，X7R（统一采购建议）</t>
+          <t>100nF/50V，建议X7R</t>
         </is>
       </c>
       <c r="E40" s="2" t="inlineStr">
@@ -4592,12 +4592,12 @@
       </c>
       <c r="H40" s="2" t="inlineStr">
         <is>
-          <t>用户已确认另购100nF/0805；数量/耐压/介质待核</t>
+          <t>已购100nF/50V/0805已确认；数量/介质待核</t>
         </is>
       </c>
       <c r="I40" s="2" t="inlineStr">
         <is>
-          <t>每板设计16只，用户回复买了0805，确认另有100nF备料；不将16只需求填作库存。50V/X7R仍为统一采购建议，实际料号/耐压/介质待核；472批次独立记4.7nF</t>
+          <t>用户补充50v，确认这批额定50V，符合当前统一采购耐压；每板设计16只，实际数量/介质/完整料号待核。X7R仍为建议，不将需求16只自动填作库存；472批次独立记4.7nF</t>
         </is>
       </c>
       <c r="J40" s="2" t="inlineStr"/>
@@ -4620,7 +4620,7 @@
       </c>
       <c r="D41" s="2" t="inlineStr">
         <is>
-          <t>100nF/50V，X7R（统一采购建议）</t>
+          <t>100nF/50V，建议X7R</t>
         </is>
       </c>
       <c r="E41" s="2" t="inlineStr">
@@ -4636,12 +4636,12 @@
       </c>
       <c r="H41" s="2" t="inlineStr">
         <is>
-          <t>用户已确认另购100nF/0805；数量/耐压/介质待核</t>
+          <t>已购100nF/50V/0805已确认；数量/介质待核</t>
         </is>
       </c>
       <c r="I41" s="2" t="inlineStr">
         <is>
-          <t>每板设计16只，用户回复买了0805，确认另有100nF备料；不将16只需求填作库存。50V/X7R仍为统一采购建议，实际料号/耐压/介质待核；472批次独立记4.7nF</t>
+          <t>用户补充50v，确认这批额定50V，符合当前统一采购耐压；每板设计16只，实际数量/介质/完整料号待核。X7R仍为建议，不将需求16只自动填作库存；472批次独立记4.7nF</t>
         </is>
       </c>
       <c r="J41" s="2" t="inlineStr"/>
@@ -4664,7 +4664,7 @@
       </c>
       <c r="D42" s="2" t="inlineStr">
         <is>
-          <t>100nF/50V，X7R（统一采购建议）</t>
+          <t>100nF/50V，建议X7R</t>
         </is>
       </c>
       <c r="E42" s="2" t="inlineStr">
@@ -4680,12 +4680,12 @@
       </c>
       <c r="H42" s="2" t="inlineStr">
         <is>
-          <t>用户已确认另购100nF/0805；数量/耐压/介质待核</t>
+          <t>已购100nF/50V/0805已确认；数量/介质待核</t>
         </is>
       </c>
       <c r="I42" s="2" t="inlineStr">
         <is>
-          <t>每板设计16只，用户回复买了0805，确认另有100nF备料；不将16只需求填作库存。50V/X7R仍为统一采购建议，实际料号/耐压/介质待核；472批次独立记4.7nF</t>
+          <t>用户补充50v，确认这批额定50V，符合当前统一采购耐压；每板设计16只，实际数量/介质/完整料号待核。X7R仍为建议，不将需求16只自动填作库存；472批次独立记4.7nF</t>
         </is>
       </c>
       <c r="J42" s="2" t="inlineStr">
@@ -8936,7 +8936,7 @@
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>原472批次实际4.7nF；现确认另购100nF/0805</t>
+          <t>原472批次实际4.7nF；另购100nF/50V/0805已确认</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
@@ -8946,7 +8946,7 @@
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>已购状态确认，数量/耐压/介质待核；不默认库存16只或已经足量</t>
+          <t>50V额定确认；数量/介质/完整料号待核，不默认库存16只或已经足量</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Confirm X7R dielectric for purchased 100nF 50V 0805 capacitors
</commit_message>
<xml_diff>
--- a/projects/2026-electronics-contest/g-buck/rev-c2/downloads/GBUCK_RevC2_updated_BOM.xlsx
+++ b/projects/2026-electronics-contest/g-buck/rev-c2/downloads/GBUCK_RevC2_updated_BOM.xlsx
@@ -484,7 +484,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>本次比较3384d1c；用户确认已购100nF/0805的额定耐压50V，更新物料记录；实际数量/介质/完整料号待核。设计参数、用量与PCB保持。</t>
+          <t>本次比较3033d8b；用户确认已购100nF/50V/0805标有X7R，更新介质确认状态；实际库存数量/完整料号与容差未提供。设计参数、用量与PCB保持。</t>
         </is>
       </c>
     </row>
@@ -592,7 +592,7 @@
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>472批次已确认4.7nF；随后用户确认另外买了100nF/0805，两批分开记录。100nF/0805已购且50V已确认，实际数量/介质/完整料号待核，不自动填16只库存或缺16只；4.7nF数量/额定也另核。</t>
+          <t>472批次已确认4.7nF；随后用户确认另外买了100nF/0805，两批分开记录。100nF/50V/0805/X7R已购并确认，实际数量/完整料号与容差待核，不自动填16只库存或缺16只；4.7nF数量/额定也另核。</t>
         </is>
       </c>
     </row>
@@ -676,7 +676,7 @@
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>相对3384d1c，仅补记已购100nF/0805的50V额定；原理图和PCB原生文件未改，网络/脚号/参数与数量保持；100nF设计仍16只。</t>
+          <t>相对3033d8b，仅补记已购100nF/50V/0805的X7R介质确认；原理图和PCB原生文件未改，网络/脚号/设计参数与数量保持；100nF设计仍16只。</t>
         </is>
       </c>
     </row>
@@ -688,7 +688,7 @@
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>100nF/50V/0805已获用户确认，符合现有统一采购耐压；仅撤销该批耐压待核标签。数量/介质/完整料号待核，不自动填写库存或补购数量。设计需求、45采购行/120位号及全部PCB几何保持，无新增器件或替换要求。</t>
+          <t>100nF/50V/0805/X7R已获用户确认；撤销该批介质待核标签，无新增器件、换料或改板要求。实际库存数量/完整料号与容差未提供，不自动填库存或补购数量；设计需求、45采购行/120位号及全部PCB几何保持。</t>
         </is>
       </c>
     </row>
@@ -1567,7 +1567,7 @@
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>100nF/50V，建议X7R</t>
+          <t>100nF/50V，X7R</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
@@ -1593,12 +1593,12 @@
       </c>
       <c r="I20" s="2" t="inlineStr">
         <is>
-          <t>已购100nF/50V/0805已确认；数量/介质待核</t>
+          <t>已购100nF/50V/0805/X7R已确认；数量待核</t>
         </is>
       </c>
       <c r="J20" s="2" t="inlineStr">
         <is>
-          <t>用户补充50v，确认这批额定50V，符合当前统一采购耐压；每板设计16只，实际数量/介质/完整料号待核。X7R仍为建议，不将需求16只自动填作库存；472批次独立记4.7nF</t>
+          <t>用户对是否标有X7R回复有，确认该批介质X7R；每板设计16只，实际库存数量/完整料号与容差未提供，不将需求16只自动填作库存；472批次独立记4.7nF</t>
         </is>
       </c>
     </row>
@@ -4004,7 +4004,7 @@
       </c>
       <c r="D27" s="2" t="inlineStr">
         <is>
-          <t>100nF/50V，建议X7R</t>
+          <t>100nF/50V，X7R</t>
         </is>
       </c>
       <c r="E27" s="2" t="inlineStr">
@@ -4020,12 +4020,12 @@
       </c>
       <c r="H27" s="2" t="inlineStr">
         <is>
-          <t>已购100nF/50V/0805已确认；数量/介质待核</t>
+          <t>已购100nF/50V/0805/X7R已确认；数量待核</t>
         </is>
       </c>
       <c r="I27" s="2" t="inlineStr">
         <is>
-          <t>用户补充50v，确认这批额定50V，符合当前统一采购耐压；每板设计16只，实际数量/介质/完整料号待核。X7R仍为建议，不将需求16只自动填作库存；472批次独立记4.7nF</t>
+          <t>用户对是否标有X7R回复有，确认该批介质X7R；每板设计16只，实际库存数量/完整料号与容差未提供，不将需求16只自动填作库存；472批次独立记4.7nF</t>
         </is>
       </c>
       <c r="J27" s="2" t="inlineStr"/>
@@ -4048,7 +4048,7 @@
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t>100nF/50V，建议X7R</t>
+          <t>100nF/50V，X7R</t>
         </is>
       </c>
       <c r="E28" s="2" t="inlineStr">
@@ -4064,12 +4064,12 @@
       </c>
       <c r="H28" s="2" t="inlineStr">
         <is>
-          <t>已购100nF/50V/0805已确认；数量/介质待核</t>
+          <t>已购100nF/50V/0805/X7R已确认；数量待核</t>
         </is>
       </c>
       <c r="I28" s="2" t="inlineStr">
         <is>
-          <t>用户补充50v，确认这批额定50V，符合当前统一采购耐压；每板设计16只，实际数量/介质/完整料号待核。X7R仍为建议，不将需求16只自动填作库存；472批次独立记4.7nF</t>
+          <t>用户对是否标有X7R回复有，确认该批介质X7R；每板设计16只，实际库存数量/完整料号与容差未提供，不将需求16只自动填作库存；472批次独立记4.7nF</t>
         </is>
       </c>
       <c r="J28" s="2" t="inlineStr"/>
@@ -4092,7 +4092,7 @@
       </c>
       <c r="D29" s="2" t="inlineStr">
         <is>
-          <t>100nF/50V，建议X7R</t>
+          <t>100nF/50V，X7R</t>
         </is>
       </c>
       <c r="E29" s="2" t="inlineStr">
@@ -4108,12 +4108,12 @@
       </c>
       <c r="H29" s="2" t="inlineStr">
         <is>
-          <t>已购100nF/50V/0805已确认；数量/介质待核</t>
+          <t>已购100nF/50V/0805/X7R已确认；数量待核</t>
         </is>
       </c>
       <c r="I29" s="2" t="inlineStr">
         <is>
-          <t>用户补充50v，确认这批额定50V，符合当前统一采购耐压；每板设计16只，实际数量/介质/完整料号待核。X7R仍为建议，不将需求16只自动填作库存；472批次独立记4.7nF</t>
+          <t>用户对是否标有X7R回复有，确认该批介质X7R；每板设计16只，实际库存数量/完整料号与容差未提供，不将需求16只自动填作库存；472批次独立记4.7nF</t>
         </is>
       </c>
       <c r="J29" s="2" t="inlineStr"/>
@@ -4136,7 +4136,7 @@
       </c>
       <c r="D30" s="2" t="inlineStr">
         <is>
-          <t>100nF/50V，建议X7R</t>
+          <t>100nF/50V，X7R</t>
         </is>
       </c>
       <c r="E30" s="2" t="inlineStr">
@@ -4152,12 +4152,12 @@
       </c>
       <c r="H30" s="2" t="inlineStr">
         <is>
-          <t>已购100nF/50V/0805已确认；数量/介质待核</t>
+          <t>已购100nF/50V/0805/X7R已确认；数量待核</t>
         </is>
       </c>
       <c r="I30" s="2" t="inlineStr">
         <is>
-          <t>用户补充50v，确认这批额定50V，符合当前统一采购耐压；每板设计16只，实际数量/介质/完整料号待核。X7R仍为建议，不将需求16只自动填作库存；472批次独立记4.7nF</t>
+          <t>用户对是否标有X7R回复有，确认该批介质X7R；每板设计16只，实际库存数量/完整料号与容差未提供，不将需求16只自动填作库存；472批次独立记4.7nF</t>
         </is>
       </c>
       <c r="J30" s="2" t="inlineStr"/>
@@ -4180,7 +4180,7 @@
       </c>
       <c r="D31" s="2" t="inlineStr">
         <is>
-          <t>100nF/50V，建议X7R</t>
+          <t>100nF/50V，X7R</t>
         </is>
       </c>
       <c r="E31" s="2" t="inlineStr">
@@ -4196,12 +4196,12 @@
       </c>
       <c r="H31" s="2" t="inlineStr">
         <is>
-          <t>已购100nF/50V/0805已确认；数量/介质待核</t>
+          <t>已购100nF/50V/0805/X7R已确认；数量待核</t>
         </is>
       </c>
       <c r="I31" s="2" t="inlineStr">
         <is>
-          <t>用户补充50v，确认这批额定50V，符合当前统一采购耐压；每板设计16只，实际数量/介质/完整料号待核。X7R仍为建议，不将需求16只自动填作库存；472批次独立记4.7nF</t>
+          <t>用户对是否标有X7R回复有，确认该批介质X7R；每板设计16只，实际库存数量/完整料号与容差未提供，不将需求16只自动填作库存；472批次独立记4.7nF</t>
         </is>
       </c>
       <c r="J31" s="2" t="inlineStr"/>
@@ -4224,7 +4224,7 @@
       </c>
       <c r="D32" s="2" t="inlineStr">
         <is>
-          <t>100nF/50V，建议X7R</t>
+          <t>100nF/50V，X7R</t>
         </is>
       </c>
       <c r="E32" s="2" t="inlineStr">
@@ -4240,12 +4240,12 @@
       </c>
       <c r="H32" s="2" t="inlineStr">
         <is>
-          <t>已购100nF/50V/0805已确认；数量/介质待核</t>
+          <t>已购100nF/50V/0805/X7R已确认；数量待核</t>
         </is>
       </c>
       <c r="I32" s="2" t="inlineStr">
         <is>
-          <t>用户补充50v，确认这批额定50V，符合当前统一采购耐压；每板设计16只，实际数量/介质/完整料号待核。X7R仍为建议，不将需求16只自动填作库存；472批次独立记4.7nF</t>
+          <t>用户对是否标有X7R回复有，确认该批介质X7R；每板设计16只，实际库存数量/完整料号与容差未提供，不将需求16只自动填作库存；472批次独立记4.7nF</t>
         </is>
       </c>
       <c r="J32" s="2" t="inlineStr"/>
@@ -4268,7 +4268,7 @@
       </c>
       <c r="D33" s="2" t="inlineStr">
         <is>
-          <t>100nF/50V，建议X7R</t>
+          <t>100nF/50V，X7R</t>
         </is>
       </c>
       <c r="E33" s="2" t="inlineStr">
@@ -4284,12 +4284,12 @@
       </c>
       <c r="H33" s="2" t="inlineStr">
         <is>
-          <t>已购100nF/50V/0805已确认；数量/介质待核</t>
+          <t>已购100nF/50V/0805/X7R已确认；数量待核</t>
         </is>
       </c>
       <c r="I33" s="2" t="inlineStr">
         <is>
-          <t>用户补充50v，确认这批额定50V，符合当前统一采购耐压；每板设计16只，实际数量/介质/完整料号待核。X7R仍为建议，不将需求16只自动填作库存；472批次独立记4.7nF</t>
+          <t>用户对是否标有X7R回复有，确认该批介质X7R；每板设计16只，实际库存数量/完整料号与容差未提供，不将需求16只自动填作库存；472批次独立记4.7nF</t>
         </is>
       </c>
       <c r="J33" s="2" t="inlineStr"/>
@@ -4312,7 +4312,7 @@
       </c>
       <c r="D34" s="2" t="inlineStr">
         <is>
-          <t>100nF/50V，建议X7R</t>
+          <t>100nF/50V，X7R</t>
         </is>
       </c>
       <c r="E34" s="2" t="inlineStr">
@@ -4328,12 +4328,12 @@
       </c>
       <c r="H34" s="2" t="inlineStr">
         <is>
-          <t>已购100nF/50V/0805已确认；数量/介质待核</t>
+          <t>已购100nF/50V/0805/X7R已确认；数量待核</t>
         </is>
       </c>
       <c r="I34" s="2" t="inlineStr">
         <is>
-          <t>用户补充50v，确认这批额定50V，符合当前统一采购耐压；每板设计16只，实际数量/介质/完整料号待核。X7R仍为建议，不将需求16只自动填作库存；472批次独立记4.7nF</t>
+          <t>用户对是否标有X7R回复有，确认该批介质X7R；每板设计16只，实际库存数量/完整料号与容差未提供，不将需求16只自动填作库存；472批次独立记4.7nF</t>
         </is>
       </c>
       <c r="J34" s="2" t="inlineStr"/>
@@ -4356,7 +4356,7 @@
       </c>
       <c r="D35" s="2" t="inlineStr">
         <is>
-          <t>100nF/50V，建议X7R</t>
+          <t>100nF/50V，X7R</t>
         </is>
       </c>
       <c r="E35" s="2" t="inlineStr">
@@ -4372,12 +4372,12 @@
       </c>
       <c r="H35" s="2" t="inlineStr">
         <is>
-          <t>已购100nF/50V/0805已确认；数量/介质待核</t>
+          <t>已购100nF/50V/0805/X7R已确认；数量待核</t>
         </is>
       </c>
       <c r="I35" s="2" t="inlineStr">
         <is>
-          <t>用户补充50v，确认这批额定50V，符合当前统一采购耐压；每板设计16只，实际数量/介质/完整料号待核。X7R仍为建议，不将需求16只自动填作库存；472批次独立记4.7nF</t>
+          <t>用户对是否标有X7R回复有，确认该批介质X7R；每板设计16只，实际库存数量/完整料号与容差未提供，不将需求16只自动填作库存；472批次独立记4.7nF</t>
         </is>
       </c>
       <c r="J35" s="2" t="inlineStr"/>
@@ -4400,7 +4400,7 @@
       </c>
       <c r="D36" s="2" t="inlineStr">
         <is>
-          <t>100nF/50V，建议X7R</t>
+          <t>100nF/50V，X7R</t>
         </is>
       </c>
       <c r="E36" s="2" t="inlineStr">
@@ -4416,12 +4416,12 @@
       </c>
       <c r="H36" s="2" t="inlineStr">
         <is>
-          <t>已购100nF/50V/0805已确认；数量/介质待核</t>
+          <t>已购100nF/50V/0805/X7R已确认；数量待核</t>
         </is>
       </c>
       <c r="I36" s="2" t="inlineStr">
         <is>
-          <t>用户补充50v，确认这批额定50V，符合当前统一采购耐压；每板设计16只，实际数量/介质/完整料号待核。X7R仍为建议，不将需求16只自动填作库存；472批次独立记4.7nF</t>
+          <t>用户对是否标有X7R回复有，确认该批介质X7R；每板设计16只，实际库存数量/完整料号与容差未提供，不将需求16只自动填作库存；472批次独立记4.7nF</t>
         </is>
       </c>
       <c r="J36" s="2" t="inlineStr"/>
@@ -4444,7 +4444,7 @@
       </c>
       <c r="D37" s="2" t="inlineStr">
         <is>
-          <t>100nF/50V，建议X7R</t>
+          <t>100nF/50V，X7R</t>
         </is>
       </c>
       <c r="E37" s="2" t="inlineStr">
@@ -4460,12 +4460,12 @@
       </c>
       <c r="H37" s="2" t="inlineStr">
         <is>
-          <t>已购100nF/50V/0805已确认；数量/介质待核</t>
+          <t>已购100nF/50V/0805/X7R已确认；数量待核</t>
         </is>
       </c>
       <c r="I37" s="2" t="inlineStr">
         <is>
-          <t>用户补充50v，确认这批额定50V，符合当前统一采购耐压；每板设计16只，实际数量/介质/完整料号待核。X7R仍为建议，不将需求16只自动填作库存；472批次独立记4.7nF</t>
+          <t>用户对是否标有X7R回复有，确认该批介质X7R；每板设计16只，实际库存数量/完整料号与容差未提供，不将需求16只自动填作库存；472批次独立记4.7nF</t>
         </is>
       </c>
       <c r="J37" s="2" t="inlineStr"/>
@@ -4488,7 +4488,7 @@
       </c>
       <c r="D38" s="2" t="inlineStr">
         <is>
-          <t>100nF/50V，建议X7R</t>
+          <t>100nF/50V，X7R</t>
         </is>
       </c>
       <c r="E38" s="2" t="inlineStr">
@@ -4504,12 +4504,12 @@
       </c>
       <c r="H38" s="2" t="inlineStr">
         <is>
-          <t>已购100nF/50V/0805已确认；数量/介质待核</t>
+          <t>已购100nF/50V/0805/X7R已确认；数量待核</t>
         </is>
       </c>
       <c r="I38" s="2" t="inlineStr">
         <is>
-          <t>用户补充50v，确认这批额定50V，符合当前统一采购耐压；每板设计16只，实际数量/介质/完整料号待核。X7R仍为建议，不将需求16只自动填作库存；472批次独立记4.7nF</t>
+          <t>用户对是否标有X7R回复有，确认该批介质X7R；每板设计16只，实际库存数量/完整料号与容差未提供，不将需求16只自动填作库存；472批次独立记4.7nF</t>
         </is>
       </c>
       <c r="J38" s="2" t="inlineStr"/>
@@ -4532,7 +4532,7 @@
       </c>
       <c r="D39" s="2" t="inlineStr">
         <is>
-          <t>100nF/50V，建议X7R</t>
+          <t>100nF/50V，X7R</t>
         </is>
       </c>
       <c r="E39" s="2" t="inlineStr">
@@ -4548,12 +4548,12 @@
       </c>
       <c r="H39" s="2" t="inlineStr">
         <is>
-          <t>已购100nF/50V/0805已确认；数量/介质待核</t>
+          <t>已购100nF/50V/0805/X7R已确认；数量待核</t>
         </is>
       </c>
       <c r="I39" s="2" t="inlineStr">
         <is>
-          <t>用户补充50v，确认这批额定50V，符合当前统一采购耐压；每板设计16只，实际数量/介质/完整料号待核。X7R仍为建议，不将需求16只自动填作库存；472批次独立记4.7nF</t>
+          <t>用户对是否标有X7R回复有，确认该批介质X7R；每板设计16只，实际库存数量/完整料号与容差未提供，不将需求16只自动填作库存；472批次独立记4.7nF</t>
         </is>
       </c>
       <c r="J39" s="2" t="inlineStr"/>
@@ -4576,7 +4576,7 @@
       </c>
       <c r="D40" s="2" t="inlineStr">
         <is>
-          <t>100nF/50V，建议X7R</t>
+          <t>100nF/50V，X7R</t>
         </is>
       </c>
       <c r="E40" s="2" t="inlineStr">
@@ -4592,12 +4592,12 @@
       </c>
       <c r="H40" s="2" t="inlineStr">
         <is>
-          <t>已购100nF/50V/0805已确认；数量/介质待核</t>
+          <t>已购100nF/50V/0805/X7R已确认；数量待核</t>
         </is>
       </c>
       <c r="I40" s="2" t="inlineStr">
         <is>
-          <t>用户补充50v，确认这批额定50V，符合当前统一采购耐压；每板设计16只，实际数量/介质/完整料号待核。X7R仍为建议，不将需求16只自动填作库存；472批次独立记4.7nF</t>
+          <t>用户对是否标有X7R回复有，确认该批介质X7R；每板设计16只，实际库存数量/完整料号与容差未提供，不将需求16只自动填作库存；472批次独立记4.7nF</t>
         </is>
       </c>
       <c r="J40" s="2" t="inlineStr"/>
@@ -4620,7 +4620,7 @@
       </c>
       <c r="D41" s="2" t="inlineStr">
         <is>
-          <t>100nF/50V，建议X7R</t>
+          <t>100nF/50V，X7R</t>
         </is>
       </c>
       <c r="E41" s="2" t="inlineStr">
@@ -4636,12 +4636,12 @@
       </c>
       <c r="H41" s="2" t="inlineStr">
         <is>
-          <t>已购100nF/50V/0805已确认；数量/介质待核</t>
+          <t>已购100nF/50V/0805/X7R已确认；数量待核</t>
         </is>
       </c>
       <c r="I41" s="2" t="inlineStr">
         <is>
-          <t>用户补充50v，确认这批额定50V，符合当前统一采购耐压；每板设计16只，实际数量/介质/完整料号待核。X7R仍为建议，不将需求16只自动填作库存；472批次独立记4.7nF</t>
+          <t>用户对是否标有X7R回复有，确认该批介质X7R；每板设计16只，实际库存数量/完整料号与容差未提供，不将需求16只自动填作库存；472批次独立记4.7nF</t>
         </is>
       </c>
       <c r="J41" s="2" t="inlineStr"/>
@@ -4664,7 +4664,7 @@
       </c>
       <c r="D42" s="2" t="inlineStr">
         <is>
-          <t>100nF/50V，建议X7R</t>
+          <t>100nF/50V，X7R</t>
         </is>
       </c>
       <c r="E42" s="2" t="inlineStr">
@@ -4680,12 +4680,12 @@
       </c>
       <c r="H42" s="2" t="inlineStr">
         <is>
-          <t>已购100nF/50V/0805已确认；数量/介质待核</t>
+          <t>已购100nF/50V/0805/X7R已确认；数量待核</t>
         </is>
       </c>
       <c r="I42" s="2" t="inlineStr">
         <is>
-          <t>用户补充50v，确认这批额定50V，符合当前统一采购耐压；每板设计16只，实际数量/介质/完整料号待核。X7R仍为建议，不将需求16只自动填作库存；472批次独立记4.7nF</t>
+          <t>用户对是否标有X7R回复有，确认该批介质X7R；每板设计16只，实际库存数量/完整料号与容差未提供，不将需求16只自动填作库存；472批次独立记4.7nF</t>
         </is>
       </c>
       <c r="J42" s="2" t="inlineStr">
@@ -8936,7 +8936,7 @@
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>原472批次实际4.7nF；另购100nF/50V/0805已确认</t>
+          <t>原472批次实际4.7nF；另购100nF/50V/0805/X7R已确认</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
@@ -8946,7 +8946,7 @@
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>50V额定确认；数量/介质/完整料号待核，不默认库存16只或已经足量</t>
+          <t>X7R介质确认；库存数量/完整料号与容差待核，不默认库存16只或已经足量</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Record 50 confirmed 100nF capacitors and calculate single-board shortfall
</commit_message>
<xml_diff>
--- a/projects/2026-electronics-contest/g-buck/rev-c2/downloads/GBUCK_RevC2_updated_BOM.xlsx
+++ b/projects/2026-electronics-contest/g-buck/rev-c2/downloads/GBUCK_RevC2_updated_BOM.xlsx
@@ -484,7 +484,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>本次比较3033d8b；用户确认已购100nF/50V/0805标有X7R，更新介质确认状态；实际库存数量/完整料号与容差未提供。设计参数、用量与PCB保持。</t>
+          <t>本次比较d2e1585；用户确认100nF/50V/0805/X7R买了50只。单板需16只，本项补购0只，装配一板后余34只；设计参数、用量与PCB保持。</t>
         </is>
       </c>
     </row>
@@ -520,7 +520,7 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>采购汇总G列填写现有可用数量，H列自动计算需补购数量；空白表示库存未核，不代表未购买。</t>
+          <t>采购汇总G列填写现有可用数量，H列自动计算需补购数量；100nF/X7R已按用户50只填G列，单板补购0只。其他空白表示库存未核，不代表未购买。</t>
         </is>
       </c>
     </row>
@@ -592,7 +592,7 @@
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>472批次已确认4.7nF；随后用户确认另外买了100nF/0805，两批分开记录。100nF/50V/0805/X7R已购并确认，实际数量/完整料号与容差待核，不自动填16只库存或缺16只；4.7nF数量/额定也另核。</t>
+          <t>472批次已确认4.7nF；随后用户确认另外买了100nF/0805，两批分开记录。100nF/50V/0805/X7R已购50只，单板需求16只，补购0只，装配一板后余34只；完整料号/容差未提供；4.7nF数量/额定也另核。</t>
         </is>
       </c>
     </row>
@@ -676,7 +676,7 @@
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>相对3033d8b，仅补记已购100nF/50V/0805的X7R介质确认；原理图和PCB原生文件未改，网络/脚号/设计参数与数量保持；100nF设计仍16只。</t>
+          <t>相对d2e1585，仅登记100nF/50V/0805/X7R的50只备料；原理图和PCB原生文件未改，网络/脚号/设计参数与用量保持，100nF单板仍需16只。</t>
         </is>
       </c>
     </row>
@@ -688,7 +688,7 @@
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>100nF/50V/0805/X7R已获用户确认；撤销该批介质待核标签，无新增器件、换料或改板要求。实际库存数量/完整料号与容差未提供，不自动填库存或补购数量；设计需求、45采购行/120位号及全部PCB几何保持。</t>
+          <t>100nF/50V/0805/X7R登记库存50只，单板补购0只，装配一板后余34只；Excel保留动态补购公式，CSV写入当前50/0。其余库存留空，设计需求、45采购行/120位号及PCB几何保持，无新增或换料要求。</t>
         </is>
       </c>
     </row>
@@ -1586,19 +1586,21 @@
       <c r="F20" s="2" t="n">
         <v>16</v>
       </c>
-      <c r="G20" s="3" t="n"/>
+      <c r="G20" s="3" t="n">
+        <v>50</v>
+      </c>
       <c r="H20" s="2">
         <f>IF(G20="","",MAX(F20-G20,0))</f>
         <v/>
       </c>
       <c r="I20" s="2" t="inlineStr">
         <is>
-          <t>已购100nF/50V/0805/X7R已确认；数量待核</t>
+          <t>100nF/50V/0805/X7R，已购50只</t>
         </is>
       </c>
       <c r="J20" s="2" t="inlineStr">
         <is>
-          <t>用户对是否标有X7R回复有，确认该批介质X7R；每板设计16只，实际库存数量/完整料号与容差未提供，不将需求16只自动填作库存；472批次独立记4.7nF</t>
+          <t>用户对数量回复50；按单板用16只，补购0只，装一板后余34只。完整料号/容差未提供；472批次独立记4.7nF，不混计库存</t>
         </is>
       </c>
     </row>
@@ -4020,12 +4022,12 @@
       </c>
       <c r="H27" s="2" t="inlineStr">
         <is>
-          <t>已购100nF/50V/0805/X7R已确认；数量待核</t>
+          <t>100nF/50V/0805/X7R，已购50只</t>
         </is>
       </c>
       <c r="I27" s="2" t="inlineStr">
         <is>
-          <t>用户对是否标有X7R回复有，确认该批介质X7R；每板设计16只，实际库存数量/完整料号与容差未提供，不将需求16只自动填作库存；472批次独立记4.7nF</t>
+          <t>用户对数量回复50；按单板用16只，补购0只，装一板后余34只。完整料号/容差未提供；472批次独立记4.7nF，不混计库存</t>
         </is>
       </c>
       <c r="J27" s="2" t="inlineStr"/>
@@ -4064,12 +4066,12 @@
       </c>
       <c r="H28" s="2" t="inlineStr">
         <is>
-          <t>已购100nF/50V/0805/X7R已确认；数量待核</t>
+          <t>100nF/50V/0805/X7R，已购50只</t>
         </is>
       </c>
       <c r="I28" s="2" t="inlineStr">
         <is>
-          <t>用户对是否标有X7R回复有，确认该批介质X7R；每板设计16只，实际库存数量/完整料号与容差未提供，不将需求16只自动填作库存；472批次独立记4.7nF</t>
+          <t>用户对数量回复50；按单板用16只，补购0只，装一板后余34只。完整料号/容差未提供；472批次独立记4.7nF，不混计库存</t>
         </is>
       </c>
       <c r="J28" s="2" t="inlineStr"/>
@@ -4108,12 +4110,12 @@
       </c>
       <c r="H29" s="2" t="inlineStr">
         <is>
-          <t>已购100nF/50V/0805/X7R已确认；数量待核</t>
+          <t>100nF/50V/0805/X7R，已购50只</t>
         </is>
       </c>
       <c r="I29" s="2" t="inlineStr">
         <is>
-          <t>用户对是否标有X7R回复有，确认该批介质X7R；每板设计16只，实际库存数量/完整料号与容差未提供，不将需求16只自动填作库存；472批次独立记4.7nF</t>
+          <t>用户对数量回复50；按单板用16只，补购0只，装一板后余34只。完整料号/容差未提供；472批次独立记4.7nF，不混计库存</t>
         </is>
       </c>
       <c r="J29" s="2" t="inlineStr"/>
@@ -4152,12 +4154,12 @@
       </c>
       <c r="H30" s="2" t="inlineStr">
         <is>
-          <t>已购100nF/50V/0805/X7R已确认；数量待核</t>
+          <t>100nF/50V/0805/X7R，已购50只</t>
         </is>
       </c>
       <c r="I30" s="2" t="inlineStr">
         <is>
-          <t>用户对是否标有X7R回复有，确认该批介质X7R；每板设计16只，实际库存数量/完整料号与容差未提供，不将需求16只自动填作库存；472批次独立记4.7nF</t>
+          <t>用户对数量回复50；按单板用16只，补购0只，装一板后余34只。完整料号/容差未提供；472批次独立记4.7nF，不混计库存</t>
         </is>
       </c>
       <c r="J30" s="2" t="inlineStr"/>
@@ -4196,12 +4198,12 @@
       </c>
       <c r="H31" s="2" t="inlineStr">
         <is>
-          <t>已购100nF/50V/0805/X7R已确认；数量待核</t>
+          <t>100nF/50V/0805/X7R，已购50只</t>
         </is>
       </c>
       <c r="I31" s="2" t="inlineStr">
         <is>
-          <t>用户对是否标有X7R回复有，确认该批介质X7R；每板设计16只，实际库存数量/完整料号与容差未提供，不将需求16只自动填作库存；472批次独立记4.7nF</t>
+          <t>用户对数量回复50；按单板用16只，补购0只，装一板后余34只。完整料号/容差未提供；472批次独立记4.7nF，不混计库存</t>
         </is>
       </c>
       <c r="J31" s="2" t="inlineStr"/>
@@ -4240,12 +4242,12 @@
       </c>
       <c r="H32" s="2" t="inlineStr">
         <is>
-          <t>已购100nF/50V/0805/X7R已确认；数量待核</t>
+          <t>100nF/50V/0805/X7R，已购50只</t>
         </is>
       </c>
       <c r="I32" s="2" t="inlineStr">
         <is>
-          <t>用户对是否标有X7R回复有，确认该批介质X7R；每板设计16只，实际库存数量/完整料号与容差未提供，不将需求16只自动填作库存；472批次独立记4.7nF</t>
+          <t>用户对数量回复50；按单板用16只，补购0只，装一板后余34只。完整料号/容差未提供；472批次独立记4.7nF，不混计库存</t>
         </is>
       </c>
       <c r="J32" s="2" t="inlineStr"/>
@@ -4284,12 +4286,12 @@
       </c>
       <c r="H33" s="2" t="inlineStr">
         <is>
-          <t>已购100nF/50V/0805/X7R已确认；数量待核</t>
+          <t>100nF/50V/0805/X7R，已购50只</t>
         </is>
       </c>
       <c r="I33" s="2" t="inlineStr">
         <is>
-          <t>用户对是否标有X7R回复有，确认该批介质X7R；每板设计16只，实际库存数量/完整料号与容差未提供，不将需求16只自动填作库存；472批次独立记4.7nF</t>
+          <t>用户对数量回复50；按单板用16只，补购0只，装一板后余34只。完整料号/容差未提供；472批次独立记4.7nF，不混计库存</t>
         </is>
       </c>
       <c r="J33" s="2" t="inlineStr"/>
@@ -4328,12 +4330,12 @@
       </c>
       <c r="H34" s="2" t="inlineStr">
         <is>
-          <t>已购100nF/50V/0805/X7R已确认；数量待核</t>
+          <t>100nF/50V/0805/X7R，已购50只</t>
         </is>
       </c>
       <c r="I34" s="2" t="inlineStr">
         <is>
-          <t>用户对是否标有X7R回复有，确认该批介质X7R；每板设计16只，实际库存数量/完整料号与容差未提供，不将需求16只自动填作库存；472批次独立记4.7nF</t>
+          <t>用户对数量回复50；按单板用16只，补购0只，装一板后余34只。完整料号/容差未提供；472批次独立记4.7nF，不混计库存</t>
         </is>
       </c>
       <c r="J34" s="2" t="inlineStr"/>
@@ -4372,12 +4374,12 @@
       </c>
       <c r="H35" s="2" t="inlineStr">
         <is>
-          <t>已购100nF/50V/0805/X7R已确认；数量待核</t>
+          <t>100nF/50V/0805/X7R，已购50只</t>
         </is>
       </c>
       <c r="I35" s="2" t="inlineStr">
         <is>
-          <t>用户对是否标有X7R回复有，确认该批介质X7R；每板设计16只，实际库存数量/完整料号与容差未提供，不将需求16只自动填作库存；472批次独立记4.7nF</t>
+          <t>用户对数量回复50；按单板用16只，补购0只，装一板后余34只。完整料号/容差未提供；472批次独立记4.7nF，不混计库存</t>
         </is>
       </c>
       <c r="J35" s="2" t="inlineStr"/>
@@ -4416,12 +4418,12 @@
       </c>
       <c r="H36" s="2" t="inlineStr">
         <is>
-          <t>已购100nF/50V/0805/X7R已确认；数量待核</t>
+          <t>100nF/50V/0805/X7R，已购50只</t>
         </is>
       </c>
       <c r="I36" s="2" t="inlineStr">
         <is>
-          <t>用户对是否标有X7R回复有，确认该批介质X7R；每板设计16只，实际库存数量/完整料号与容差未提供，不将需求16只自动填作库存；472批次独立记4.7nF</t>
+          <t>用户对数量回复50；按单板用16只，补购0只，装一板后余34只。完整料号/容差未提供；472批次独立记4.7nF，不混计库存</t>
         </is>
       </c>
       <c r="J36" s="2" t="inlineStr"/>
@@ -4460,12 +4462,12 @@
       </c>
       <c r="H37" s="2" t="inlineStr">
         <is>
-          <t>已购100nF/50V/0805/X7R已确认；数量待核</t>
+          <t>100nF/50V/0805/X7R，已购50只</t>
         </is>
       </c>
       <c r="I37" s="2" t="inlineStr">
         <is>
-          <t>用户对是否标有X7R回复有，确认该批介质X7R；每板设计16只，实际库存数量/完整料号与容差未提供，不将需求16只自动填作库存；472批次独立记4.7nF</t>
+          <t>用户对数量回复50；按单板用16只，补购0只，装一板后余34只。完整料号/容差未提供；472批次独立记4.7nF，不混计库存</t>
         </is>
       </c>
       <c r="J37" s="2" t="inlineStr"/>
@@ -4504,12 +4506,12 @@
       </c>
       <c r="H38" s="2" t="inlineStr">
         <is>
-          <t>已购100nF/50V/0805/X7R已确认；数量待核</t>
+          <t>100nF/50V/0805/X7R，已购50只</t>
         </is>
       </c>
       <c r="I38" s="2" t="inlineStr">
         <is>
-          <t>用户对是否标有X7R回复有，确认该批介质X7R；每板设计16只，实际库存数量/完整料号与容差未提供，不将需求16只自动填作库存；472批次独立记4.7nF</t>
+          <t>用户对数量回复50；按单板用16只，补购0只，装一板后余34只。完整料号/容差未提供；472批次独立记4.7nF，不混计库存</t>
         </is>
       </c>
       <c r="J38" s="2" t="inlineStr"/>
@@ -4548,12 +4550,12 @@
       </c>
       <c r="H39" s="2" t="inlineStr">
         <is>
-          <t>已购100nF/50V/0805/X7R已确认；数量待核</t>
+          <t>100nF/50V/0805/X7R，已购50只</t>
         </is>
       </c>
       <c r="I39" s="2" t="inlineStr">
         <is>
-          <t>用户对是否标有X7R回复有，确认该批介质X7R；每板设计16只，实际库存数量/完整料号与容差未提供，不将需求16只自动填作库存；472批次独立记4.7nF</t>
+          <t>用户对数量回复50；按单板用16只，补购0只，装一板后余34只。完整料号/容差未提供；472批次独立记4.7nF，不混计库存</t>
         </is>
       </c>
       <c r="J39" s="2" t="inlineStr"/>
@@ -4592,12 +4594,12 @@
       </c>
       <c r="H40" s="2" t="inlineStr">
         <is>
-          <t>已购100nF/50V/0805/X7R已确认；数量待核</t>
+          <t>100nF/50V/0805/X7R，已购50只</t>
         </is>
       </c>
       <c r="I40" s="2" t="inlineStr">
         <is>
-          <t>用户对是否标有X7R回复有，确认该批介质X7R；每板设计16只，实际库存数量/完整料号与容差未提供，不将需求16只自动填作库存；472批次独立记4.7nF</t>
+          <t>用户对数量回复50；按单板用16只，补购0只，装一板后余34只。完整料号/容差未提供；472批次独立记4.7nF，不混计库存</t>
         </is>
       </c>
       <c r="J40" s="2" t="inlineStr"/>
@@ -4636,12 +4638,12 @@
       </c>
       <c r="H41" s="2" t="inlineStr">
         <is>
-          <t>已购100nF/50V/0805/X7R已确认；数量待核</t>
+          <t>100nF/50V/0805/X7R，已购50只</t>
         </is>
       </c>
       <c r="I41" s="2" t="inlineStr">
         <is>
-          <t>用户对是否标有X7R回复有，确认该批介质X7R；每板设计16只，实际库存数量/完整料号与容差未提供，不将需求16只自动填作库存；472批次独立记4.7nF</t>
+          <t>用户对数量回复50；按单板用16只，补购0只，装一板后余34只。完整料号/容差未提供；472批次独立记4.7nF，不混计库存</t>
         </is>
       </c>
       <c r="J41" s="2" t="inlineStr"/>
@@ -4680,12 +4682,12 @@
       </c>
       <c r="H42" s="2" t="inlineStr">
         <is>
-          <t>已购100nF/50V/0805/X7R已确认；数量待核</t>
+          <t>100nF/50V/0805/X7R，已购50只</t>
         </is>
       </c>
       <c r="I42" s="2" t="inlineStr">
         <is>
-          <t>用户对是否标有X7R回复有，确认该批介质X7R；每板设计16只，实际库存数量/完整料号与容差未提供，不将需求16只自动填作库存；472批次独立记4.7nF</t>
+          <t>用户对数量回复50；按单板用16只，补购0只，装一板后余34只。完整料号/容差未提供；472批次独立记4.7nF，不混计库存</t>
         </is>
       </c>
       <c r="J42" s="2" t="inlineStr">
@@ -8936,17 +8938,17 @@
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>原472批次实际4.7nF；另购100nF/50V/0805/X7R已确认</t>
+          <t>原472批次实际4.7nF；另购100nF/50V/0805/X7R共50只</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>Rev C2仍需100nF共16只</t>
+          <t>Rev C2单板需100nF共16只</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>X7R介质确认；库存数量/完整料号与容差待核，不默认库存16只或已经足量</t>
+          <t>本项补购0只，装配一板后余34只；完整料号/容差未提供</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Confirm C0G dielectric for the 4.7nF capacitor batch
</commit_message>
<xml_diff>
--- a/projects/2026-electronics-contest/g-buck/rev-c2/downloads/GBUCK_RevC2_updated_BOM.xlsx
+++ b/projects/2026-electronics-contest/g-buck/rev-c2/downloads/GBUCK_RevC2_updated_BOM.xlsx
@@ -484,7 +484,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>本次比较d2e1585；用户确认100nF/50V/0805/X7R买了50只。单板需16只，本项补购0只，装配一板后余34只；设计参数、用量与PCB保持。</t>
+          <t>本次比较68cd4f9；用户确认4.7nF这批标有C0G，更新介质状态；该批耐压/数量/完整料号待核。100nF库存50只保留，设计参数、用量与PCB保持。</t>
         </is>
       </c>
     </row>
@@ -592,7 +592,7 @@
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>472批次已确认4.7nF；随后用户确认另外买了100nF/0805，两批分开记录。100nF/50V/0805/X7R已购50只，单板需求16只，补购0只，装配一板后余34只；完整料号/容差未提供；4.7nF数量/额定也另核。</t>
+          <t>472批次已确认4.7nF；随后用户确认另外买了100nF/0805，两批分开记录。100nF/50V/0805/X7R已购50只，单板需求16只，补购0只，装配一板后余34只；完整料号/容差未提供；4.7nF的C0G介质已获用户确认，数量/耐压/完整料号另核；不把原表CL21B472JBANNNC直接登记为已确认C0G料号。</t>
         </is>
       </c>
     </row>
@@ -676,7 +676,7 @@
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>相对d2e1585，仅登记100nF/50V/0805/X7R的50只备料；原理图和PCB原生文件未改，网络/脚号/设计参数与用量保持，100nF单板仍需16只。</t>
+          <t>相对68cd4f9，仅补记4.7nF批次的C0G介质确认；原理图和PCB原生文件未改，网络/脚号/设计参数与用量保持，4.7nF单板仍需5只。</t>
         </is>
       </c>
     </row>
@@ -688,7 +688,7 @@
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>100nF/50V/0805/X7R登记库存50只，单板补购0只，装配一板后余34只；Excel保留动态补购公式，CSV写入当前50/0。其余库存留空，设计需求、45采购行/120位号及PCB几何保持，无新增或换料要求。</t>
+          <t>4.7nF/C0G撤销介质待核标签，符合C_VINP_ADC的C0G要求；该批耐压/数量/完整料号待核，不据此填可用库存。100nF的50只库存/单板补购0保持。设计需求、45采购行/120位号及PCB几何保持，无本轮新增或换料要求。</t>
         </is>
       </c>
     </row>
@@ -1612,7 +1612,7 @@
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>4.7nF/50V，建议统一C0G/NP0</t>
+          <t>4.7nF/50V，C0G</t>
         </is>
       </c>
       <c r="C21" s="2" t="inlineStr">
@@ -1638,12 +1638,12 @@
       </c>
       <c r="I21" s="2" t="inlineStr">
         <is>
-          <t>用户已确认该批容量4.7nF；数量/介质另核</t>
+          <t>用户已确认4.7nF/C0G；耐压/数量待核</t>
         </is>
       </c>
       <c r="J21" s="2" t="inlineStr">
         <is>
-          <t>设计共5只；参数表CL21B472JBANNNC与本轮确认容量一致，不计入100nF。容量确认不证明耐压/介质相容；C_VINP_ADC明确C0G，不能凭容量直接抵扣可用库存</t>
+          <t>用户回复有cog，按C0G记录，符合C_VINP_ADC的介质要求；单板5只，50V为当前采购耐压要求，尚未由用户确认这批实际耐压。完整料号/数量/容差待核；原表CL21B472JBANNNC保留历史，不作为本批C0G完整料号</t>
         </is>
       </c>
     </row>
@@ -4714,7 +4714,7 @@
       </c>
       <c r="D43" s="2" t="inlineStr">
         <is>
-          <t>4.7nF/50V，建议统一C0G/NP0</t>
+          <t>4.7nF/50V，C0G</t>
         </is>
       </c>
       <c r="E43" s="2" t="inlineStr">
@@ -4730,12 +4730,12 @@
       </c>
       <c r="H43" s="2" t="inlineStr">
         <is>
-          <t>用户已确认该批容量4.7nF；数量/介质另核</t>
+          <t>用户已确认4.7nF/C0G；耐压/数量待核</t>
         </is>
       </c>
       <c r="I43" s="2" t="inlineStr">
         <is>
-          <t>设计共5只；参数表CL21B472JBANNNC与本轮确认容量一致，不计入100nF。容量确认不证明耐压/介质相容；C_VINP_ADC明确C0G，不能凭容量直接抵扣可用库存</t>
+          <t>用户回复有cog，按C0G记录，符合C_VINP_ADC的介质要求；单板5只，50V为当前采购耐压要求，尚未由用户确认这批实际耐压。完整料号/数量/容差待核；原表CL21B472JBANNNC保留历史，不作为本批C0G完整料号</t>
         </is>
       </c>
       <c r="J43" s="2" t="inlineStr"/>
@@ -4758,7 +4758,7 @@
       </c>
       <c r="D44" s="2" t="inlineStr">
         <is>
-          <t>4.7nF/50V，建议统一C0G/NP0</t>
+          <t>4.7nF/50V，C0G</t>
         </is>
       </c>
       <c r="E44" s="2" t="inlineStr">
@@ -4774,12 +4774,12 @@
       </c>
       <c r="H44" s="2" t="inlineStr">
         <is>
-          <t>用户已确认该批容量4.7nF；数量/介质另核</t>
+          <t>用户已确认4.7nF/C0G；耐压/数量待核</t>
         </is>
       </c>
       <c r="I44" s="2" t="inlineStr">
         <is>
-          <t>设计共5只；参数表CL21B472JBANNNC与本轮确认容量一致，不计入100nF。容量确认不证明耐压/介质相容；C_VINP_ADC明确C0G，不能凭容量直接抵扣可用库存</t>
+          <t>用户回复有cog，按C0G记录，符合C_VINP_ADC的介质要求；单板5只，50V为当前采购耐压要求，尚未由用户确认这批实际耐压。完整料号/数量/容差待核；原表CL21B472JBANNNC保留历史，不作为本批C0G完整料号</t>
         </is>
       </c>
       <c r="J44" s="2" t="inlineStr"/>
@@ -4802,7 +4802,7 @@
       </c>
       <c r="D45" s="2" t="inlineStr">
         <is>
-          <t>4.7nF/50V，建议统一C0G/NP0</t>
+          <t>4.7nF/50V，C0G</t>
         </is>
       </c>
       <c r="E45" s="2" t="inlineStr">
@@ -4818,12 +4818,12 @@
       </c>
       <c r="H45" s="2" t="inlineStr">
         <is>
-          <t>用户已确认该批容量4.7nF；数量/介质另核</t>
+          <t>用户已确认4.7nF/C0G；耐压/数量待核</t>
         </is>
       </c>
       <c r="I45" s="2" t="inlineStr">
         <is>
-          <t>设计共5只；参数表CL21B472JBANNNC与本轮确认容量一致，不计入100nF。容量确认不证明耐压/介质相容；C_VINP_ADC明确C0G，不能凭容量直接抵扣可用库存</t>
+          <t>用户回复有cog，按C0G记录，符合C_VINP_ADC的介质要求；单板5只，50V为当前采购耐压要求，尚未由用户确认这批实际耐压。完整料号/数量/容差待核；原表CL21B472JBANNNC保留历史，不作为本批C0G完整料号</t>
         </is>
       </c>
       <c r="J45" s="2" t="inlineStr"/>
@@ -4846,7 +4846,7 @@
       </c>
       <c r="D46" s="2" t="inlineStr">
         <is>
-          <t>4.7nF/50V，建议统一C0G/NP0</t>
+          <t>4.7nF/50V，C0G</t>
         </is>
       </c>
       <c r="E46" s="2" t="inlineStr">
@@ -4862,12 +4862,12 @@
       </c>
       <c r="H46" s="2" t="inlineStr">
         <is>
-          <t>用户已确认该批容量4.7nF；数量/介质另核</t>
+          <t>用户已确认4.7nF/C0G；耐压/数量待核</t>
         </is>
       </c>
       <c r="I46" s="2" t="inlineStr">
         <is>
-          <t>设计共5只；参数表CL21B472JBANNNC与本轮确认容量一致，不计入100nF。容量确认不证明耐压/介质相容；C_VINP_ADC明确C0G，不能凭容量直接抵扣可用库存</t>
+          <t>用户回复有cog，按C0G记录，符合C_VINP_ADC的介质要求；单板5只，50V为当前采购耐压要求，尚未由用户确认这批实际耐压。完整料号/数量/容差待核；原表CL21B472JBANNNC保留历史，不作为本批C0G完整料号</t>
         </is>
       </c>
       <c r="J46" s="2" t="inlineStr"/>
@@ -4890,7 +4890,7 @@
       </c>
       <c r="D47" s="2" t="inlineStr">
         <is>
-          <t>4.7nF/50V，建议统一C0G/NP0</t>
+          <t>4.7nF/50V，C0G</t>
         </is>
       </c>
       <c r="E47" s="2" t="inlineStr">
@@ -4906,12 +4906,12 @@
       </c>
       <c r="H47" s="2" t="inlineStr">
         <is>
-          <t>用户已确认该批容量4.7nF；数量/介质另核</t>
+          <t>用户已确认4.7nF/C0G；耐压/数量待核</t>
         </is>
       </c>
       <c r="I47" s="2" t="inlineStr">
         <is>
-          <t>设计共5只；参数表CL21B472JBANNNC与本轮确认容量一致，不计入100nF。容量确认不证明耐压/介质相容；C_VINP_ADC明确C0G，不能凭容量直接抵扣可用库存</t>
+          <t>用户回复有cog，按C0G记录，符合C_VINP_ADC的介质要求；单板5只，50V为当前采购耐压要求，尚未由用户确认这批实际耐压。完整料号/数量/容差待核；原表CL21B472JBANNNC保留历史，不作为本批C0G完整料号</t>
         </is>
       </c>
       <c r="J47" s="2" t="inlineStr">
@@ -8960,7 +8960,7 @@
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>用户确认所询问批次实际4.7nF</t>
+          <t>用户确认该批4.7nF且标有C0G</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
@@ -8970,7 +8970,7 @@
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>容量确认；可用数量/耐压/介质另核，C_VINP_ADC要求C0G，不凭容量认定相容</t>
+          <t>C0G介质确认；该批耐压/数量/完整料号另核，原表料号不作为C0G的完整料号证据</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Distinguish generic MLCC code charts from purchased capacitor evidence
</commit_message>
<xml_diff>
--- a/projects/2026-electronics-contest/g-buck/rev-c2/downloads/GBUCK_RevC2_updated_BOM.xlsx
+++ b/projects/2026-electronics-contest/g-buck/rev-c2/downloads/GBUCK_RevC2_updated_BOM.xlsx
@@ -484,7 +484,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>本次比较68cd4f9；用户确认4.7nF这批标有C0G，更新介质状态；该批耐压/数量/完整料号待核。100nF库存50只保留，设计参数、用量与PCB保持。</t>
+          <t>本次比较8e2722c；新图为通用电容编码说明，不是实购型号证明。原表料号按图解码为X7R/50V，与先前口头C0G有差异，4.7nF实际介质/耐压改记待核；设计与100nF库存保持。</t>
         </is>
       </c>
     </row>
@@ -592,7 +592,7 @@
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>472批次已确认4.7nF；随后用户确认另外买了100nF/0805，两批分开记录。100nF/50V/0805/X7R已购50只，单板需求16只，补购0只，装配一板后余34只；完整料号/容差未提供；4.7nF的C0G介质已获用户确认，数量/耐压/完整料号另核；不把原表CL21B472JBANNNC直接登记为已确认C0G料号。</t>
+          <t>472批次已确认4.7nF；随后用户确认另外买了100nF/0805，两批分开记录。100nF/50V/0805/X7R已购50只，单板需求16只，补购0只，装配一板后余34只；完整料号/容差未提供；4.7nF先前口头C0G与原表型号解码X7R有差异，实际完整型号待核；不从通用图的C0G选项推定实物介质，不把解码出的50V当成实物已确认。</t>
         </is>
       </c>
     </row>
@@ -676,7 +676,7 @@
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>相对68cd4f9，仅补记4.7nF批次的C0G介质确认；原理图和PCB原生文件未改，网络/脚号/设计参数与用量保持，4.7nF单板仍需5只。</t>
+          <t>相对8e2722c，仅更新4.7nF证据复核状态；原理图和PCB原生文件未改，网络/脚号/设计参数与用量保持，4.7nF单板仍需5只，C_VINP_ADC仍要求C0G。</t>
         </is>
       </c>
     </row>
@@ -688,7 +688,7 @@
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>4.7nF/C0G撤销介质待核标签，符合C_VINP_ADC的C0G要求；该批耐压/数量/完整料号待核，不据此填可用库存。100nF的50只库存/单板补购0保持。设计需求、45采购行/120位号及PCB几何保持，无本轮新增或换料要求。</t>
+          <t>4.7nF实际型号/介质/耐压/数量待核，C0G仍是C_VINP_ADC的要求；若实物是原表X7R款，不直接代装该位置，是否补购待实际型号/库存核实。100nF库存50只/单板补购0保持；45采购行/120位号及全部PCB几何未改，本轮没有执行换料。</t>
         </is>
       </c>
     </row>
@@ -1612,7 +1612,7 @@
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>4.7nF/50V，C0G</t>
+          <t>4.7nF/50V，C0G（统一采购建议）</t>
         </is>
       </c>
       <c r="C21" s="2" t="inlineStr">
@@ -1638,12 +1638,12 @@
       </c>
       <c r="I21" s="2" t="inlineStr">
         <is>
-          <t>用户已确认4.7nF/C0G；耐压/数量待核</t>
+          <t>通用编码图未显示实购型号；介质/耐压待核</t>
         </is>
       </c>
       <c r="J21" s="2" t="inlineStr">
         <is>
-          <t>用户回复有cog，按C0G记录，符合C_VINP_ADC的介质要求；单板5只，50V为当前采购耐压要求，尚未由用户确认这批实际耐压。完整料号/数量/容差待核；原表CL21B472JBANNNC保留历史，不作为本批C0G完整料号</t>
+          <t>用户先前称有C0G，随后提供通用编码图；不能据图中C=C0G确认所选实物。若实际仍为原表CL21B472JBANNNC，按图解码0805/4.7nF/±5%/50V/X7R，与口头C0G有差异。请核对实际完整型号；C_VINP_ADC要求C0G，不直接以X7R代装，其他位置也须按要求核对。单板共5只、库存数量未知</t>
         </is>
       </c>
     </row>
@@ -4714,7 +4714,7 @@
       </c>
       <c r="D43" s="2" t="inlineStr">
         <is>
-          <t>4.7nF/50V，C0G</t>
+          <t>4.7nF/50V，C0G（统一采购建议）</t>
         </is>
       </c>
       <c r="E43" s="2" t="inlineStr">
@@ -4730,12 +4730,12 @@
       </c>
       <c r="H43" s="2" t="inlineStr">
         <is>
-          <t>用户已确认4.7nF/C0G；耐压/数量待核</t>
+          <t>通用编码图未显示实购型号；介质/耐压待核</t>
         </is>
       </c>
       <c r="I43" s="2" t="inlineStr">
         <is>
-          <t>用户回复有cog，按C0G记录，符合C_VINP_ADC的介质要求；单板5只，50V为当前采购耐压要求，尚未由用户确认这批实际耐压。完整料号/数量/容差待核；原表CL21B472JBANNNC保留历史，不作为本批C0G完整料号</t>
+          <t>用户先前称有C0G，随后提供通用编码图；不能据图中C=C0G确认所选实物。若实际仍为原表CL21B472JBANNNC，按图解码0805/4.7nF/±5%/50V/X7R，与口头C0G有差异。请核对实际完整型号；C_VINP_ADC要求C0G，不直接以X7R代装，其他位置也须按要求核对。单板共5只、库存数量未知</t>
         </is>
       </c>
       <c r="J43" s="2" t="inlineStr"/>
@@ -4758,7 +4758,7 @@
       </c>
       <c r="D44" s="2" t="inlineStr">
         <is>
-          <t>4.7nF/50V，C0G</t>
+          <t>4.7nF/50V，C0G（统一采购建议）</t>
         </is>
       </c>
       <c r="E44" s="2" t="inlineStr">
@@ -4774,12 +4774,12 @@
       </c>
       <c r="H44" s="2" t="inlineStr">
         <is>
-          <t>用户已确认4.7nF/C0G；耐压/数量待核</t>
+          <t>通用编码图未显示实购型号；介质/耐压待核</t>
         </is>
       </c>
       <c r="I44" s="2" t="inlineStr">
         <is>
-          <t>用户回复有cog，按C0G记录，符合C_VINP_ADC的介质要求；单板5只，50V为当前采购耐压要求，尚未由用户确认这批实际耐压。完整料号/数量/容差待核；原表CL21B472JBANNNC保留历史，不作为本批C0G完整料号</t>
+          <t>用户先前称有C0G，随后提供通用编码图；不能据图中C=C0G确认所选实物。若实际仍为原表CL21B472JBANNNC，按图解码0805/4.7nF/±5%/50V/X7R，与口头C0G有差异。请核对实际完整型号；C_VINP_ADC要求C0G，不直接以X7R代装，其他位置也须按要求核对。单板共5只、库存数量未知</t>
         </is>
       </c>
       <c r="J44" s="2" t="inlineStr"/>
@@ -4802,7 +4802,7 @@
       </c>
       <c r="D45" s="2" t="inlineStr">
         <is>
-          <t>4.7nF/50V，C0G</t>
+          <t>4.7nF/50V，C0G（统一采购建议）</t>
         </is>
       </c>
       <c r="E45" s="2" t="inlineStr">
@@ -4818,12 +4818,12 @@
       </c>
       <c r="H45" s="2" t="inlineStr">
         <is>
-          <t>用户已确认4.7nF/C0G；耐压/数量待核</t>
+          <t>通用编码图未显示实购型号；介质/耐压待核</t>
         </is>
       </c>
       <c r="I45" s="2" t="inlineStr">
         <is>
-          <t>用户回复有cog，按C0G记录，符合C_VINP_ADC的介质要求；单板5只，50V为当前采购耐压要求，尚未由用户确认这批实际耐压。完整料号/数量/容差待核；原表CL21B472JBANNNC保留历史，不作为本批C0G完整料号</t>
+          <t>用户先前称有C0G，随后提供通用编码图；不能据图中C=C0G确认所选实物。若实际仍为原表CL21B472JBANNNC，按图解码0805/4.7nF/±5%/50V/X7R，与口头C0G有差异。请核对实际完整型号；C_VINP_ADC要求C0G，不直接以X7R代装，其他位置也须按要求核对。单板共5只、库存数量未知</t>
         </is>
       </c>
       <c r="J45" s="2" t="inlineStr"/>
@@ -4846,7 +4846,7 @@
       </c>
       <c r="D46" s="2" t="inlineStr">
         <is>
-          <t>4.7nF/50V，C0G</t>
+          <t>4.7nF/50V，C0G（统一采购建议）</t>
         </is>
       </c>
       <c r="E46" s="2" t="inlineStr">
@@ -4862,12 +4862,12 @@
       </c>
       <c r="H46" s="2" t="inlineStr">
         <is>
-          <t>用户已确认4.7nF/C0G；耐压/数量待核</t>
+          <t>通用编码图未显示实购型号；介质/耐压待核</t>
         </is>
       </c>
       <c r="I46" s="2" t="inlineStr">
         <is>
-          <t>用户回复有cog，按C0G记录，符合C_VINP_ADC的介质要求；单板5只，50V为当前采购耐压要求，尚未由用户确认这批实际耐压。完整料号/数量/容差待核；原表CL21B472JBANNNC保留历史，不作为本批C0G完整料号</t>
+          <t>用户先前称有C0G，随后提供通用编码图；不能据图中C=C0G确认所选实物。若实际仍为原表CL21B472JBANNNC，按图解码0805/4.7nF/±5%/50V/X7R，与口头C0G有差异。请核对实际完整型号；C_VINP_ADC要求C0G，不直接以X7R代装，其他位置也须按要求核对。单板共5只、库存数量未知</t>
         </is>
       </c>
       <c r="J46" s="2" t="inlineStr"/>
@@ -4890,7 +4890,7 @@
       </c>
       <c r="D47" s="2" t="inlineStr">
         <is>
-          <t>4.7nF/50V，C0G</t>
+          <t>4.7nF/50V，C0G（统一采购建议）</t>
         </is>
       </c>
       <c r="E47" s="2" t="inlineStr">
@@ -4906,12 +4906,12 @@
       </c>
       <c r="H47" s="2" t="inlineStr">
         <is>
-          <t>用户已确认4.7nF/C0G；耐压/数量待核</t>
+          <t>通用编码图未显示实购型号；介质/耐压待核</t>
         </is>
       </c>
       <c r="I47" s="2" t="inlineStr">
         <is>
-          <t>用户回复有cog，按C0G记录，符合C_VINP_ADC的介质要求；单板5只，50V为当前采购耐压要求，尚未由用户确认这批实际耐压。完整料号/数量/容差待核；原表CL21B472JBANNNC保留历史，不作为本批C0G完整料号</t>
+          <t>用户先前称有C0G，随后提供通用编码图；不能据图中C=C0G确认所选实物。若实际仍为原表CL21B472JBANNNC，按图解码0805/4.7nF/±5%/50V/X7R，与口头C0G有差异。请核对实际完整型号；C_VINP_ADC要求C0G，不直接以X7R代装，其他位置也须按要求核对。单板共5只、库存数量未知</t>
         </is>
       </c>
       <c r="J47" s="2" t="inlineStr">
@@ -8960,7 +8960,7 @@
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>用户确认该批4.7nF且标有C0G</t>
+          <t>口头C0G；原表CL21B472JBANNNC按新图解码X7R/50V</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
@@ -8970,7 +8970,7 @@
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>C0G介质确认；该批耐压/数量/完整料号另核，原表料号不作为C0G的完整料号证据</t>
+          <t>实际完整型号待核；通用图不证明所选款，C_VINP_ADC仍需C0G，不能据本次图直接认定实物合格</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Confirm actual X7R part and separate C0G requirement for VIN ADC
</commit_message>
<xml_diff>
--- a/projects/2026-electronics-contest/g-buck/rev-c2/downloads/GBUCK_RevC2_updated_BOM.xlsx
+++ b/projects/2026-electronics-contest/g-buck/rev-c2/downloads/GBUCK_RevC2_updated_BOM.xlsx
@@ -16,7 +16,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'使用说明'!$A$1:$B$20</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'使用说明'!$1:$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'采购汇总'!$A$1:$J$46</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'采购汇总'!$A$1:$J$47</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'采购汇总'!$1:$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'逐位号_120项'!$A$1:$J$121</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="2">'逐位号_120项'!$1:$1</definedName>
@@ -484,7 +484,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>本次比较8e2722c；新图为通用电容编码说明，不是实购型号证明。原表料号按图解码为X7R/50V，与先前口头C0G有差异，4.7nF实际介质/耐压改记待核；设计与100nF库存保持。</t>
+          <t>本次比较dc43f34；用户确认实际型号就是CL21B472JBANNNC，确定为4.7nF/50V/0805/±5%/X7R；C7～C10按该款4只列料，C_VINP_ADC的C0G另列1只，设计不改。</t>
         </is>
       </c>
     </row>
@@ -592,7 +592,7 @@
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>472批次已确认4.7nF；随后用户确认另外买了100nF/0805，两批分开记录。100nF/50V/0805/X7R已购50只，单板需求16只，补购0只，装配一板后余34只；完整料号/容差未提供；4.7nF先前口头C0G与原表型号解码X7R有差异，实际完整型号待核；不从通用图的C0G选项推定实物介质，不把解码出的50V当成实物已确认。</t>
+          <t>472批次已确认4.7nF；随后用户确认另外买了100nF/0805，两批分开记录。100nF/50V/0805/X7R已购50只，单板需求16只，补购0只，装配一板后余34只；完整料号/容差未提供；用户现已确认实际型号CL21B472JBANNNC，先前口头C0G由实际型号纠正为X7R；该款50V/±5%/0805按用户编码图明确。C_VINP_ADC仍须另备C0G，是否另购及两类库存数量待核。</t>
         </is>
       </c>
     </row>
@@ -676,7 +676,7 @@
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>相对8e2722c，仅更新4.7nF证据复核状态；原理图和PCB原生文件未改，网络/脚号/设计参数与用量保持，4.7nF单板仍需5只，C_VINP_ADC仍要求C0G。</t>
+          <t>相对dc43f34，原理图和PCB原生文件未改，网络/脚号/设计参数与用量保持；4.7nF仍5只，其中C7～C10原图未指定介质，C_VINP_ADC明确C0G要求保留。</t>
         </is>
       </c>
     </row>
@@ -688,7 +688,7 @@
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>4.7nF实际型号/介质/耐压/数量待核，C0G仍是C_VINP_ADC的要求；若实物是原表X7R款，不直接代装该位置，是否补购待实际型号/库存核实。100nF库存50只/单板补购0保持；45采购行/120位号及全部PCB几何未改，本轮没有执行换料。</t>
+          <t>已确认X7R款列C7～C10共4只，C_VINP_ADC的4.7nF/50V/C0G/0805单列1只待备；C0G库存未核，补购数量不猜填。采购行45→46，逻辑位号仍120、默认有料仍104，PCB几何及100nF库存50只保持；无新增逻辑器件或改板要求。</t>
         </is>
       </c>
     </row>
@@ -718,7 +718,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:J46"/>
+  <dimension ref="A1:J47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -1612,7 +1612,7 @@
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>4.7nF/50V，C0G（统一采购建议）</t>
+          <t>CL21B472JBANNNC；4.7nF/50V，±5%，X7R</t>
         </is>
       </c>
       <c r="C21" s="2" t="inlineStr">
@@ -1622,14 +1622,14 @@
       </c>
       <c r="D21" s="2" t="inlineStr">
         <is>
-          <t>C7、C8、C9、C10、C_VINP_ADC</t>
+          <t>C7、C8、C9、C10</t>
         </is>
       </c>
       <c r="E21" s="2" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F21" s="2" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="G21" s="3" t="n"/>
       <c r="H21" s="2">
@@ -1638,12 +1638,12 @@
       </c>
       <c r="I21" s="2" t="inlineStr">
         <is>
-          <t>通用编码图未显示实购型号；介质/耐压待核</t>
+          <t>用户已确认完整型号；库存数量待核</t>
         </is>
       </c>
       <c r="J21" s="2" t="inlineStr">
         <is>
-          <t>用户先前称有C0G，随后提供通用编码图；不能据图中C=C0G确认所选实物。若实际仍为原表CL21B472JBANNNC，按图解码0805/4.7nF/±5%/50V/X7R，与口头C0G有差异。请核对实际完整型号；C_VINP_ADC要求C0G，不直接以X7R代装，其他位置也须按要求核对。单板共5只、库存数量未知</t>
+          <t>用户回复就是这个型号；按其编码图确认为0805/4.7nF/50V/±5%/X7R，单板4只，四个位号源图未指定C0G。不得用于C_VINP_ADC，不与C0G库存混计</t>
         </is>
       </c>
     </row>
@@ -1655,7 +1655,7 @@
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>1nF/50V，建议C0G/NP0</t>
+          <t>4.7nF/50V，C0G/NP0</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
@@ -1665,14 +1665,14 @@
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t>C_IL_ADC、C_IL_PROT</t>
+          <t>C_VINP_ADC</t>
         </is>
       </c>
       <c r="E22" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F22" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G22" s="3" t="n"/>
       <c r="H22" s="2">
@@ -1681,12 +1681,12 @@
       </c>
       <c r="I22" s="2" t="inlineStr">
         <is>
-          <t>核对已购物料</t>
+          <t>需单独备C0G；是否另购/库存待核</t>
         </is>
       </c>
       <c r="J22" s="2" t="inlineStr">
         <is>
-          <t>正常装配2只；C_IL_PROT明确C0G</t>
+          <t>单板1只；源图明确C0G，已确认的CL21B472JBANNNC为X7R，不能代装。无已确认C0G完整料号及数量，库存/补购数留空，不默认库存0或已购</t>
         </is>
       </c>
     </row>
@@ -1698,7 +1698,7 @@
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>1nF/100V，C0G/NP0，DNP</t>
+          <t>1nF/50V，建议C0G/NP0</t>
         </is>
       </c>
       <c r="C23" s="2" t="inlineStr">
@@ -1708,14 +1708,14 @@
       </c>
       <c r="D23" s="2" t="inlineStr">
         <is>
-          <t>C_SN</t>
+          <t>C_IL_ADC、C_IL_PROT</t>
         </is>
       </c>
       <c r="E23" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F23" s="2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G23" s="3" t="n"/>
       <c r="H23" s="2">
@@ -1724,24 +1724,24 @@
       </c>
       <c r="I23" s="2" t="inlineStr">
         <is>
-          <t>DNP，默认不装</t>
+          <t>核对已购物料</t>
         </is>
       </c>
       <c r="J23" s="2" t="inlineStr">
         <is>
-          <t>吸收电路预留，实测振铃后决定是否装配及调值</t>
+          <t>正常装配2只；C_IL_PROT明确C0G</t>
         </is>
       </c>
     </row>
     <row r="24" ht="58" customHeight="1">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>普通电阻</t>
+          <t>贴片电容</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>4.7Ω，建议1%、≥0.125W</t>
+          <t>1nF/100V，C0G/NP0，DNP</t>
         </is>
       </c>
       <c r="C24" s="2" t="inlineStr">
@@ -1751,14 +1751,14 @@
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>RG_H、RG_L</t>
+          <t>C_SN</t>
         </is>
       </c>
       <c r="E24" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F24" s="2" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G24" s="3" t="n"/>
       <c r="H24" s="2">
@@ -1767,12 +1767,12 @@
       </c>
       <c r="I24" s="2" t="inlineStr">
         <is>
-          <t>核对已购物料</t>
+          <t>DNP，默认不装</t>
         </is>
       </c>
       <c r="J24" s="2" t="inlineStr">
         <is>
-          <t>不要沿用Rev B中的旧栅极电阻值</t>
+          <t>吸收电路预留，实测振铃后决定是否装配及调值</t>
         </is>
       </c>
     </row>
@@ -1784,7 +1784,7 @@
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>1Ω，建议1%、≥0.125W</t>
+          <t>4.7Ω，建议1%、≥0.125W</t>
         </is>
       </c>
       <c r="C25" s="2" t="inlineStr">
@@ -1794,14 +1794,14 @@
       </c>
       <c r="D25" s="2" t="inlineStr">
         <is>
-          <t>R_VDDA</t>
+          <t>RG_H、RG_L</t>
         </is>
       </c>
       <c r="E25" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F25" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G25" s="3" t="n"/>
       <c r="H25" s="2">
@@ -1815,7 +1815,7 @@
       </c>
       <c r="J25" s="2" t="inlineStr">
         <is>
-          <t>模拟电源串联电阻，不能错装成0Ω</t>
+          <t>不要沿用Rev B中的旧栅极电阻值</t>
         </is>
       </c>
     </row>
@@ -1827,7 +1827,7 @@
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>100Ω，建议1%、≥0.125W</t>
+          <t>1Ω，建议1%、≥0.125W</t>
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr">
@@ -1837,7 +1837,7 @@
       </c>
       <c r="D26" s="2" t="inlineStr">
         <is>
-          <t>R_PWM</t>
+          <t>R_VDDA</t>
         </is>
       </c>
       <c r="E26" s="2" t="n">
@@ -1858,7 +1858,7 @@
       </c>
       <c r="J26" s="2" t="inlineStr">
         <is>
-          <t>与100Ω/0.1%精密电阻分开采购</t>
+          <t>模拟电源串联电阻，不能错装成0Ω</t>
         </is>
       </c>
     </row>
@@ -1870,7 +1870,7 @@
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>1kΩ，1%、≥0.125W（统一采购建议）</t>
+          <t>100Ω，建议1%、≥0.125W</t>
         </is>
       </c>
       <c r="C27" s="2" t="inlineStr">
@@ -1880,14 +1880,14 @@
       </c>
       <c r="D27" s="2" t="inlineStr">
         <is>
-          <t>R3、R6、R7、R8、R_IL_ADC、R_VINP_ADC、R_IL_PROT、R_IOUT_PROT</t>
+          <t>R_PWM</t>
         </is>
       </c>
       <c r="E27" s="2" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="F27" s="2" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="G27" s="3" t="n"/>
       <c r="H27" s="2">
@@ -1901,7 +1901,7 @@
       </c>
       <c r="J27" s="2" t="inlineStr">
         <is>
-          <t>共8只；两项保护电阻明确要求1%；原图其余未明确精度，建议统一1%</t>
+          <t>与100Ω/0.1%精密电阻分开采购</t>
         </is>
       </c>
     </row>
@@ -1913,7 +1913,7 @@
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>10kΩ，建议1%、≥0.125W</t>
+          <t>1kΩ，1%、≥0.125W（统一采购建议）</t>
         </is>
       </c>
       <c r="C28" s="2" t="inlineStr">
@@ -1923,14 +1923,14 @@
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t>R_GSH、R_GSL、R_IN_PD、R_SD_PD、R12、R13、R14、R_EN_PD、R_ARM_PD、R_IOUT_PU</t>
+          <t>R3、R6、R7、R8、R_IL_ADC、R_VINP_ADC、R_IL_PROT、R_IOUT_PROT</t>
         </is>
       </c>
       <c r="E28" s="2" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="F28" s="2" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="G28" s="3" t="n"/>
       <c r="H28" s="2">
@@ -1944,7 +1944,7 @@
       </c>
       <c r="J28" s="2" t="inlineStr">
         <is>
-          <t>普通10kΩ共10只；不替代0.1%分压/参考电阻</t>
+          <t>共8只；两项保护电阻明确要求1%；原图其余未明确精度，建议统一1%</t>
         </is>
       </c>
     </row>
@@ -1956,7 +1956,7 @@
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>23kΩ，建议1%、≥0.125W</t>
+          <t>10kΩ，建议1%、≥0.125W</t>
         </is>
       </c>
       <c r="C29" s="2" t="inlineStr">
@@ -1966,14 +1966,14 @@
       </c>
       <c r="D29" s="2" t="inlineStr">
         <is>
-          <t>R11</t>
+          <t>R_GSH、R_GSL、R_IN_PD、R_SD_PD、R12、R13、R14、R_EN_PD、R_ARM_PD、R_IOUT_PU</t>
         </is>
       </c>
       <c r="E29" s="2" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F29" s="2" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="G29" s="3" t="n"/>
       <c r="H29" s="2">
@@ -1987,19 +1987,19 @@
       </c>
       <c r="J29" s="2" t="inlineStr">
         <is>
-          <t>按23kΩ采购；不直接换成22kΩ</t>
+          <t>普通10kΩ共10只；不替代0.1%分压/参考电阻</t>
         </is>
       </c>
     </row>
     <row r="30" ht="58" customHeight="1">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>精密电阻</t>
+          <t>普通电阻</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>100kΩ，0.1%，≥0.125W</t>
+          <t>23kΩ，建议1%、≥0.125W</t>
         </is>
       </c>
       <c r="C30" s="2" t="inlineStr">
@@ -2009,14 +2009,14 @@
       </c>
       <c r="D30" s="2" t="inlineStr">
         <is>
-          <t>R1、R_VINP_TOP</t>
+          <t>R11</t>
         </is>
       </c>
       <c r="E30" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F30" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G30" s="3" t="n"/>
       <c r="H30" s="2">
@@ -2025,12 +2025,12 @@
       </c>
       <c r="I30" s="2" t="inlineStr">
         <is>
-          <t>精度/料号待核</t>
+          <t>核对已购物料</t>
         </is>
       </c>
       <c r="J30" s="2" t="inlineStr">
         <is>
-          <t>温漂未在源图固定；按实购物料记录，不虚构已确认参数</t>
+          <t>按23kΩ采购；不直接换成22kΩ</t>
         </is>
       </c>
     </row>
@@ -2042,7 +2042,7 @@
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>10kΩ，0.1%，≥0.125W</t>
+          <t>100kΩ，0.1%，≥0.125W</t>
         </is>
       </c>
       <c r="C31" s="2" t="inlineStr">
@@ -2052,14 +2052,14 @@
       </c>
       <c r="D31" s="2" t="inlineStr">
         <is>
-          <t>R2、R4、R9、R16、R_IOUT_BOT、R_VINP_BOT</t>
+          <t>R1、R_VINP_TOP</t>
         </is>
       </c>
       <c r="E31" s="2" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="F31" s="2" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="G31" s="3" t="n"/>
       <c r="H31" s="2">
@@ -2073,7 +2073,7 @@
       </c>
       <c r="J31" s="2" t="inlineStr">
         <is>
-          <t>共6只，与普通10kΩ区分</t>
+          <t>温漂未在源图固定；按实购物料记录，不虚构已确认参数</t>
         </is>
       </c>
     </row>
@@ -2085,7 +2085,7 @@
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>1kΩ，0.1%，≥0.125W</t>
+          <t>10kΩ，0.1%，≥0.125W</t>
         </is>
       </c>
       <c r="C32" s="2" t="inlineStr">
@@ -2095,14 +2095,14 @@
       </c>
       <c r="D32" s="2" t="inlineStr">
         <is>
-          <t>R5</t>
+          <t>R2、R4、R9、R16、R_IOUT_BOT、R_VINP_BOT</t>
         </is>
       </c>
       <c r="E32" s="2" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="F32" s="2" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="G32" s="3" t="n"/>
       <c r="H32" s="2">
@@ -2116,7 +2116,7 @@
       </c>
       <c r="J32" s="2" t="inlineStr">
         <is>
-          <t>与普通1kΩ区分</t>
+          <t>共6只，与普通10kΩ区分</t>
         </is>
       </c>
     </row>
@@ -2128,7 +2128,7 @@
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>49.9kΩ，0.1%，≥0.125W</t>
+          <t>1kΩ，0.1%，≥0.125W</t>
         </is>
       </c>
       <c r="C33" s="2" t="inlineStr">
@@ -2138,14 +2138,14 @@
       </c>
       <c r="D33" s="2" t="inlineStr">
         <is>
-          <t>R10A、R15A</t>
+          <t>R5</t>
         </is>
       </c>
       <c r="E33" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F33" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G33" s="3" t="n"/>
       <c r="H33" s="2">
@@ -2159,7 +2159,7 @@
       </c>
       <c r="J33" s="2" t="inlineStr">
         <is>
-          <t>保留49.9kΩ，不用近似值替代</t>
+          <t>与普通1kΩ区分</t>
         </is>
       </c>
     </row>
@@ -2171,7 +2171,7 @@
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>100Ω，0.1%，≥0.125W</t>
+          <t>49.9kΩ，0.1%，≥0.125W</t>
         </is>
       </c>
       <c r="C34" s="2" t="inlineStr">
@@ -2181,7 +2181,7 @@
       </c>
       <c r="D34" s="2" t="inlineStr">
         <is>
-          <t>R10B、R15B</t>
+          <t>R10A、R15A</t>
         </is>
       </c>
       <c r="E34" s="2" t="n">
@@ -2202,7 +2202,7 @@
       </c>
       <c r="J34" s="2" t="inlineStr">
         <is>
-          <t>共2只，与R_PWM分开</t>
+          <t>保留49.9kΩ，不用近似值替代</t>
         </is>
       </c>
     </row>
@@ -2214,7 +2214,7 @@
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t>20kΩ，0.1%，≥0.125W</t>
+          <t>100Ω，0.1%，≥0.125W</t>
         </is>
       </c>
       <c r="C35" s="2" t="inlineStr">
@@ -2224,14 +2224,14 @@
       </c>
       <c r="D35" s="2" t="inlineStr">
         <is>
-          <t>R_IOUT_TOP</t>
+          <t>R10B、R15B</t>
         </is>
       </c>
       <c r="E35" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F35" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G35" s="3" t="n"/>
       <c r="H35" s="2">
@@ -2245,29 +2245,29 @@
       </c>
       <c r="J35" s="2" t="inlineStr">
         <is>
-          <t>输出告警参考上臂</t>
+          <t>共2只，与R_PWM分开</t>
         </is>
       </c>
     </row>
     <row r="36" ht="58" customHeight="1">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>功率电阻</t>
+          <t>精密电阻</t>
         </is>
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>2.2kΩ，≥0.25W</t>
+          <t>20kΩ，0.1%，≥0.125W</t>
         </is>
       </c>
       <c r="C36" s="2" t="inlineStr">
         <is>
-          <t>1206</t>
+          <t>0805</t>
         </is>
       </c>
       <c r="D36" s="2" t="inlineStr">
         <is>
-          <t>R_BL</t>
+          <t>R_IOUT_TOP</t>
         </is>
       </c>
       <c r="E36" s="2" t="n">
@@ -2283,12 +2283,12 @@
       </c>
       <c r="I36" s="2" t="inlineStr">
         <is>
-          <t>功率/料号待核</t>
+          <t>精度/料号待核</t>
         </is>
       </c>
       <c r="J36" s="2" t="inlineStr">
         <is>
-          <t>确认实物额定功率，不能买成普通0805</t>
+          <t>输出告警参考上臂</t>
         </is>
       </c>
     </row>
@@ -2300,7 +2300,7 @@
       </c>
       <c r="B37" s="2" t="inlineStr">
         <is>
-          <t>10Ω，≥0.25W，DNP</t>
+          <t>2.2kΩ，≥0.25W</t>
         </is>
       </c>
       <c r="C37" s="2" t="inlineStr">
@@ -2310,14 +2310,14 @@
       </c>
       <c r="D37" s="2" t="inlineStr">
         <is>
-          <t>R_SN</t>
+          <t>R_BL</t>
         </is>
       </c>
       <c r="E37" s="2" t="n">
         <v>1</v>
       </c>
       <c r="F37" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G37" s="3" t="n"/>
       <c r="H37" s="2">
@@ -2326,41 +2326,41 @@
       </c>
       <c r="I37" s="2" t="inlineStr">
         <is>
-          <t>DNP，默认不装</t>
+          <t>功率/料号待核</t>
         </is>
       </c>
       <c r="J37" s="2" t="inlineStr">
         <is>
-          <t>与C_SN配套；由旧0805占位改1206</t>
+          <t>确认实物额定功率，不能买成普通0805</t>
         </is>
       </c>
     </row>
     <row r="38" ht="58" customHeight="1">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>二极管</t>
+          <t>功率电阻</t>
         </is>
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>SR560，目标60V/5A（用户选型）</t>
+          <t>10Ω，≥0.25W，DNP</t>
         </is>
       </c>
       <c r="C38" s="2" t="inlineStr">
         <is>
-          <t>SMB / DO-214AA，贴片</t>
+          <t>1206</t>
         </is>
       </c>
       <c r="D38" s="2" t="inlineStr">
         <is>
-          <t>D1、D_FREE</t>
+          <t>R_SN</t>
         </is>
       </c>
       <c r="E38" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F38" s="2" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G38" s="3" t="n"/>
       <c r="H38" s="2">
@@ -2369,12 +2369,12 @@
       </c>
       <c r="I38" s="2" t="inlineStr">
         <is>
-          <t>用户已确认SMB；厂家资料待最终复核</t>
+          <t>DNP，默认不装</t>
         </is>
       </c>
       <c r="J38" s="2" t="inlineStr">
         <is>
-          <t>共2只；1=K色条端、2=A。沿用原SMB焊盘；SR560为用户确认选型，原轴向目录不作为SMB厂家尺寸/电气手册；完整订货型号/额定条件/推荐焊盘待归档</t>
+          <t>与C_SN配套；由旧0805占位改1206</t>
         </is>
       </c>
     </row>
@@ -2386,24 +2386,24 @@
       </c>
       <c r="B39" s="2" t="inlineStr">
         <is>
-          <t>UF4007，快恢复</t>
+          <t>SR560，目标60V/5A（用户选型）</t>
         </is>
       </c>
       <c r="C39" s="2" t="inlineStr">
         <is>
-          <t>DO-41，成型P10.16待核</t>
+          <t>SMB / DO-214AA，贴片</t>
         </is>
       </c>
       <c r="D39" s="2" t="inlineStr">
         <is>
-          <t>D_BOOT</t>
+          <t>D1、D_FREE</t>
         </is>
       </c>
       <c r="E39" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F39" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G39" s="3" t="n"/>
       <c r="H39" s="2">
@@ -2412,12 +2412,12 @@
       </c>
       <c r="I39" s="2" t="inlineStr">
         <is>
-          <t>成型脚距待核</t>
+          <t>用户已确认SMB；厂家资料待最终复核</t>
         </is>
       </c>
       <c r="J39" s="2" t="inlineStr">
         <is>
-          <t>工程定义1=A、2=K；不是普通1N4007</t>
+          <t>共2只；1=K色条端、2=A。沿用原SMB焊盘；SR560为用户确认选型，原轴向目录不作为SMB厂家尺寸/电气手册；完整订货型号/额定条件/推荐焊盘待归档</t>
         </is>
       </c>
     </row>
@@ -2429,24 +2429,24 @@
       </c>
       <c r="B40" s="2" t="inlineStr">
         <is>
-          <t>BAT54S，串联双肖特基</t>
+          <t>UF4007，快恢复</t>
         </is>
       </c>
       <c r="C40" s="2" t="inlineStr">
         <is>
-          <t>SOT-23</t>
+          <t>DO-41，成型P10.16待核</t>
         </is>
       </c>
       <c r="D40" s="2" t="inlineStr">
         <is>
-          <t>D_ADC1、D_ADC2、D_ADC3、D_ADC4、D_ADC5、D_ADC6</t>
+          <t>D_BOOT</t>
         </is>
       </c>
       <c r="E40" s="2" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="F40" s="2" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="G40" s="3" t="n"/>
       <c r="H40" s="2">
@@ -2455,12 +2455,12 @@
       </c>
       <c r="I40" s="2" t="inlineStr">
         <is>
-          <t>核对已购物料</t>
+          <t>成型脚距待核</t>
         </is>
       </c>
       <c r="J40" s="2" t="inlineStr">
         <is>
-          <t>共6只；1=A1、2=K2、3=K1/A2；不能装BAT54/BAT54C</t>
+          <t>工程定义1=A、2=K；不是普通1N4007</t>
         </is>
       </c>
     </row>
@@ -2472,7 +2472,7 @@
       </c>
       <c r="B41" s="2" t="inlineStr">
         <is>
-          <t>BAT54，单肖特基</t>
+          <t>BAT54S，串联双肖特基</t>
         </is>
       </c>
       <c r="C41" s="2" t="inlineStr">
@@ -2482,14 +2482,14 @@
       </c>
       <c r="D41" s="2" t="inlineStr">
         <is>
-          <t>D_POR</t>
+          <t>D_ADC1、D_ADC2、D_ADC3、D_ADC4、D_ADC5、D_ADC6</t>
         </is>
       </c>
       <c r="E41" s="2" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="F41" s="2" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="G41" s="3" t="n"/>
       <c r="H41" s="2">
@@ -2503,29 +2503,29 @@
       </c>
       <c r="J41" s="2" t="inlineStr">
         <is>
-          <t>1=A、3=K、2=NC；不能与BAT54S混装</t>
+          <t>共6只；1=A1、2=K2、3=K1/A2；不能装BAT54/BAT54C</t>
         </is>
       </c>
     </row>
     <row r="42" ht="58" customHeight="1">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>保险</t>
+          <t>二极管</t>
         </is>
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t>2A快断保险管，5×20mm，商品标250V</t>
+          <t>BAT54，单肖特基</t>
         </is>
       </c>
       <c r="C42" s="2" t="inlineStr">
         <is>
-          <t>配5×20mm管夹</t>
+          <t>SOT-23</t>
         </is>
       </c>
       <c r="D42" s="2" t="inlineStr">
         <is>
-          <t>F1</t>
+          <t>D_POR</t>
         </is>
       </c>
       <c r="E42" s="2" t="n">
@@ -2541,41 +2541,41 @@
       </c>
       <c r="I42" s="2" t="inlineStr">
         <is>
-          <t>尺寸/快断已给资料；实际电气性能待核</t>
+          <t>核对已购物料</t>
         </is>
       </c>
       <c r="J42" s="2" t="inlineStr">
         <is>
-          <t>商品BXG16519；250V未注明AC/DC分断条件，启动不误熔断与故障分断待验证；管夹另列2只</t>
+          <t>1=A、3=K、2=NC；不能与BAT54S混装</t>
         </is>
       </c>
     </row>
     <row r="43" ht="58" customHeight="1">
       <c r="A43" s="2" t="inlineStr">
         <is>
-          <t>连接器</t>
+          <t>保险</t>
         </is>
       </c>
       <c r="B43" s="2" t="inlineStr">
         <is>
-          <t>2P接线端子，P2.54，≥3A</t>
+          <t>2A快断保险管，5×20mm，商品标250V</t>
         </is>
       </c>
       <c r="C43" s="2" t="inlineStr">
         <is>
-          <t>图示5.48×6.30×8.80mm；孔1.30</t>
+          <t>配5×20mm管夹</t>
         </is>
       </c>
       <c r="D43" s="2" t="inlineStr">
         <is>
-          <t>J1、J2、J_BYP、J_MON</t>
+          <t>F1</t>
         </is>
       </c>
       <c r="E43" s="2" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="F43" s="2" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="G43" s="3" t="n"/>
       <c r="H43" s="2">
@@ -2584,12 +2584,12 @@
       </c>
       <c r="I43" s="2" t="inlineStr">
         <is>
-          <t>完整型号/朝向待核</t>
+          <t>尺寸/快断已给资料；实际电气性能待核</t>
         </is>
       </c>
       <c r="J43" s="2" t="inlineStr">
         <is>
-          <t>共4只；照片标称6A/150V；J_BYP是接口，不包含外接开关</t>
+          <t>商品BXG16519；250V未注明AC/DC分断条件，启动不误熔断与故障分断待验证；管夹另列2只</t>
         </is>
       </c>
     </row>
@@ -2601,24 +2601,24 @@
       </c>
       <c r="B44" s="2" t="inlineStr">
         <is>
-          <t>1×4直排针，P2.54</t>
+          <t>2P接线端子，P2.54，≥3A</t>
         </is>
       </c>
       <c r="C44" s="2" t="inlineStr">
         <is>
-          <t>直插，针长/塑高待核</t>
+          <t>图示5.48×6.30×8.80mm；孔1.30</t>
         </is>
       </c>
       <c r="D44" s="2" t="inlineStr">
         <is>
-          <t>J_AUX12、J_AUX5</t>
+          <t>J1、J2、J_BYP、J_MON</t>
         </is>
       </c>
       <c r="E44" s="2" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="F44" s="2" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="G44" s="3" t="n"/>
       <c r="H44" s="2">
@@ -2627,12 +2627,12 @@
       </c>
       <c r="I44" s="2" t="inlineStr">
         <is>
-          <t>配对件待核</t>
+          <t>完整型号/朝向待核</t>
         </is>
       </c>
       <c r="J44" s="2" t="inlineStr">
         <is>
-          <t>共2只；与LM2596HV通过排线相接，不直接按四角焊盘插装</t>
+          <t>共4只；照片标称6A/150V；J_BYP是接口，不包含外接开关</t>
         </is>
       </c>
     </row>
@@ -2644,24 +2644,24 @@
       </c>
       <c r="B45" s="2" t="inlineStr">
         <is>
-          <t>2×8排针，P2.54</t>
+          <t>1×4直排针，P2.54</t>
         </is>
       </c>
       <c r="C45" s="2" t="inlineStr">
         <is>
-          <t>直插；配对高度待核</t>
+          <t>直插，针长/塑高待核</t>
         </is>
       </c>
       <c r="D45" s="2" t="inlineStr">
         <is>
-          <t>J_CTL</t>
+          <t>J_AUX12、J_AUX5</t>
         </is>
       </c>
       <c r="E45" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F45" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G45" s="3" t="n"/>
       <c r="H45" s="2">
@@ -2675,36 +2675,36 @@
       </c>
       <c r="J45" s="2" t="inlineStr">
         <is>
-          <t>1只，16针；PA6监测走独立J_MON，不占此16针</t>
+          <t>共2只；与LM2596HV通过排线相接，不直接按四角焊盘插装</t>
         </is>
       </c>
     </row>
     <row r="46" ht="58" customHeight="1">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>测试点</t>
+          <t>连接器</t>
         </is>
       </c>
       <c r="B46" s="2" t="inlineStr">
         <is>
-          <t>裸铜测试焊盘，直径1.5mm</t>
+          <t>2×8排针，P2.54</t>
         </is>
       </c>
       <c r="C46" s="2" t="inlineStr">
         <is>
-          <t>PCB焊盘；默认不买测试柱</t>
+          <t>直插；配对高度待核</t>
         </is>
       </c>
       <c r="D46" s="2" t="inlineStr">
         <is>
-          <t>TP1、TP2、TP3、TP4、TP5、TP6、TP7、TP8、TP9、TP10、TP11、TP12、TP13、TP14</t>
+          <t>J_CTL</t>
         </is>
       </c>
       <c r="E46" s="2" t="n">
-        <v>14</v>
+        <v>1</v>
       </c>
       <c r="F46" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G46" s="3" t="n"/>
       <c r="H46" s="2">
@@ -2713,19 +2713,62 @@
       </c>
       <c r="I46" s="2" t="inlineStr">
         <is>
+          <t>配对件待核</t>
+        </is>
+      </c>
+      <c r="J46" s="2" t="inlineStr">
+        <is>
+          <t>1只，16针；PA6监测走独立J_MON，不占此16针</t>
+        </is>
+      </c>
+    </row>
+    <row r="47" ht="58" customHeight="1">
+      <c r="A47" s="2" t="inlineStr">
+        <is>
+          <t>测试点</t>
+        </is>
+      </c>
+      <c r="B47" s="2" t="inlineStr">
+        <is>
+          <t>裸铜测试焊盘，直径1.5mm</t>
+        </is>
+      </c>
+      <c r="C47" s="2" t="inlineStr">
+        <is>
+          <t>PCB焊盘；默认不买测试柱</t>
+        </is>
+      </c>
+      <c r="D47" s="2" t="inlineStr">
+        <is>
+          <t>TP1、TP2、TP3、TP4、TP5、TP6、TP7、TP8、TP9、TP10、TP11、TP12、TP13、TP14</t>
+        </is>
+      </c>
+      <c r="E47" s="2" t="n">
+        <v>14</v>
+      </c>
+      <c r="F47" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G47" s="3" t="n"/>
+      <c r="H47" s="2">
+        <f>IF(G47="","",MAX(F47-G47,0))</f>
+        <v/>
+      </c>
+      <c r="I47" s="2" t="inlineStr">
+        <is>
           <t>默认无需采购</t>
         </is>
       </c>
-      <c r="J46" s="2" t="inlineStr">
+      <c r="J47" s="2" t="inlineStr">
         <is>
           <t>14个设计测试点，实物采购数量为0；若改测试柱需同步封装</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:J46"/>
+  <autoFilter ref="A1:J47"/>
   <dataValidations count="1">
-    <dataValidation sqref="G2:G46" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="请输入非负整数" error="库存数量应为0或正整数" type="whole" operator="greaterThanOrEqual">
+    <dataValidation sqref="G2:G47" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="请输入非负整数" error="库存数量应为0或正整数" type="whole" operator="greaterThanOrEqual">
       <formula1>0</formula1>
     </dataValidation>
   </dataValidations>
@@ -4714,7 +4757,7 @@
       </c>
       <c r="D43" s="2" t="inlineStr">
         <is>
-          <t>4.7nF/50V，C0G（统一采购建议）</t>
+          <t>CL21B472JBANNNC；4.7nF/50V，±5%，X7R</t>
         </is>
       </c>
       <c r="E43" s="2" t="inlineStr">
@@ -4730,12 +4773,12 @@
       </c>
       <c r="H43" s="2" t="inlineStr">
         <is>
-          <t>通用编码图未显示实购型号；介质/耐压待核</t>
+          <t>用户已确认完整型号；库存数量待核</t>
         </is>
       </c>
       <c r="I43" s="2" t="inlineStr">
         <is>
-          <t>用户先前称有C0G，随后提供通用编码图；不能据图中C=C0G确认所选实物。若实际仍为原表CL21B472JBANNNC，按图解码0805/4.7nF/±5%/50V/X7R，与口头C0G有差异。请核对实际完整型号；C_VINP_ADC要求C0G，不直接以X7R代装，其他位置也须按要求核对。单板共5只、库存数量未知</t>
+          <t>用户回复就是这个型号；按其编码图确认为0805/4.7nF/50V/±5%/X7R，单板4只，四个位号源图未指定C0G。不得用于C_VINP_ADC，不与C0G库存混计</t>
         </is>
       </c>
       <c r="J43" s="2" t="inlineStr"/>
@@ -4758,7 +4801,7 @@
       </c>
       <c r="D44" s="2" t="inlineStr">
         <is>
-          <t>4.7nF/50V，C0G（统一采购建议）</t>
+          <t>CL21B472JBANNNC；4.7nF/50V，±5%，X7R</t>
         </is>
       </c>
       <c r="E44" s="2" t="inlineStr">
@@ -4774,12 +4817,12 @@
       </c>
       <c r="H44" s="2" t="inlineStr">
         <is>
-          <t>通用编码图未显示实购型号；介质/耐压待核</t>
+          <t>用户已确认完整型号；库存数量待核</t>
         </is>
       </c>
       <c r="I44" s="2" t="inlineStr">
         <is>
-          <t>用户先前称有C0G，随后提供通用编码图；不能据图中C=C0G确认所选实物。若实际仍为原表CL21B472JBANNNC，按图解码0805/4.7nF/±5%/50V/X7R，与口头C0G有差异。请核对实际完整型号；C_VINP_ADC要求C0G，不直接以X7R代装，其他位置也须按要求核对。单板共5只、库存数量未知</t>
+          <t>用户回复就是这个型号；按其编码图确认为0805/4.7nF/50V/±5%/X7R，单板4只，四个位号源图未指定C0G。不得用于C_VINP_ADC，不与C0G库存混计</t>
         </is>
       </c>
       <c r="J44" s="2" t="inlineStr"/>
@@ -4802,7 +4845,7 @@
       </c>
       <c r="D45" s="2" t="inlineStr">
         <is>
-          <t>4.7nF/50V，C0G（统一采购建议）</t>
+          <t>CL21B472JBANNNC；4.7nF/50V，±5%，X7R</t>
         </is>
       </c>
       <c r="E45" s="2" t="inlineStr">
@@ -4818,12 +4861,12 @@
       </c>
       <c r="H45" s="2" t="inlineStr">
         <is>
-          <t>通用编码图未显示实购型号；介质/耐压待核</t>
+          <t>用户已确认完整型号；库存数量待核</t>
         </is>
       </c>
       <c r="I45" s="2" t="inlineStr">
         <is>
-          <t>用户先前称有C0G，随后提供通用编码图；不能据图中C=C0G确认所选实物。若实际仍为原表CL21B472JBANNNC，按图解码0805/4.7nF/±5%/50V/X7R，与口头C0G有差异。请核对实际完整型号；C_VINP_ADC要求C0G，不直接以X7R代装，其他位置也须按要求核对。单板共5只、库存数量未知</t>
+          <t>用户回复就是这个型号；按其编码图确认为0805/4.7nF/50V/±5%/X7R，单板4只，四个位号源图未指定C0G。不得用于C_VINP_ADC，不与C0G库存混计</t>
         </is>
       </c>
       <c r="J45" s="2" t="inlineStr"/>
@@ -4846,7 +4889,7 @@
       </c>
       <c r="D46" s="2" t="inlineStr">
         <is>
-          <t>4.7nF/50V，C0G（统一采购建议）</t>
+          <t>CL21B472JBANNNC；4.7nF/50V，±5%，X7R</t>
         </is>
       </c>
       <c r="E46" s="2" t="inlineStr">
@@ -4862,12 +4905,12 @@
       </c>
       <c r="H46" s="2" t="inlineStr">
         <is>
-          <t>通用编码图未显示实购型号；介质/耐压待核</t>
+          <t>用户已确认完整型号；库存数量待核</t>
         </is>
       </c>
       <c r="I46" s="2" t="inlineStr">
         <is>
-          <t>用户先前称有C0G，随后提供通用编码图；不能据图中C=C0G确认所选实物。若实际仍为原表CL21B472JBANNNC，按图解码0805/4.7nF/±5%/50V/X7R，与口头C0G有差异。请核对实际完整型号；C_VINP_ADC要求C0G，不直接以X7R代装，其他位置也须按要求核对。单板共5只、库存数量未知</t>
+          <t>用户回复就是这个型号；按其编码图确认为0805/4.7nF/50V/±5%/X7R，单板4只，四个位号源图未指定C0G。不得用于C_VINP_ADC，不与C0G库存混计</t>
         </is>
       </c>
       <c r="J46" s="2" t="inlineStr"/>
@@ -4890,7 +4933,7 @@
       </c>
       <c r="D47" s="2" t="inlineStr">
         <is>
-          <t>4.7nF/50V，C0G（统一采购建议）</t>
+          <t>4.7nF/50V，C0G/NP0</t>
         </is>
       </c>
       <c r="E47" s="2" t="inlineStr">
@@ -4906,12 +4949,12 @@
       </c>
       <c r="H47" s="2" t="inlineStr">
         <is>
-          <t>通用编码图未显示实购型号；介质/耐压待核</t>
+          <t>需单独备C0G；是否另购/库存待核</t>
         </is>
       </c>
       <c r="I47" s="2" t="inlineStr">
         <is>
-          <t>用户先前称有C0G，随后提供通用编码图；不能据图中C=C0G确认所选实物。若实际仍为原表CL21B472JBANNNC，按图解码0805/4.7nF/±5%/50V/X7R，与口头C0G有差异。请核对实际完整型号；C_VINP_ADC要求C0G，不直接以X7R代装，其他位置也须按要求核对。单板共5只、库存数量未知</t>
+          <t>单板1只；源图明确C0G，已确认的CL21B472JBANNNC为X7R，不能代装。无已确认C0G完整料号及数量，库存/补购数留空，不默认库存0或已购</t>
         </is>
       </c>
       <c r="J47" s="2" t="inlineStr">
@@ -8960,17 +9003,17 @@
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>口头C0G；原表CL21B472JBANNNC按新图解码X7R/50V</t>
+          <t>实际型号已确认CL21B472JBANNNC，纠正口头C0G为X7R</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>C7/C8/C9/C10/C_VINP_ADC共5只</t>
+          <t>C7/C8/C9/C10用X7R共4只；C_VINP_ADC另用C0G 1只</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>实际完整型号待核；通用图不证明所选款，C_VINP_ADC仍需C0G，不能据本次图直接认定实物合格</t>
+          <t>已拆分采购行；C0G完整料号/是否另购及库存待核，不把X7R代装C_VINP_ADC</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Record separate C0G capacitor purchase for VIN ADC
</commit_message>
<xml_diff>
--- a/projects/2026-electronics-contest/g-buck/rev-c2/downloads/GBUCK_RevC2_updated_BOM.xlsx
+++ b/projects/2026-electronics-contest/g-buck/rev-c2/downloads/GBUCK_RevC2_updated_BOM.xlsx
@@ -484,7 +484,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>本次比较dc43f34；用户确认实际型号就是CL21B472JBANNNC，确定为4.7nF/50V/0805/±5%/X7R；C7～C10按该款4只列料，C_VINP_ADC的C0G另列1只，设计不改。</t>
+          <t>本次比较0473d32；用户确认另购4.7nF/50V/C0G（NP0）/0805，用于C_VINP_ADC，每板1只；数量/完整料号/容差待核，与X7R款分开登记，设计不改。</t>
         </is>
       </c>
     </row>
@@ -592,7 +592,7 @@
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>472批次已确认4.7nF；随后用户确认另外买了100nF/0805，两批分开记录。100nF/50V/0805/X7R已购50只，单板需求16只，补购0只，装配一板后余34只；完整料号/容差未提供；用户现已确认实际型号CL21B472JBANNNC，先前口头C0G由实际型号纠正为X7R；该款50V/±5%/0805按用户编码图明确。C_VINP_ADC仍须另备C0G，是否另购及两类库存数量待核。</t>
+          <t>472批次已确认4.7nF；随后用户确认另外买了100nF/0805，两批分开记录。100nF/50V/0805/X7R已购50只，单板需求16只，补购0只，装配一板后余34只；完整料号/容差未提供；用户现已确认实际型号CL21B472JBANNNC，先前口头C0G由实际型号纠正为X7R；该款50V/±5%/0805按用户编码图明确。C_VINP_ADC所需的4.7nF/50V/C0G/0805另购状态已获确认；该批数量/完整料号/容差及X7R库存数量待核，两类不混计。</t>
         </is>
       </c>
     </row>
@@ -676,7 +676,7 @@
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>相对dc43f34，原理图和PCB原生文件未改，网络/脚号/设计参数与用量保持；4.7nF仍5只，其中C7～C10原图未指定介质，C_VINP_ADC明确C0G要求保留。</t>
+          <t>相对0473d32，仅补记C_VINP_ADC所需C0G款已另外购买；原理图和PCB原生文件未改，网络/脚号/设计参数与用量保持，4.7nF仍4只X7R加1只C0G。</t>
         </is>
       </c>
     </row>
@@ -688,7 +688,7 @@
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>已确认X7R款列C7～C10共4只，C_VINP_ADC的4.7nF/50V/C0G/0805单列1只待备；C0G库存未核，补购数量不猜填。采购行45→46，逻辑位号仍120、默认有料仍104，PCB几何及100nF库存50只保持；无新增逻辑器件或改板要求。</t>
+          <t>C_VINP_ADC的4.7nF/50V/C0G/0805由待备改为用户确认另购；数量/完整料号/容差待核，库存与补购数不猜填。采购行仍46、逻辑位号120、默认有料104，PCB几何及100nF库存50只保持；无新增器件或改板要求。</t>
         </is>
       </c>
     </row>
@@ -1681,12 +1681,12 @@
       </c>
       <c r="I22" s="2" t="inlineStr">
         <is>
-          <t>需单独备C0G；是否另购/库存待核</t>
+          <t>用户已确认另购4.7nF/50V/C0G/0805；数量待核</t>
         </is>
       </c>
       <c r="J22" s="2" t="inlineStr">
         <is>
-          <t>单板1只；源图明确C0G，已确认的CL21B472JBANNNC为X7R，不能代装。无已确认C0G完整料号及数量，库存/补购数留空，不默认库存0或已购</t>
+          <t>用户对是否另购此规格回复是的；单板1只，与C7～C10的CL21B472JBANNNC/X7R分开登记。实际数量/完整料号/容差未提供，库存与补购数仍留空，不自动填1只或视作缺货</t>
         </is>
       </c>
     </row>
@@ -4949,12 +4949,12 @@
       </c>
       <c r="H47" s="2" t="inlineStr">
         <is>
-          <t>需单独备C0G；是否另购/库存待核</t>
+          <t>用户已确认另购4.7nF/50V/C0G/0805；数量待核</t>
         </is>
       </c>
       <c r="I47" s="2" t="inlineStr">
         <is>
-          <t>单板1只；源图明确C0G，已确认的CL21B472JBANNNC为X7R，不能代装。无已确认C0G完整料号及数量，库存/补购数留空，不默认库存0或已购</t>
+          <t>用户对是否另购此规格回复是的；单板1只，与C7～C10的CL21B472JBANNNC/X7R分开登记。实际数量/完整料号/容差未提供，库存与补购数仍留空，不自动填1只或视作缺货</t>
         </is>
       </c>
       <c r="J47" s="2" t="inlineStr">
@@ -9003,17 +9003,17 @@
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>实际型号已确认CL21B472JBANNNC，纠正口头C0G为X7R</t>
+          <t>C7～C10实购CL21B472JBANNNC/X7R；现另购C0G款也获确认</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>C7/C8/C9/C10用X7R共4只；C_VINP_ADC另用C0G 1只</t>
+          <t>C7/C8/C9/C10用X7R共4只；C_VINP_ADC用C0G 1只</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>已拆分采购行；C0G完整料号/是否另购及库存待核，不把X7R代装C_VINP_ADC</t>
+          <t>两类分开登记；C0G数量/完整料号/容差待核，不把X7R代装C_VINP_ADC</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Record two C0G capacitors and zero single-board shortfall
</commit_message>
<xml_diff>
--- a/projects/2026-electronics-contest/g-buck/rev-c2/downloads/GBUCK_RevC2_updated_BOM.xlsx
+++ b/projects/2026-electronics-contest/g-buck/rev-c2/downloads/GBUCK_RevC2_updated_BOM.xlsx
@@ -484,7 +484,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>本次比较0473d32；用户确认另购4.7nF/50V/C0G（NP0）/0805，用于C_VINP_ADC，每板1只；数量/完整料号/容差待核，与X7R款分开登记，设计不改。</t>
+          <t>本次比较afd277e；用户确认另购C0G批次有2只，单板1只、补购0只、装一板后余1只。仅更新库存和补购记录；X7R批次数量仍待核，设计不改。</t>
         </is>
       </c>
     </row>
@@ -520,7 +520,7 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>采购汇总G列填写现有可用数量，H列自动计算需补购数量；100nF/X7R已按用户50只填G列，单板补购0只。其他空白表示库存未核，不代表未购买。</t>
+          <t>采购汇总G列填写现有可用数量，H列自动计算需补购数量；100nF/X7R已填50只，4.7nF/C0G已填2只，两项单板补购均0只。其他空白表示库存未核，不代表未购买。</t>
         </is>
       </c>
     </row>
@@ -592,7 +592,7 @@
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>472批次已确认4.7nF；随后用户确认另外买了100nF/0805，两批分开记录。100nF/50V/0805/X7R已购50只，单板需求16只，补购0只，装配一板后余34只；完整料号/容差未提供；用户现已确认实际型号CL21B472JBANNNC，先前口头C0G由实际型号纠正为X7R；该款50V/±5%/0805按用户编码图明确。C_VINP_ADC所需的4.7nF/50V/C0G/0805另购状态已获确认；该批数量/完整料号/容差及X7R库存数量待核，两类不混计。</t>
+          <t>472批次已确认4.7nF；随后用户确认另外买了100nF/0805，两批分开记录。100nF/50V/0805/X7R已购50只，单板需求16只，补购0只，装配一板后余34只；完整料号/容差未提供；用户现已确认实际型号CL21B472JBANNNC，先前口头C0G由实际型号纠正为X7R；该款50V/±5%/0805按用户编码图明确。C_VINP_ADC所需的4.7nF/50V/C0G/0805另购状态已获确认；该批C0G库存2只、单板用1只/补购0只；完整料号/容差及X7R库存数量待核，两类不混计。</t>
         </is>
       </c>
     </row>
@@ -676,7 +676,7 @@
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>相对0473d32，仅补记C_VINP_ADC所需C0G款已另外购买；原理图和PCB原生文件未改，网络/脚号/设计参数与用量保持，4.7nF仍4只X7R加1只C0G。</t>
+          <t>相对afd277e，仅登记C_VINP_ADC所需C0G库存2只；原理图和PCB原生文件未改，网络/脚号/设计参数与单板用量保持，4.7nF仍4只X7R加1只C0G。</t>
         </is>
       </c>
     </row>
@@ -688,7 +688,7 @@
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>C_VINP_ADC的4.7nF/50V/C0G/0805由待备改为用户确认另购；数量/完整料号/容差待核，库存与补购数不猜填。采购行仍46、逻辑位号120、默认有料104，PCB几何及100nF库存50只保持；无新增器件或改板要求。</t>
+          <t>C_VINP_ADC的C0G款已购2只，单板用1只，补购0只，预计装一板余1只；Excel保留补购公式，CSV写当前2/0，未实际扣减库存。完整料号/容差待核；46采购行/120位号/104默认有料、PCB几何及100nF库存50只保持，无新增或改板要求。</t>
         </is>
       </c>
     </row>
@@ -1674,19 +1674,21 @@
       <c r="F22" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="G22" s="3" t="n"/>
+      <c r="G22" s="3" t="n">
+        <v>2</v>
+      </c>
       <c r="H22" s="2">
         <f>IF(G22="","",MAX(F22-G22,0))</f>
         <v/>
       </c>
       <c r="I22" s="2" t="inlineStr">
         <is>
-          <t>用户已确认另购4.7nF/50V/C0G/0805；数量待核</t>
+          <t>4.7nF/50V/C0G/0805，已购2只</t>
         </is>
       </c>
       <c r="J22" s="2" t="inlineStr">
         <is>
-          <t>用户对是否另购此规格回复是的；单板1只，与C7～C10的CL21B472JBANNNC/X7R分开登记。实际数量/完整料号/容差未提供，库存与补购数仍留空，不自动填1只或视作缺货</t>
+          <t>用户对C0G批次数量回复2；单板1只，补购0只，装配一板后余1只。与C7～C10的CL21B472JBANNNC/X7R库存分开；完整料号/容差未提供</t>
         </is>
       </c>
     </row>
@@ -4949,12 +4951,12 @@
       </c>
       <c r="H47" s="2" t="inlineStr">
         <is>
-          <t>用户已确认另购4.7nF/50V/C0G/0805；数量待核</t>
+          <t>4.7nF/50V/C0G/0805，已购2只</t>
         </is>
       </c>
       <c r="I47" s="2" t="inlineStr">
         <is>
-          <t>用户对是否另购此规格回复是的；单板1只，与C7～C10的CL21B472JBANNNC/X7R分开登记。实际数量/完整料号/容差未提供，库存与补购数仍留空，不自动填1只或视作缺货</t>
+          <t>用户对C0G批次数量回复2；单板1只，补购0只，装配一板后余1只。与C7～C10的CL21B472JBANNNC/X7R库存分开；完整料号/容差未提供</t>
         </is>
       </c>
       <c r="J47" s="2" t="inlineStr">
@@ -9013,7 +9015,7 @@
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>两类分开登记；C0G数量/完整料号/容差待核，不把X7R代装C_VINP_ADC</t>
+          <t>C0G库存2只，单板需1只/补购0只；X7R库存数量及C0G完整料号/容差待核，两类不混装</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Record 50 X7R 4.7nF capacitors and single-board inventory balance
</commit_message>
<xml_diff>
--- a/projects/2026-electronics-contest/g-buck/rev-c2/downloads/GBUCK_RevC2_updated_BOM.xlsx
+++ b/projects/2026-electronics-contest/g-buck/rev-c2/downloads/GBUCK_RevC2_updated_BOM.xlsx
@@ -484,7 +484,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>本次比较afd277e；用户确认另购C0G批次有2只，单板1只、补购0只、装一板后余1只。仅更新库存和补购记录；X7R批次数量仍待核，设计不改。</t>
+          <t>本次比较238203e；用户确认CL21B472JBANNNC/X7R这批有50只，单板4只、补购0只、装一板后余46只；C0G库存2只和100nF库存50只保持，仅更新库存，设计不改。</t>
         </is>
       </c>
     </row>
@@ -520,7 +520,7 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>采购汇总G列填写现有可用数量，H列自动计算需补购数量；100nF/X7R已填50只，4.7nF/C0G已填2只，两项单板补购均0只。其他空白表示库存未核，不代表未购买。</t>
+          <t>采购汇总G列填写现有可用数量，H列自动计算需补购数量；100nF/X7R已填50只、4.7nF/X7R已填50只、4.7nF/C0G已填2只，三项单板补购均0只。其他空白表示库存未核，不代表未购买。</t>
         </is>
       </c>
     </row>
@@ -592,7 +592,7 @@
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>472批次已确认4.7nF；随后用户确认另外买了100nF/0805，两批分开记录。100nF/50V/0805/X7R已购50只，单板需求16只，补购0只，装配一板后余34只；完整料号/容差未提供；用户现已确认实际型号CL21B472JBANNNC，先前口头C0G由实际型号纠正为X7R；该款50V/±5%/0805按用户编码图明确。C_VINP_ADC所需的4.7nF/50V/C0G/0805另购状态已获确认；该批C0G库存2只、单板用1只/补购0只；完整料号/容差及X7R库存数量待核，两类不混计。</t>
+          <t>472批次已确认4.7nF；随后用户确认另外买了100nF/0805，两批分开记录。100nF/50V/0805/X7R已购50只，单板需求16只，补购0只，装配一板后余34只；完整料号/容差未提供；用户现已确认实际型号CL21B472JBANNNC，先前口头C0G由实际型号纠正为X7R；该款50V/±5%/0805按用户编码图明确。C_VINP_ADC所需的4.7nF/50V/C0G/0805另购状态已获确认；该批C0G库存2只、单板用1只/补购0只；C0G完整料号/容差待归档；CL21B472JBANNNC/X7R库存现已确认50只、单板用4只/补购0只，两类不混计。</t>
         </is>
       </c>
     </row>
@@ -676,7 +676,7 @@
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>相对afd277e，仅登记C_VINP_ADC所需C0G库存2只；原理图和PCB原生文件未改，网络/脚号/设计参数与单板用量保持，4.7nF仍4只X7R加1只C0G。</t>
+          <t>相对238203e，仅登记C7～C10所用CL21B472JBANNNC/X7R库存50只；原理图和PCB原生文件未改，网络/脚号/设计参数与单板用量保持，4.7nF仍4只X7R加1只C0G。</t>
         </is>
       </c>
     </row>
@@ -688,7 +688,7 @@
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>C_VINP_ADC的C0G款已购2只，单板用1只，补购0只，预计装一板余1只；Excel保留补购公式，CSV写当前2/0，未实际扣减库存。完整料号/容差待核；46采购行/120位号/104默认有料、PCB几何及100nF库存50只保持，无新增或改板要求。</t>
+          <t>C7～C10的X7R款已购50只，单板用4只，补购0只，预计装一板余46只；Excel保留公式，CSV写当前50/0，未实际扣减库存。C0G库存2只、100nF库存50只、46采购行/120位号/104默认有料及PCB几何保持，无新增或改板要求。</t>
         </is>
       </c>
     </row>
@@ -1631,19 +1631,21 @@
       <c r="F21" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="G21" s="3" t="n"/>
+      <c r="G21" s="3" t="n">
+        <v>50</v>
+      </c>
       <c r="H21" s="2">
         <f>IF(G21="","",MAX(F21-G21,0))</f>
         <v/>
       </c>
       <c r="I21" s="2" t="inlineStr">
         <is>
-          <t>用户已确认完整型号；库存数量待核</t>
+          <t>CL21B472JBANNNC，已购50只</t>
         </is>
       </c>
       <c r="J21" s="2" t="inlineStr">
         <is>
-          <t>用户回复就是这个型号；按其编码图确认为0805/4.7nF/50V/±5%/X7R，单板4只，四个位号源图未指定C0G。不得用于C_VINP_ADC，不与C0G库存混计</t>
+          <t>用户对这批X7R数量回复50；0805/4.7nF/50V/±5%/X7R，单板4只，补购0只，装一板后余46只。不得用于C_VINP_ADC；与另购C0G库存2只分开</t>
         </is>
       </c>
     </row>
@@ -4775,12 +4777,12 @@
       </c>
       <c r="H43" s="2" t="inlineStr">
         <is>
-          <t>用户已确认完整型号；库存数量待核</t>
+          <t>CL21B472JBANNNC，已购50只</t>
         </is>
       </c>
       <c r="I43" s="2" t="inlineStr">
         <is>
-          <t>用户回复就是这个型号；按其编码图确认为0805/4.7nF/50V/±5%/X7R，单板4只，四个位号源图未指定C0G。不得用于C_VINP_ADC，不与C0G库存混计</t>
+          <t>用户对这批X7R数量回复50；0805/4.7nF/50V/±5%/X7R，单板4只，补购0只，装一板后余46只。不得用于C_VINP_ADC；与另购C0G库存2只分开</t>
         </is>
       </c>
       <c r="J43" s="2" t="inlineStr"/>
@@ -4819,12 +4821,12 @@
       </c>
       <c r="H44" s="2" t="inlineStr">
         <is>
-          <t>用户已确认完整型号；库存数量待核</t>
+          <t>CL21B472JBANNNC，已购50只</t>
         </is>
       </c>
       <c r="I44" s="2" t="inlineStr">
         <is>
-          <t>用户回复就是这个型号；按其编码图确认为0805/4.7nF/50V/±5%/X7R，单板4只，四个位号源图未指定C0G。不得用于C_VINP_ADC，不与C0G库存混计</t>
+          <t>用户对这批X7R数量回复50；0805/4.7nF/50V/±5%/X7R，单板4只，补购0只，装一板后余46只。不得用于C_VINP_ADC；与另购C0G库存2只分开</t>
         </is>
       </c>
       <c r="J44" s="2" t="inlineStr"/>
@@ -4863,12 +4865,12 @@
       </c>
       <c r="H45" s="2" t="inlineStr">
         <is>
-          <t>用户已确认完整型号；库存数量待核</t>
+          <t>CL21B472JBANNNC，已购50只</t>
         </is>
       </c>
       <c r="I45" s="2" t="inlineStr">
         <is>
-          <t>用户回复就是这个型号；按其编码图确认为0805/4.7nF/50V/±5%/X7R，单板4只，四个位号源图未指定C0G。不得用于C_VINP_ADC，不与C0G库存混计</t>
+          <t>用户对这批X7R数量回复50；0805/4.7nF/50V/±5%/X7R，单板4只，补购0只，装一板后余46只。不得用于C_VINP_ADC；与另购C0G库存2只分开</t>
         </is>
       </c>
       <c r="J45" s="2" t="inlineStr"/>
@@ -4907,12 +4909,12 @@
       </c>
       <c r="H46" s="2" t="inlineStr">
         <is>
-          <t>用户已确认完整型号；库存数量待核</t>
+          <t>CL21B472JBANNNC，已购50只</t>
         </is>
       </c>
       <c r="I46" s="2" t="inlineStr">
         <is>
-          <t>用户回复就是这个型号；按其编码图确认为0805/4.7nF/50V/±5%/X7R，单板4只，四个位号源图未指定C0G。不得用于C_VINP_ADC，不与C0G库存混计</t>
+          <t>用户对这批X7R数量回复50；0805/4.7nF/50V/±5%/X7R，单板4只，补购0只，装一板后余46只。不得用于C_VINP_ADC；与另购C0G库存2只分开</t>
         </is>
       </c>
       <c r="J46" s="2" t="inlineStr"/>
@@ -9015,7 +9017,7 @@
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>C0G库存2只，单板需1只/补购0只；X7R库存数量及C0G完整料号/容差待核，两类不混装</t>
+          <t>X7R库存50只，单板4只/补购0只；C0G库存2只，单板1只/补购0只，两类不混装；C0G完整料号/容差待归档</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Record 1206 X7R 1nF purchase mismatch without changing PCB requirements
</commit_message>
<xml_diff>
--- a/projects/2026-electronics-contest/g-buck/rev-c2/downloads/GBUCK_RevC2_updated_BOM.xlsx
+++ b/projects/2026-electronics-contest/g-buck/rev-c2/downloads/GBUCK_RevC2_updated_BOM.xlsx
@@ -14,7 +14,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="重点变化与待确认" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'使用说明'!$A$1:$B$20</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'使用说明'!$A$1:$B$21</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'使用说明'!$1:$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'采购汇总'!$A$1:$J$47</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'采购汇总'!$1:$1</definedName>
@@ -457,7 +457,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:B20"/>
+  <dimension ref="A1:B21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="23" customWidth="1" min="1" max="1"/>
@@ -479,233 +479,245 @@
     <row r="2" ht="46" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>版本基准</t>
+          <t>最新1nF图片核对</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>本次比较238203e；用户确认CL21B472JBANNNC/X7R这批有50只，单板4只、补购0只、装一板后余46只；C0G库存2只和100nF库存50只保持，仅更新库存，设计不改。</t>
+          <t>比较8d57b27：用户新图已选规格为1206、1nF、±10%、50V、X7R，50只；无完整厂家型号。原理图C_IL_ADC/C_IL_PROT正常装配共2只，PCB均C0805，且C_IL_PROT明确C0G。这批1206/X7R不能视作0805/C0G可直接装配库存，50只不填入目标行库存。建议另备1nF/50V/C0G/0805共2只以统一备料；是否已有该款待核，不自动认定缺货2只。C_SN另为1nF/100V/C0G、DNP，本图也不能用于确认该项。原理图/PCB原生文件、网络、设计值和封装均未改；没有放大焊盘或放宽介质要求。仅更新实购物料记录及BOM待核状态，仿真/固件未修改或运行。</t>
         </is>
       </c>
     </row>
     <row r="3" ht="46" customHeight="1">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>计数口径</t>
+          <t>版本基准</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>120个逻辑位号含14个裸测试点、2个DNP预留和1个外置R_PRE。120不等于需购买120个独立实体。</t>
+          <t>本次比较238203e；用户确认CL21B472JBANNNC/X7R这批有50只，单板4只、补购0只、装一板后余46只；C0G库存2只和100nF库存50只保持，仅更新库存，设计不改。</t>
         </is>
       </c>
     </row>
     <row r="4" ht="46" customHeight="1">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>默认装配</t>
+          <t>计数口径</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>120−14裸测试点−2个DNP=104个有料逻辑位号；含R_PRE外置电阻。管夹、模块、开关和线束另表计数。</t>
+          <t>120个逻辑位号含14个裸测试点、2个DNP预留和1个外置R_PRE。120不等于需购买120个独立实体。</t>
         </is>
       </c>
     </row>
     <row r="5" ht="46" customHeight="1">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>库存填写</t>
+          <t>默认装配</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>采购汇总G列填写现有可用数量，H列自动计算需补购数量；100nF/X7R已填50只、4.7nF/X7R已填50只、4.7nF/C0G已填2只，三项单板补购均0只。其他空白表示库存未核，不代表未购买。</t>
+          <t>120−14裸测试点−2个DNP=104个有料逻辑位号；含R_PRE外置电阻。管夹、模块、开关和线束另表计数。</t>
         </is>
       </c>
     </row>
     <row r="6" ht="46" customHeight="1">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>DNP</t>
+          <t>库存填写</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>R_SN/C_SN各设计1个，默认装配0个；实测振铃后决定是否装配和调值。</t>
+          <t>采购汇总G列填写现有可用数量，H列自动计算需补购数量；100nF/X7R已填50只、4.7nF/X7R已填50只、4.7nF/C0G已填2只，三项单板补购均0只。其他空白表示库存未核，不代表未购买。</t>
         </is>
       </c>
     </row>
     <row r="7" ht="46" customHeight="1">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>采购规格</t>
+          <t>DNP</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>标“建议/统一采购”的额定、精度或介质是采购建议，区别于源图原始标注；实际原始值在逐位号页保留。</t>
+          <t>R_SN/C_SN各设计1个，默认装配0个；实测振铃后决定是否装配和调值。</t>
         </is>
       </c>
     </row>
     <row r="8" ht="46" customHeight="1">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>普通/精密电阻功率</t>
+          <t>采购规格</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>除源图另有功率要求的R_BL/R_SN/R_PRE和分流器外，0805电阻统一≥0.125W是本表采购建议，不冒充源图已规定的功率。</t>
+          <t>标“建议/统一采购”的额定、精度或介质是采购建议，区别于源图原始标注；实际原始值在逐位号页保留。</t>
         </is>
       </c>
     </row>
     <row r="9" ht="46" customHeight="1">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>优先核对</t>
+          <t>普通/精密电阻功率</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>U1型号家族/直插类别已确认；保留IR2184PbF设计标注，不再列为型号封装待确认或默认补购；库存数量另填，IR2104不可代装。RS_L 25mΩ在B3清单中已包含，旧表记未购，现库存待核，不再自动假定库存为0。</t>
+          <t>除源图另有功率要求的R_BL/R_SN/R_PRE和分流器外，0805电阻统一≥0.125W是本表采购建议，不冒充源图已规定的功率。</t>
         </is>
       </c>
     </row>
     <row r="10" ht="46" customHeight="1">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>电容数量</t>
+          <t>优先核对</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>100nF共16只、4.7nF共5只、默认1nF共2只，另有1只DNP的1nF/100V。</t>
+          <t>U1型号家族/直插类别已确认；保留IR2184PbF设计标注，不再列为型号封装待确认或默认补购；库存数量另填，IR2104不可代装。RS_L 25mΩ在B3清单中已包含，旧表记未购，现库存待核，不再自动假定库存为0。</t>
         </is>
       </c>
     </row>
     <row r="11" ht="46" customHeight="1">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>料号纠错</t>
+          <t>电容数量</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>472批次已确认4.7nF；随后用户确认另外买了100nF/0805，两批分开记录。100nF/50V/0805/X7R已购50只，单板需求16只，补购0只，装配一板后余34只；完整料号/容差未提供；用户现已确认实际型号CL21B472JBANNNC，先前口头C0G由实际型号纠正为X7R；该款50V/±5%/0805按用户编码图明确。C_VINP_ADC所需的4.7nF/50V/C0G/0805另购状态已获确认；该批C0G库存2只、单板用1只/补购0只；C0G完整料号/容差待归档；CL21B472JBANNNC/X7R库存现已确认50只、单板用4只/补购0只，两类不混计。</t>
+          <t>100nF共16只、4.7nF共5只、默认1nF共2只，另有1只DNP的1nF/100V。</t>
         </is>
       </c>
     </row>
     <row r="12" ht="46" customHeight="1">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>分流器新证据</t>
+          <t>料号纠错</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>RS_IN/OUT：50mΩ P10、图示线径0.8、体高12、标称5A；RS_L：25mΩ P5、图示线径0.7、体高7。电阻体线径不自动证明焊接直脚径，精度/连续功率仍待核。</t>
+          <t>472批次已确认4.7nF；随后用户确认另外买了100nF/0805，两批分开记录。100nF/50V/0805/X7R已购50只，单板需求16只，补购0只，装配一板后余34只；完整料号/容差未提供；用户现已确认实际型号CL21B472JBANNNC，先前口头C0G由实际型号纠正为X7R；该款50V/±5%/0805按用户编码图明确。C_VINP_ADC所需的4.7nF/50V/C0G/0805另购状态已获确认；该批C0G库存2只、单板用1只/补购0只；C0G完整料号/容差待归档；CL21B472JBANNNC/X7R库存现已确认50只、单板用4只/补购0只，两类不混计。</t>
         </is>
       </c>
     </row>
     <row r="13" ht="46" customHeight="1">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>保险夹确认</t>
+          <t>分流器新证据</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>用户明确单夹脚中心距5.66mm；脚宽1.1/材料厚0.5。槽0.9×1.5及双夹中心距15mm是设计选择，装入5×20实物核对端帽接触/止挡后方可冻结；不能使用旧6×30/7.7尺寸。</t>
+          <t>RS_IN/OUT：50mΩ P10、图示线径0.8、体高12、标称5A；RS_L：25mΩ P5、图示线径0.7、体高7。电阻体线径不自动证明焊接直脚径，精度/连续功率仍待核。</t>
         </is>
       </c>
     </row>
     <row r="14" ht="46" customHeight="1">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>二极管确认</t>
+          <t>保险夹确认</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>两只SR560/SMB已由用户明确；沿用现有SMB标准几何，1=K/2=A。DO-201AD图不用于贴片建库，厂家完整电气手册/推荐焊盘最终复核仍需归档。</t>
+          <t>用户明确单夹脚中心距5.66mm；脚宽1.1/材料厚0.5。槽0.9×1.5及双夹中心距15mm是设计选择，装入5×20实物核对端帽接触/止挡后方可冻结；不能使用旧6×30/7.7尺寸。</t>
         </is>
       </c>
     </row>
     <row r="15" ht="46" customHeight="1">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>未确认封装</t>
+          <t>二极管确认</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>C_A3的0805类别已确认；F1组合试装、分流器完整包络及外壳固定仍待核。C_A3完整料号/介质/偏压有效容量、二极管厂家数据待最终复核。</t>
+          <t>两只SR560/SMB已由用户明确；沿用现有SMB标准几何，1=K/2=A。DO-201AD图不用于贴片建库，厂家完整电气手册/推荐焊盘最终复核仍需归档。</t>
         </is>
       </c>
     </row>
     <row r="16" ht="46" customHeight="1">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>电感</t>
+          <t>未确认封装</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>65125图示6A Max不是饱和电流保证；源设计仍要求Isat≥3A、Irms≥1.5A、DCR≤0.15Ω。</t>
+          <t>C_A3的0805类别已确认；F1组合试装、分流器完整包络及外壳固定仍待核。C_A3完整料号/介质/偏压有效容量、二极管厂家数据待最终复核。</t>
         </is>
       </c>
     </row>
     <row r="17" ht="46" customHeight="1">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>当前制造状态</t>
+          <t>电感</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>PCB仍有未布连接，客户端打开、原生ERC/DRC未完成；清单提供采购核对依据，不是制板放行。</t>
+          <t>65125图示6A Max不是饱和电流保证；源设计仍要求Isat≥3A、Irms≥1.5A、DCR≤0.15Ω。</t>
         </is>
       </c>
     </row>
     <row r="18" ht="46" customHeight="1">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>本次原理图影响</t>
+          <t>当前制造状态</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>相对238203e，仅登记C7～C10所用CL21B472JBANNNC/X7R库存50只；原理图和PCB原生文件未改，网络/脚号/设计参数与单板用量保持，4.7nF仍4只X7R加1只C0G。</t>
+          <t>PCB仍有未布连接，客户端打开、原生ERC/DRC未完成；清单提供采购核对依据，不是制板放行。</t>
         </is>
       </c>
     </row>
     <row r="19" ht="46" customHeight="1">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>本次器件/PCB影响</t>
+          <t>本次原理图影响</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>C7～C10的X7R款已购50只，单板用4只，补购0只，预计装一板余46只；Excel保留公式，CSV写当前50/0，未实际扣减库存。C0G库存2只、100nF库存50只、46采购行/120位号/104默认有料及PCB几何保持，无新增或改板要求。</t>
+          <t>相对238203e，仅登记C7～C10所用CL21B472JBANNNC/X7R库存50只；原理图和PCB原生文件未改，网络/脚号/设计参数与单板用量保持，4.7nF仍4只X7R加1只C0G。</t>
         </is>
       </c>
     </row>
     <row r="20" ht="46" customHeight="1">
       <c r="A20" s="2" t="inlineStr">
         <is>
+          <t>本次器件/PCB影响</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>C7～C10的X7R款已购50只，单板用4只，补购0只，预计装一板余46只；Excel保留公式，CSV写当前50/0，未实际扣减库存。C0G库存2只、100nF库存50只、46采购行/120位号/104默认有料及PCB几何保持，无新增或改板要求。</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="46" customHeight="1">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
           <t>本次仿真/固件影响</t>
         </is>
       </c>
-      <c r="B20" s="2" t="inlineStr">
+      <c r="B21" s="2" t="inlineStr">
         <is>
           <t>未修改或运行Multisim/ngspice/STM32固件，旧器件/功能等效模型未同步为SR560厂家模型，不证明新选型压降、温升、效率或保护实测通过。</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:B20"/>
+  <autoFilter ref="A1:B21"/>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" paperSize="8" fitToHeight="0" fitToWidth="1"/>
@@ -1728,12 +1740,12 @@
       </c>
       <c r="I23" s="2" t="inlineStr">
         <is>
-          <t>核对已购物料</t>
+          <t>实购图为1206/X7R，与设计不符</t>
         </is>
       </c>
       <c r="J23" s="2" t="inlineStr">
         <is>
-          <t>正常装配2只；C_IL_PROT明确C0G</t>
+          <t>正常装配2只、当前PCB均0805；C_IL_PROT明确C0G。用户图片已选1206/1nF/±10%/50V/X7R/50只，不能计作本行直接可装库存；保留设计，另备0805/C0G款或另行评估改版</t>
         </is>
       </c>
     </row>
@@ -5001,12 +5013,12 @@
       </c>
       <c r="H48" s="2" t="inlineStr">
         <is>
-          <t>核对已购物料</t>
+          <t>实购图为1206/X7R，与设计不符</t>
         </is>
       </c>
       <c r="I48" s="2" t="inlineStr">
         <is>
-          <t>正常装配2只；C_IL_PROT明确C0G</t>
+          <t>正常装配2只、当前PCB均0805；C_IL_PROT明确C0G。用户图片已选1206/1nF/±10%/50V/X7R/50只，不能计作本行直接可装库存；保留设计，另备0805/C0G款或另行评估改版</t>
         </is>
       </c>
       <c r="J48" s="2" t="inlineStr"/>
@@ -5045,12 +5057,12 @@
       </c>
       <c r="H49" s="2" t="inlineStr">
         <is>
-          <t>核对已购物料</t>
+          <t>实购图为1206/X7R，与设计不符</t>
         </is>
       </c>
       <c r="I49" s="2" t="inlineStr">
         <is>
-          <t>正常装配2只；C_IL_PROT明确C0G</t>
+          <t>正常装配2只、当前PCB均0805；C_IL_PROT明确C0G。用户图片已选1206/1nF/±10%/50V/X7R/50只，不能计作本行直接可装库存；保留设计，另备0805/C0G款或另行评估改版</t>
         </is>
       </c>
       <c r="J49" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Record separately purchased 0805 C0G 1nF capacitors
</commit_message>
<xml_diff>
--- a/projects/2026-electronics-contest/g-buck/rev-c2/downloads/GBUCK_RevC2_updated_BOM.xlsx
+++ b/projects/2026-electronics-contest/g-buck/rev-c2/downloads/GBUCK_RevC2_updated_BOM.xlsx
@@ -14,7 +14,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="重点变化与待确认" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'使用说明'!$A$1:$B$21</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'使用说明'!$A$1:$B$22</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'使用说明'!$1:$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'采购汇总'!$A$1:$J$47</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'采购汇总'!$1:$1</definedName>
@@ -457,7 +457,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:B21"/>
+  <dimension ref="A1:B22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="23" customWidth="1" min="1" max="1"/>
@@ -479,245 +479,257 @@
     <row r="2" ht="46" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>最新1nF图片核对</t>
+          <t>最新1nF另购确认</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>比较8d57b27：用户新图已选规格为1206、1nF、±10%、50V、X7R，50只；无完整厂家型号。原理图C_IL_ADC/C_IL_PROT正常装配共2只，PCB均C0805，且C_IL_PROT明确C0G。这批1206/X7R不能视作0805/C0G可直接装配库存，50只不填入目标行库存。建议另备1nF/50V/C0G/0805共2只以统一备料；是否已有该款待核，不自动认定缺货2只。C_SN另为1nF/100V/C0G、DNP，本图也不能用于确认该项。原理图/PCB原生文件、网络、设计值和封装均未改；没有放大焊盘或放宽介质要求。仅更新实购物料记录及BOM待核状态，仿真/固件未修改或运行。</t>
+          <t>比较1dac34a：用户对是否另有1nF/50V/C0G（NP0）/0805回复“买了”，确认正常装配C_IL_ADC、C_IL_PROT所需C0G款已另购，每板共2只。实际数量、完整料号和容差未提供，库存/补购栏留空，不把设计需求2只当成库存。此前图片1206/1nF/±10%/50V/X7R/50只仍单独登记，不抵扣0805/C0G需求；本轮50V规格确认不用于C_SN的1nF/100V/C0G/DNP预留。原理图和PCB原生文件、网络、脚号、设计值/封装及用量均未改；仅更新BOM已购状态，不需要本轮改板或新增逻辑器件。46采购行、120逻辑位号、104默认有料及先前三类已确认库存保持；仿真/固件未修改或运行。</t>
         </is>
       </c>
     </row>
     <row r="3" ht="46" customHeight="1">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>版本基准</t>
+          <t>历史1nF图片核对（后续另购见最新项）</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>本次比较238203e；用户确认CL21B472JBANNNC/X7R这批有50只，单板4只、补购0只、装一板后余46只；C0G库存2只和100nF库存50只保持，仅更新库存，设计不改。</t>
+          <t>比较8d57b27：用户新图已选规格为1206、1nF、±10%、50V、X7R，50只；无完整厂家型号。原理图C_IL_ADC/C_IL_PROT正常装配共2只，PCB均C0805，且C_IL_PROT明确C0G。这批1206/X7R不能视作0805/C0G可直接装配库存，50只不填入目标行库存。建议另备1nF/50V/C0G/0805共2只以统一备料；是否已有该款待核，不自动认定缺货2只。C_SN另为1nF/100V/C0G、DNP，本图也不能用于确认该项。原理图/PCB原生文件、网络、设计值和封装均未改；没有放大焊盘或放宽介质要求。仅更新实购物料记录及BOM待核状态，仿真/固件未修改或运行。</t>
         </is>
       </c>
     </row>
     <row r="4" ht="46" customHeight="1">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>计数口径</t>
+          <t>版本基准</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>120个逻辑位号含14个裸测试点、2个DNP预留和1个外置R_PRE。120不等于需购买120个独立实体。</t>
+          <t>本次比较1dac34a；1nF/50V/C0G/0805另购已确认，数量待核。设计及既有库存保持。</t>
         </is>
       </c>
     </row>
     <row r="5" ht="46" customHeight="1">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>默认装配</t>
+          <t>计数口径</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>120−14裸测试点−2个DNP=104个有料逻辑位号；含R_PRE外置电阻。管夹、模块、开关和线束另表计数。</t>
+          <t>120个逻辑位号含14个裸测试点、2个DNP预留和1个外置R_PRE。120不等于需购买120个独立实体。</t>
         </is>
       </c>
     </row>
     <row r="6" ht="46" customHeight="1">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>库存填写</t>
+          <t>默认装配</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>采购汇总G列填写现有可用数量，H列自动计算需补购数量；100nF/X7R已填50只、4.7nF/X7R已填50只、4.7nF/C0G已填2只，三项单板补购均0只。其他空白表示库存未核，不代表未购买。</t>
+          <t>120−14裸测试点−2个DNP=104个有料逻辑位号；含R_PRE外置电阻。管夹、模块、开关和线束另表计数。</t>
         </is>
       </c>
     </row>
     <row r="7" ht="46" customHeight="1">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>DNP</t>
+          <t>库存填写</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>R_SN/C_SN各设计1个，默认装配0个；实测振铃后决定是否装配和调值。</t>
+          <t>采购汇总G列填写现有可用数量，H列自动计算需补购数量；100nF/X7R已填50只、4.7nF/X7R已填50只、4.7nF/C0G已填2只，三项单板补购均0只。其他空白表示库存未核，不代表未购买。</t>
         </is>
       </c>
     </row>
     <row r="8" ht="46" customHeight="1">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>采购规格</t>
+          <t>DNP</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>标“建议/统一采购”的额定、精度或介质是采购建议，区别于源图原始标注；实际原始值在逐位号页保留。</t>
+          <t>R_SN/C_SN各设计1个，默认装配0个；实测振铃后决定是否装配和调值。</t>
         </is>
       </c>
     </row>
     <row r="9" ht="46" customHeight="1">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>普通/精密电阻功率</t>
+          <t>采购规格</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>除源图另有功率要求的R_BL/R_SN/R_PRE和分流器外，0805电阻统一≥0.125W是本表采购建议，不冒充源图已规定的功率。</t>
+          <t>标“建议/统一采购”的额定、精度或介质是采购建议，区别于源图原始标注；实际原始值在逐位号页保留。</t>
         </is>
       </c>
     </row>
     <row r="10" ht="46" customHeight="1">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>优先核对</t>
+          <t>普通/精密电阻功率</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>U1型号家族/直插类别已确认；保留IR2184PbF设计标注，不再列为型号封装待确认或默认补购；库存数量另填，IR2104不可代装。RS_L 25mΩ在B3清单中已包含，旧表记未购，现库存待核，不再自动假定库存为0。</t>
+          <t>除源图另有功率要求的R_BL/R_SN/R_PRE和分流器外，0805电阻统一≥0.125W是本表采购建议，不冒充源图已规定的功率。</t>
         </is>
       </c>
     </row>
     <row r="11" ht="46" customHeight="1">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>电容数量</t>
+          <t>优先核对</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>100nF共16只、4.7nF共5只、默认1nF共2只，另有1只DNP的1nF/100V。</t>
+          <t>U1型号家族/直插类别已确认；保留IR2184PbF设计标注，不再列为型号封装待确认或默认补购；库存数量另填，IR2104不可代装。RS_L 25mΩ在B3清单中已包含，旧表记未购，现库存待核，不再自动假定库存为0。</t>
         </is>
       </c>
     </row>
     <row r="12" ht="46" customHeight="1">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>料号纠错</t>
+          <t>电容数量</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>472批次已确认4.7nF；随后用户确认另外买了100nF/0805，两批分开记录。100nF/50V/0805/X7R已购50只，单板需求16只，补购0只，装配一板后余34只；完整料号/容差未提供；用户现已确认实际型号CL21B472JBANNNC，先前口头C0G由实际型号纠正为X7R；该款50V/±5%/0805按用户编码图明确。C_VINP_ADC所需的4.7nF/50V/C0G/0805另购状态已获确认；该批C0G库存2只、单板用1只/补购0只；C0G完整料号/容差待归档；CL21B472JBANNNC/X7R库存现已确认50只、单板用4只/补购0只，两类不混计。</t>
+          <t>100nF共16只、4.7nF共5只、默认1nF共2只，另有1只DNP的1nF/100V。</t>
         </is>
       </c>
     </row>
     <row r="13" ht="46" customHeight="1">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>分流器新证据</t>
+          <t>料号纠错</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>RS_IN/OUT：50mΩ P10、图示线径0.8、体高12、标称5A；RS_L：25mΩ P5、图示线径0.7、体高7。电阻体线径不自动证明焊接直脚径，精度/连续功率仍待核。</t>
+          <t>472批次已确认4.7nF；随后用户确认另外买了100nF/0805，两批分开记录。100nF/50V/0805/X7R已购50只，单板需求16只，补购0只，装配一板后余34只；完整料号/容差未提供；用户现已确认实际型号CL21B472JBANNNC，先前口头C0G由实际型号纠正为X7R；该款50V/±5%/0805按用户编码图明确。C_VINP_ADC所需的4.7nF/50V/C0G/0805另购状态已获确认；该批C0G库存2只、单板用1只/补购0只；C0G完整料号/容差待归档；CL21B472JBANNNC/X7R库存现已确认50只、单板用4只/补购0只，两类不混计。</t>
         </is>
       </c>
     </row>
     <row r="14" ht="46" customHeight="1">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>保险夹确认</t>
+          <t>分流器新证据</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>用户明确单夹脚中心距5.66mm；脚宽1.1/材料厚0.5。槽0.9×1.5及双夹中心距15mm是设计选择，装入5×20实物核对端帽接触/止挡后方可冻结；不能使用旧6×30/7.7尺寸。</t>
+          <t>RS_IN/OUT：50mΩ P10、图示线径0.8、体高12、标称5A；RS_L：25mΩ P5、图示线径0.7、体高7。电阻体线径不自动证明焊接直脚径，精度/连续功率仍待核。</t>
         </is>
       </c>
     </row>
     <row r="15" ht="46" customHeight="1">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>二极管确认</t>
+          <t>保险夹确认</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>两只SR560/SMB已由用户明确；沿用现有SMB标准几何，1=K/2=A。DO-201AD图不用于贴片建库，厂家完整电气手册/推荐焊盘最终复核仍需归档。</t>
+          <t>用户明确单夹脚中心距5.66mm；脚宽1.1/材料厚0.5。槽0.9×1.5及双夹中心距15mm是设计选择，装入5×20实物核对端帽接触/止挡后方可冻结；不能使用旧6×30/7.7尺寸。</t>
         </is>
       </c>
     </row>
     <row r="16" ht="46" customHeight="1">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>未确认封装</t>
+          <t>二极管确认</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>C_A3的0805类别已确认；F1组合试装、分流器完整包络及外壳固定仍待核。C_A3完整料号/介质/偏压有效容量、二极管厂家数据待最终复核。</t>
+          <t>两只SR560/SMB已由用户明确；沿用现有SMB标准几何，1=K/2=A。DO-201AD图不用于贴片建库，厂家完整电气手册/推荐焊盘最终复核仍需归档。</t>
         </is>
       </c>
     </row>
     <row r="17" ht="46" customHeight="1">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>电感</t>
+          <t>未确认封装</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>65125图示6A Max不是饱和电流保证；源设计仍要求Isat≥3A、Irms≥1.5A、DCR≤0.15Ω。</t>
+          <t>C_A3的0805类别已确认；F1组合试装、分流器完整包络及外壳固定仍待核。C_A3完整料号/介质/偏压有效容量、二极管厂家数据待最终复核。</t>
         </is>
       </c>
     </row>
     <row r="18" ht="46" customHeight="1">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>当前制造状态</t>
+          <t>电感</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>PCB仍有未布连接，客户端打开、原生ERC/DRC未完成；清单提供采购核对依据，不是制板放行。</t>
+          <t>65125图示6A Max不是饱和电流保证；源设计仍要求Isat≥3A、Irms≥1.5A、DCR≤0.15Ω。</t>
         </is>
       </c>
     </row>
     <row r="19" ht="46" customHeight="1">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>本次原理图影响</t>
+          <t>当前制造状态</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>相对238203e，仅登记C7～C10所用CL21B472JBANNNC/X7R库存50只；原理图和PCB原生文件未改，网络/脚号/设计参数与单板用量保持，4.7nF仍4只X7R加1只C0G。</t>
+          <t>PCB仍有未布连接，客户端打开、原生ERC/DRC未完成；清单提供采购核对依据，不是制板放行。</t>
         </is>
       </c>
     </row>
     <row r="20" ht="46" customHeight="1">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>本次器件/PCB影响</t>
+          <t>本次原理图影响</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>C7～C10的X7R款已购50只，单板用4只，补购0只，预计装一板余46只；Excel保留公式，CSV写当前50/0，未实际扣减库存。C0G库存2只、100nF库存50只、46采购行/120位号/104默认有料及PCB几何保持，无新增或改板要求。</t>
+          <t>相对1dac34a，原理图和PCB原生文件未改，网络/脚号/设计值/封装和单板用量保持。</t>
         </is>
       </c>
     </row>
     <row r="21" ht="46" customHeight="1">
       <c r="A21" s="2" t="inlineStr">
         <is>
+          <t>本次器件/PCB影响</t>
+        </is>
+      </c>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>1nF/50V/C0G/0805已另购，每板2只，数量/完整料号/容差待核；1206/X7R款分开，不自动填可装库存。46采购行/120位号/104默认有料及已确认三类库存保持，无本轮改板要求。</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="46" customHeight="1">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
           <t>本次仿真/固件影响</t>
         </is>
       </c>
-      <c r="B21" s="2" t="inlineStr">
+      <c r="B22" s="2" t="inlineStr">
         <is>
           <t>未修改或运行Multisim/ngspice/STM32固件，旧器件/功能等效模型未同步为SR560厂家模型，不证明新选型压降、温升、效率或保护实测通过。</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:B21"/>
+  <autoFilter ref="A1:B22"/>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" paperSize="8" fitToHeight="0" fitToWidth="1"/>
@@ -1714,7 +1726,7 @@
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>1nF/50V，建议C0G/NP0</t>
+          <t>1nF/50V，C0G/NP0</t>
         </is>
       </c>
       <c r="C23" s="2" t="inlineStr">
@@ -1740,12 +1752,12 @@
       </c>
       <c r="I23" s="2" t="inlineStr">
         <is>
-          <t>实购图为1206/X7R，与设计不符</t>
+          <t>用户确认另购0805/C0G款；数量待核</t>
         </is>
       </c>
       <c r="J23" s="2" t="inlineStr">
         <is>
-          <t>正常装配2只、当前PCB均0805；C_IL_PROT明确C0G。用户图片已选1206/1nF/±10%/50V/X7R/50只，不能计作本行直接可装库存；保留设计，另备0805/C0G款或另行评估改版</t>
+          <t>用户对是否另有1nF/50V/C0G/0805回复买了；正常装配共2只，与图片1206/X7R/50只分开。实际数量/完整料号/容差未提供，库存和补购栏留空，不自动填2只；不覆盖C_SN的100V/DNP项</t>
         </is>
       </c>
     </row>
@@ -4997,7 +5009,7 @@
       </c>
       <c r="D48" s="2" t="inlineStr">
         <is>
-          <t>1nF/50V，建议C0G/NP0</t>
+          <t>1nF/50V，C0G/NP0</t>
         </is>
       </c>
       <c r="E48" s="2" t="inlineStr">
@@ -5013,12 +5025,12 @@
       </c>
       <c r="H48" s="2" t="inlineStr">
         <is>
-          <t>实购图为1206/X7R，与设计不符</t>
+          <t>用户确认另购0805/C0G款；数量待核</t>
         </is>
       </c>
       <c r="I48" s="2" t="inlineStr">
         <is>
-          <t>正常装配2只、当前PCB均0805；C_IL_PROT明确C0G。用户图片已选1206/1nF/±10%/50V/X7R/50只，不能计作本行直接可装库存；保留设计，另备0805/C0G款或另行评估改版</t>
+          <t>用户对是否另有1nF/50V/C0G/0805回复买了；正常装配共2只，与图片1206/X7R/50只分开。实际数量/完整料号/容差未提供，库存和补购栏留空，不自动填2只；不覆盖C_SN的100V/DNP项</t>
         </is>
       </c>
       <c r="J48" s="2" t="inlineStr"/>
@@ -5041,7 +5053,7 @@
       </c>
       <c r="D49" s="2" t="inlineStr">
         <is>
-          <t>1nF/50V，建议C0G/NP0</t>
+          <t>1nF/50V，C0G/NP0</t>
         </is>
       </c>
       <c r="E49" s="2" t="inlineStr">
@@ -5057,12 +5069,12 @@
       </c>
       <c r="H49" s="2" t="inlineStr">
         <is>
-          <t>实购图为1206/X7R，与设计不符</t>
+          <t>用户确认另购0805/C0G款；数量待核</t>
         </is>
       </c>
       <c r="I49" s="2" t="inlineStr">
         <is>
-          <t>正常装配2只、当前PCB均0805；C_IL_PROT明确C0G。用户图片已选1206/1nF/±10%/50V/X7R/50只，不能计作本行直接可装库存；保留设计，另备0805/C0G款或另行评估改版</t>
+          <t>用户对是否另有1nF/50V/C0G/0805回复买了；正常装配共2只，与图片1206/X7R/50只分开。实际数量/完整料号/容差未提供，库存和补购栏留空，不自动填2只；不覆盖C_SN的100V/DNP项</t>
         </is>
       </c>
       <c r="J49" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Record four 0805 C0G 1nF capacitors and single-board inventory balance
</commit_message>
<xml_diff>
--- a/projects/2026-electronics-contest/g-buck/rev-c2/downloads/GBUCK_RevC2_updated_BOM.xlsx
+++ b/projects/2026-electronics-contest/g-buck/rev-c2/downloads/GBUCK_RevC2_updated_BOM.xlsx
@@ -14,7 +14,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="重点变化与待确认" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'使用说明'!$A$1:$B$22</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'使用说明'!$A$1:$B$23</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'使用说明'!$1:$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'采购汇总'!$A$1:$J$47</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'采购汇总'!$1:$1</definedName>
@@ -457,7 +457,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:B22"/>
+  <dimension ref="A1:B23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="23" customWidth="1" min="1" max="1"/>
@@ -479,257 +479,269 @@
     <row r="2" ht="46" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>最新1nF另购确认</t>
+          <t>最新1nF数量确认</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>比较1dac34a：用户对是否另有1nF/50V/C0G（NP0）/0805回复“买了”，确认正常装配C_IL_ADC、C_IL_PROT所需C0G款已另购，每板共2只。实际数量、完整料号和容差未提供，库存/补购栏留空，不把设计需求2只当成库存。此前图片1206/1nF/±10%/50V/X7R/50只仍单独登记，不抵扣0805/C0G需求；本轮50V规格确认不用于C_SN的1nF/100V/C0G/DNP预留。原理图和PCB原生文件、网络、脚号、设计值/封装及用量均未改；仅更新BOM已购状态，不需要本轮改板或新增逻辑器件。46采购行、120逻辑位号、104默认有料及先前三类已确认库存保持；仿真/固件未修改或运行。</t>
+          <t>比较6f26307：用户对另购1nF/50V/C0G（NP0）/0805数量回复“4”，登记库存4只。C_IL_ADC、C_IL_PROT单板各1只，共2只；需补购0只，预计装一板后余2只，尚未实际扣减库存。Excel库存填4、补购保留动态公式，CSV写当前4/0。图片中的1206/X7R/50只另记，不混入本项；本次50V备料不覆盖C_SN的100V/C0G/DNP预留。完整料号/容差待归档；采购46行、120逻辑位号/104默认有料及先前三类库存保持。原理图/PCB原生文件、网络、脚号、设计值/封装及单板用量未改，仅更新库存和补购记录，无新增器件或改板要求；仿真/固件未修改或运行。</t>
         </is>
       </c>
     </row>
     <row r="3" ht="46" customHeight="1">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>历史1nF图片核对（后续另购见最新项）</t>
+          <t>历史1nF另购确认（数量已后补）</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>比较8d57b27：用户新图已选规格为1206、1nF、±10%、50V、X7R，50只；无完整厂家型号。原理图C_IL_ADC/C_IL_PROT正常装配共2只，PCB均C0805，且C_IL_PROT明确C0G。这批1206/X7R不能视作0805/C0G可直接装配库存，50只不填入目标行库存。建议另备1nF/50V/C0G/0805共2只以统一备料；是否已有该款待核，不自动认定缺货2只。C_SN另为1nF/100V/C0G、DNP，本图也不能用于确认该项。原理图/PCB原生文件、网络、设计值和封装均未改；没有放大焊盘或放宽介质要求。仅更新实购物料记录及BOM待核状态，仿真/固件未修改或运行。</t>
+          <t>比较1dac34a：用户对是否另有1nF/50V/C0G（NP0）/0805回复“买了”，确认正常装配C_IL_ADC、C_IL_PROT所需C0G款已另购，每板共2只。实际数量、完整料号和容差未提供，库存/补购栏留空，不把设计需求2只当成库存。此前图片1206/1nF/±10%/50V/X7R/50只仍单独登记，不抵扣0805/C0G需求；本轮50V规格确认不用于C_SN的1nF/100V/C0G/DNP预留。原理图和PCB原生文件、网络、脚号、设计值/封装及用量均未改；仅更新BOM已购状态，不需要本轮改板或新增逻辑器件。46采购行、120逻辑位号、104默认有料及先前三类已确认库存保持；仿真/固件未修改或运行。</t>
         </is>
       </c>
     </row>
     <row r="4" ht="46" customHeight="1">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>版本基准</t>
+          <t>历史1nF图片核对（后续另购见最新项）</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>本次比较1dac34a；1nF/50V/C0G/0805另购已确认，数量待核。设计及既有库存保持。</t>
+          <t>比较8d57b27：用户新图已选规格为1206、1nF、±10%、50V、X7R，50只；无完整厂家型号。原理图C_IL_ADC/C_IL_PROT正常装配共2只，PCB均C0805，且C_IL_PROT明确C0G。这批1206/X7R不能视作0805/C0G可直接装配库存，50只不填入目标行库存。建议另备1nF/50V/C0G/0805共2只以统一备料；是否已有该款待核，不自动认定缺货2只。C_SN另为1nF/100V/C0G、DNP，本图也不能用于确认该项。原理图/PCB原生文件、网络、设计值和封装均未改；没有放大焊盘或放宽介质要求。仅更新实购物料记录及BOM待核状态，仿真/固件未修改或运行。</t>
         </is>
       </c>
     </row>
     <row r="5" ht="46" customHeight="1">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>计数口径</t>
+          <t>版本基准</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>120个逻辑位号含14个裸测试点、2个DNP预留和1个外置R_PRE。120不等于需购买120个独立实体。</t>
+          <t>本次比较6f26307；1nF/50V/C0G/0805已购4只，单板用2只/补购0只/装一板余2只；仅更新库存，设计保持。</t>
         </is>
       </c>
     </row>
     <row r="6" ht="46" customHeight="1">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>默认装配</t>
+          <t>计数口径</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>120−14裸测试点−2个DNP=104个有料逻辑位号；含R_PRE外置电阻。管夹、模块、开关和线束另表计数。</t>
+          <t>120个逻辑位号含14个裸测试点、2个DNP预留和1个外置R_PRE。120不等于需购买120个独立实体。</t>
         </is>
       </c>
     </row>
     <row r="7" ht="46" customHeight="1">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>库存填写</t>
+          <t>默认装配</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>采购汇总G列填写现有可用数量，H列自动计算需补购数量；100nF/X7R已填50只、4.7nF/X7R已填50只、4.7nF/C0G已填2只，三项单板补购均0只。其他空白表示库存未核，不代表未购买。</t>
+          <t>120−14裸测试点−2个DNP=104个有料逻辑位号；含R_PRE外置电阻。管夹、模块、开关和线束另表计数。</t>
         </is>
       </c>
     </row>
     <row r="8" ht="46" customHeight="1">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>DNP</t>
+          <t>库存填写</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>R_SN/C_SN各设计1个，默认装配0个；实测振铃后决定是否装配和调值。</t>
+          <t>G列已填用户确认库存：100nF/X7R 50只、4.7nF/X7R 50只、4.7nF/C0G 2只、1nF/C0G 4只，四项单板补购均0。其他空白表示未知，不代表未购。</t>
         </is>
       </c>
     </row>
     <row r="9" ht="46" customHeight="1">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>采购规格</t>
+          <t>DNP</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>标“建议/统一采购”的额定、精度或介质是采购建议，区别于源图原始标注；实际原始值在逐位号页保留。</t>
+          <t>R_SN/C_SN各设计1个，默认装配0个；实测振铃后决定是否装配和调值。</t>
         </is>
       </c>
     </row>
     <row r="10" ht="46" customHeight="1">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>普通/精密电阻功率</t>
+          <t>采购规格</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>除源图另有功率要求的R_BL/R_SN/R_PRE和分流器外，0805电阻统一≥0.125W是本表采购建议，不冒充源图已规定的功率。</t>
+          <t>标“建议/统一采购”的额定、精度或介质是采购建议，区别于源图原始标注；实际原始值在逐位号页保留。</t>
         </is>
       </c>
     </row>
     <row r="11" ht="46" customHeight="1">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>优先核对</t>
+          <t>普通/精密电阻功率</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>U1型号家族/直插类别已确认；保留IR2184PbF设计标注，不再列为型号封装待确认或默认补购；库存数量另填，IR2104不可代装。RS_L 25mΩ在B3清单中已包含，旧表记未购，现库存待核，不再自动假定库存为0。</t>
+          <t>除源图另有功率要求的R_BL/R_SN/R_PRE和分流器外，0805电阻统一≥0.125W是本表采购建议，不冒充源图已规定的功率。</t>
         </is>
       </c>
     </row>
     <row r="12" ht="46" customHeight="1">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>电容数量</t>
+          <t>优先核对</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>100nF共16只、4.7nF共5只、默认1nF共2只，另有1只DNP的1nF/100V。</t>
+          <t>U1型号家族/直插类别已确认；保留IR2184PbF设计标注，不再列为型号封装待确认或默认补购；库存数量另填，IR2104不可代装。RS_L 25mΩ在B3清单中已包含，旧表记未购，现库存待核，不再自动假定库存为0。</t>
         </is>
       </c>
     </row>
     <row r="13" ht="46" customHeight="1">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>料号纠错</t>
+          <t>电容数量</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>472批次已确认4.7nF；随后用户确认另外买了100nF/0805，两批分开记录。100nF/50V/0805/X7R已购50只，单板需求16只，补购0只，装配一板后余34只；完整料号/容差未提供；用户现已确认实际型号CL21B472JBANNNC，先前口头C0G由实际型号纠正为X7R；该款50V/±5%/0805按用户编码图明确。C_VINP_ADC所需的4.7nF/50V/C0G/0805另购状态已获确认；该批C0G库存2只、单板用1只/补购0只；C0G完整料号/容差待归档；CL21B472JBANNNC/X7R库存现已确认50只、单板用4只/补购0只，两类不混计。</t>
+          <t>100nF共16只、4.7nF共5只、默认1nF共2只，另有1只DNP的1nF/100V。</t>
         </is>
       </c>
     </row>
     <row r="14" ht="46" customHeight="1">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>分流器新证据</t>
+          <t>料号纠错</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>RS_IN/OUT：50mΩ P10、图示线径0.8、体高12、标称5A；RS_L：25mΩ P5、图示线径0.7、体高7。电阻体线径不自动证明焊接直脚径，精度/连续功率仍待核。</t>
+          <t>472批次已确认4.7nF；随后用户确认另外买了100nF/0805，两批分开记录。100nF/50V/0805/X7R已购50只，单板需求16只，补购0只，装配一板后余34只；完整料号/容差未提供；用户现已确认实际型号CL21B472JBANNNC，先前口头C0G由实际型号纠正为X7R；该款50V/±5%/0805按用户编码图明确。C_VINP_ADC所需的4.7nF/50V/C0G/0805另购状态已获确认；该批C0G库存2只、单板用1只/补购0只；C0G完整料号/容差待归档；CL21B472JBANNNC/X7R库存现已确认50只、单板用4只/补购0只，两类不混计。</t>
         </is>
       </c>
     </row>
     <row r="15" ht="46" customHeight="1">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>保险夹确认</t>
+          <t>分流器新证据</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>用户明确单夹脚中心距5.66mm；脚宽1.1/材料厚0.5。槽0.9×1.5及双夹中心距15mm是设计选择，装入5×20实物核对端帽接触/止挡后方可冻结；不能使用旧6×30/7.7尺寸。</t>
+          <t>RS_IN/OUT：50mΩ P10、图示线径0.8、体高12、标称5A；RS_L：25mΩ P5、图示线径0.7、体高7。电阻体线径不自动证明焊接直脚径，精度/连续功率仍待核。</t>
         </is>
       </c>
     </row>
     <row r="16" ht="46" customHeight="1">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>二极管确认</t>
+          <t>保险夹确认</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>两只SR560/SMB已由用户明确；沿用现有SMB标准几何，1=K/2=A。DO-201AD图不用于贴片建库，厂家完整电气手册/推荐焊盘最终复核仍需归档。</t>
+          <t>用户明确单夹脚中心距5.66mm；脚宽1.1/材料厚0.5。槽0.9×1.5及双夹中心距15mm是设计选择，装入5×20实物核对端帽接触/止挡后方可冻结；不能使用旧6×30/7.7尺寸。</t>
         </is>
       </c>
     </row>
     <row r="17" ht="46" customHeight="1">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>未确认封装</t>
+          <t>二极管确认</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>C_A3的0805类别已确认；F1组合试装、分流器完整包络及外壳固定仍待核。C_A3完整料号/介质/偏压有效容量、二极管厂家数据待最终复核。</t>
+          <t>两只SR560/SMB已由用户明确；沿用现有SMB标准几何，1=K/2=A。DO-201AD图不用于贴片建库，厂家完整电气手册/推荐焊盘最终复核仍需归档。</t>
         </is>
       </c>
     </row>
     <row r="18" ht="46" customHeight="1">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>电感</t>
+          <t>未确认封装</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>65125图示6A Max不是饱和电流保证；源设计仍要求Isat≥3A、Irms≥1.5A、DCR≤0.15Ω。</t>
+          <t>C_A3的0805类别已确认；F1组合试装、分流器完整包络及外壳固定仍待核。C_A3完整料号/介质/偏压有效容量、二极管厂家数据待最终复核。</t>
         </is>
       </c>
     </row>
     <row r="19" ht="46" customHeight="1">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>当前制造状态</t>
+          <t>电感</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>PCB仍有未布连接，客户端打开、原生ERC/DRC未完成；清单提供采购核对依据，不是制板放行。</t>
+          <t>65125图示6A Max不是饱和电流保证；源设计仍要求Isat≥3A、Irms≥1.5A、DCR≤0.15Ω。</t>
         </is>
       </c>
     </row>
     <row r="20" ht="46" customHeight="1">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>本次原理图影响</t>
+          <t>当前制造状态</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>相对1dac34a，原理图和PCB原生文件未改，网络/脚号/设计值/封装和单板用量保持。</t>
+          <t>PCB仍有未布连接，客户端打开、原生ERC/DRC未完成；清单提供采购核对依据，不是制板放行。</t>
         </is>
       </c>
     </row>
     <row r="21" ht="46" customHeight="1">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>本次器件/PCB影响</t>
+          <t>本次原理图影响</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>1nF/50V/C0G/0805已另购，每板2只，数量/完整料号/容差待核；1206/X7R款分开，不自动填可装库存。46采购行/120位号/104默认有料及已确认三类库存保持，无本轮改板要求。</t>
+          <t>相对6f26307，原理图和PCB原生文件未改，网络/脚号/设计值/封装与单板用量保持。</t>
         </is>
       </c>
     </row>
     <row r="22" ht="46" customHeight="1">
       <c r="A22" s="2" t="inlineStr">
         <is>
+          <t>本次器件/PCB影响</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>1nF/50V/C0G/0805登记库存4只，单板用2只/补购0只，预计装一板余2只；1206/X7R款分开。完整料号/容差待归档，46采购行/120位号/104默认有料及既有三类库存保持，无新增或改板要求。</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="46" customHeight="1">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
           <t>本次仿真/固件影响</t>
         </is>
       </c>
-      <c r="B22" s="2" t="inlineStr">
+      <c r="B23" s="2" t="inlineStr">
         <is>
           <t>未修改或运行Multisim/ngspice/STM32固件，旧器件/功能等效模型未同步为SR560厂家模型，不证明新选型压降、温升、效率或保护实测通过。</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:B22"/>
+  <autoFilter ref="A1:B23"/>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" paperSize="8" fitToHeight="0" fitToWidth="1"/>
@@ -1745,19 +1757,21 @@
       <c r="F23" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="G23" s="3" t="n"/>
+      <c r="G23" s="3" t="n">
+        <v>4</v>
+      </c>
       <c r="H23" s="2">
         <f>IF(G23="","",MAX(F23-G23,0))</f>
         <v/>
       </c>
       <c r="I23" s="2" t="inlineStr">
         <is>
-          <t>用户确认另购0805/C0G款；数量待核</t>
+          <t>1nF/50V/C0G/0805，已购4只</t>
         </is>
       </c>
       <c r="J23" s="2" t="inlineStr">
         <is>
-          <t>用户对是否另有1nF/50V/C0G/0805回复买了；正常装配共2只，与图片1206/X7R/50只分开。实际数量/完整料号/容差未提供，库存和补购栏留空，不自动填2只；不覆盖C_SN的100V/DNP项</t>
+          <t>用户对这批0805/C0G的数量回复4；正常装配共2只，单板补购0只，装一板后余2只。与图片1206/X7R/50只分开；完整料号/容差未提供，不覆盖C_SN的100V/DNP项</t>
         </is>
       </c>
     </row>
@@ -5025,12 +5039,12 @@
       </c>
       <c r="H48" s="2" t="inlineStr">
         <is>
-          <t>用户确认另购0805/C0G款；数量待核</t>
+          <t>1nF/50V/C0G/0805，已购4只</t>
         </is>
       </c>
       <c r="I48" s="2" t="inlineStr">
         <is>
-          <t>用户对是否另有1nF/50V/C0G/0805回复买了；正常装配共2只，与图片1206/X7R/50只分开。实际数量/完整料号/容差未提供，库存和补购栏留空，不自动填2只；不覆盖C_SN的100V/DNP项</t>
+          <t>用户对这批0805/C0G的数量回复4；正常装配共2只，单板补购0只，装一板后余2只。与图片1206/X7R/50只分开；完整料号/容差未提供，不覆盖C_SN的100V/DNP项</t>
         </is>
       </c>
       <c r="J48" s="2" t="inlineStr"/>
@@ -5069,12 +5083,12 @@
       </c>
       <c r="H49" s="2" t="inlineStr">
         <is>
-          <t>用户确认另购0805/C0G款；数量待核</t>
+          <t>1nF/50V/C0G/0805，已购4只</t>
         </is>
       </c>
       <c r="I49" s="2" t="inlineStr">
         <is>
-          <t>用户对是否另有1nF/50V/C0G/0805回复买了；正常装配共2只，与图片1206/X7R/50只分开。实际数量/完整料号/容差未提供，库存和补购栏留空，不自动填2只；不覆盖C_SN的100V/DNP项</t>
+          <t>用户对这批0805/C0G的数量回复4；正常装配共2只，单板补购0只，装一板后余2只。与图片1206/X7R/50只分开；完整料号/容差未提供，不覆盖C_SN的100V/DNP项</t>
         </is>
       </c>
       <c r="J49" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Specify MN11SS4W01 for external precharge bypass and document replacement limits
</commit_message>
<xml_diff>
--- a/projects/2026-electronics-contest/g-buck/rev-c2/downloads/GBUCK_RevC2_updated_BOM.xlsx
+++ b/projects/2026-electronics-contest/g-buck/rev-c2/downloads/GBUCK_RevC2_updated_BOM.xlsx
@@ -14,7 +14,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="重点变化与待确认" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'使用说明'!$A$1:$B$23</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'使用说明'!$A$1:$B$24</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'使用说明'!$1:$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'采购汇总'!$A$1:$J$47</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'采购汇总'!$1:$1</definedName>
@@ -457,7 +457,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:B23"/>
+  <dimension ref="A1:B24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="23" customWidth="1" min="1" max="1"/>
@@ -479,269 +479,281 @@
     <row r="2" ht="46" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>最新1nF数量确认</t>
+          <t>2026-10-28旁路开关选型</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>比较6f26307：用户对另购1nF/50V/C0G（NP0）/0805数量回复“4”，登记库存4只。C_IL_ADC、C_IL_PROT单板各1只，共2只；需补购0只，预计装一板后余2只，尚未实际扣减库存。Excel库存填4、补购保留动态公式，CSV写当前4/0。图片中的1206/X7R/50只另记，不混入本项；本次50V备料不覆盖C_SN的100V/C0G/DNP预留。完整料号/容差待归档；采购46行、120逻辑位号/104默认有料及先前三类库存保持。原理图/PCB原生文件、网络、脚号、设计值/封装及单板用量未改，仅更新库存和补购记录，无新增器件或改板要求；仿真/固件未修改或运行。</t>
+          <t>比较8fe83d4：用户提出MN11SS4W01替代MSS-22D18。按当前唯一对应的J_BYP两线外接旁路用途，采用NKK MN11SS4W01，4A/30VDC满足≥3A/30VDC要求；SPST保持型，两焊片接FUSED/IN_PRE，不接GND。旧MSS-22D18未在工程中明确标注，其实际双路/换向使用情况未确认，不能宣称六脚通用替换。原理图/PCB原生文件、Gerber、接口及仿真/固件不改；外接开关BOM型号改变、需面板Ø6.5mm固定和两线焊接。库存/已购数量未知，不默认已经购买。预充后闭合、停机断电后打开，不作为电源隔离开关。</t>
         </is>
       </c>
     </row>
     <row r="3" ht="46" customHeight="1">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>历史1nF另购确认（数量已后补）</t>
+          <t>最新1nF数量确认</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>比较1dac34a：用户对是否另有1nF/50V/C0G（NP0）/0805回复“买了”，确认正常装配C_IL_ADC、C_IL_PROT所需C0G款已另购，每板共2只。实际数量、完整料号和容差未提供，库存/补购栏留空，不把设计需求2只当成库存。此前图片1206/1nF/±10%/50V/X7R/50只仍单独登记，不抵扣0805/C0G需求；本轮50V规格确认不用于C_SN的1nF/100V/C0G/DNP预留。原理图和PCB原生文件、网络、脚号、设计值/封装及用量均未改；仅更新BOM已购状态，不需要本轮改板或新增逻辑器件。46采购行、120逻辑位号、104默认有料及先前三类已确认库存保持；仿真/固件未修改或运行。</t>
+          <t>比较6f26307：用户对另购1nF/50V/C0G（NP0）/0805数量回复“4”，登记库存4只。C_IL_ADC、C_IL_PROT单板各1只，共2只；需补购0只，预计装一板后余2只，尚未实际扣减库存。Excel库存填4、补购保留动态公式，CSV写当前4/0。图片中的1206/X7R/50只另记，不混入本项；本次50V备料不覆盖C_SN的100V/C0G/DNP预留。完整料号/容差待归档；采购46行、120逻辑位号/104默认有料及先前三类库存保持。原理图/PCB原生文件、网络、脚号、设计值/封装及单板用量未改，仅更新库存和补购记录，无新增器件或改板要求；仿真/固件未修改或运行。</t>
         </is>
       </c>
     </row>
     <row r="4" ht="46" customHeight="1">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>历史1nF图片核对（后续另购见最新项）</t>
+          <t>历史1nF另购确认（数量已后补）</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>比较8d57b27：用户新图已选规格为1206、1nF、±10%、50V、X7R，50只；无完整厂家型号。原理图C_IL_ADC/C_IL_PROT正常装配共2只，PCB均C0805，且C_IL_PROT明确C0G。这批1206/X7R不能视作0805/C0G可直接装配库存，50只不填入目标行库存。建议另备1nF/50V/C0G/0805共2只以统一备料；是否已有该款待核，不自动认定缺货2只。C_SN另为1nF/100V/C0G、DNP，本图也不能用于确认该项。原理图/PCB原生文件、网络、设计值和封装均未改；没有放大焊盘或放宽介质要求。仅更新实购物料记录及BOM待核状态，仿真/固件未修改或运行。</t>
+          <t>比较1dac34a：用户对是否另有1nF/50V/C0G（NP0）/0805回复“买了”，确认正常装配C_IL_ADC、C_IL_PROT所需C0G款已另购，每板共2只。实际数量、完整料号和容差未提供，库存/补购栏留空，不把设计需求2只当成库存。此前图片1206/1nF/±10%/50V/X7R/50只仍单独登记，不抵扣0805/C0G需求；本轮50V规格确认不用于C_SN的1nF/100V/C0G/DNP预留。原理图和PCB原生文件、网络、脚号、设计值/封装及用量均未改；仅更新BOM已购状态，不需要本轮改板或新增逻辑器件。46采购行、120逻辑位号、104默认有料及先前三类已确认库存保持；仿真/固件未修改或运行。</t>
         </is>
       </c>
     </row>
     <row r="5" ht="46" customHeight="1">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>版本基准</t>
+          <t>历史1nF图片核对（后续另购见最新项）</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>本次比较6f26307；1nF/50V/C0G/0805已购4只，单板用2只/补购0只/装一板余2只；仅更新库存，设计保持。</t>
+          <t>比较8d57b27：用户新图已选规格为1206、1nF、±10%、50V、X7R，50只；无完整厂家型号。原理图C_IL_ADC/C_IL_PROT正常装配共2只，PCB均C0805，且C_IL_PROT明确C0G。这批1206/X7R不能视作0805/C0G可直接装配库存，50只不填入目标行库存。建议另备1nF/50V/C0G/0805共2只以统一备料；是否已有该款待核，不自动认定缺货2只。C_SN另为1nF/100V/C0G、DNP，本图也不能用于确认该项。原理图/PCB原生文件、网络、设计值和封装均未改；没有放大焊盘或放宽介质要求。仅更新实购物料记录及BOM待核状态，仿真/固件未修改或运行。</t>
         </is>
       </c>
     </row>
     <row r="6" ht="46" customHeight="1">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>计数口径</t>
+          <t>版本基准</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>120个逻辑位号含14个裸测试点、2个DNP预留和1个外置R_PRE。120不等于需购买120个独立实体。</t>
+          <t>本次比较6f26307；1nF/50V/C0G/0805已购4只，单板用2只/补购0只/装一板余2只；仅更新库存，设计保持。</t>
         </is>
       </c>
     </row>
     <row r="7" ht="46" customHeight="1">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>默认装配</t>
+          <t>计数口径</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>120−14裸测试点−2个DNP=104个有料逻辑位号；含R_PRE外置电阻。管夹、模块、开关和线束另表计数。</t>
+          <t>120个逻辑位号含14个裸测试点、2个DNP预留和1个外置R_PRE。120不等于需购买120个独立实体。</t>
         </is>
       </c>
     </row>
     <row r="8" ht="46" customHeight="1">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>库存填写</t>
+          <t>默认装配</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>G列已填用户确认库存：100nF/X7R 50只、4.7nF/X7R 50只、4.7nF/C0G 2只、1nF/C0G 4只，四项单板补购均0。其他空白表示未知，不代表未购。</t>
+          <t>120−14裸测试点−2个DNP=104个有料逻辑位号；含R_PRE外置电阻。管夹、模块、开关和线束另表计数。</t>
         </is>
       </c>
     </row>
     <row r="9" ht="46" customHeight="1">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>DNP</t>
+          <t>库存填写</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>R_SN/C_SN各设计1个，默认装配0个；实测振铃后决定是否装配和调值。</t>
+          <t>G列已填用户确认库存：100nF/X7R 50只、4.7nF/X7R 50只、4.7nF/C0G 2只、1nF/C0G 4只，四项单板补购均0。其他空白表示未知，不代表未购。</t>
         </is>
       </c>
     </row>
     <row r="10" ht="46" customHeight="1">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>采购规格</t>
+          <t>DNP</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>标“建议/统一采购”的额定、精度或介质是采购建议，区别于源图原始标注；实际原始值在逐位号页保留。</t>
+          <t>R_SN/C_SN各设计1个，默认装配0个；实测振铃后决定是否装配和调值。</t>
         </is>
       </c>
     </row>
     <row r="11" ht="46" customHeight="1">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>普通/精密电阻功率</t>
+          <t>采购规格</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>除源图另有功率要求的R_BL/R_SN/R_PRE和分流器外，0805电阻统一≥0.125W是本表采购建议，不冒充源图已规定的功率。</t>
+          <t>标“建议/统一采购”的额定、精度或介质是采购建议，区别于源图原始标注；实际原始值在逐位号页保留。</t>
         </is>
       </c>
     </row>
     <row r="12" ht="46" customHeight="1">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>优先核对</t>
+          <t>普通/精密电阻功率</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>U1型号家族/直插类别已确认；保留IR2184PbF设计标注，不再列为型号封装待确认或默认补购；库存数量另填，IR2104不可代装。RS_L 25mΩ在B3清单中已包含，旧表记未购，现库存待核，不再自动假定库存为0。</t>
+          <t>除源图另有功率要求的R_BL/R_SN/R_PRE和分流器外，0805电阻统一≥0.125W是本表采购建议，不冒充源图已规定的功率。</t>
         </is>
       </c>
     </row>
     <row r="13" ht="46" customHeight="1">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>电容数量</t>
+          <t>优先核对</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>100nF共16只、4.7nF共5只、默认1nF共2只，另有1只DNP的1nF/100V。</t>
+          <t>U1型号家族/直插类别已确认；保留IR2184PbF设计标注，不再列为型号封装待确认或默认补购；库存数量另填，IR2104不可代装。RS_L 25mΩ在B3清单中已包含，旧表记未购，现库存待核，不再自动假定库存为0。</t>
         </is>
       </c>
     </row>
     <row r="14" ht="46" customHeight="1">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>料号纠错</t>
+          <t>电容数量</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>472批次已确认4.7nF；随后用户确认另外买了100nF/0805，两批分开记录。100nF/50V/0805/X7R已购50只，单板需求16只，补购0只，装配一板后余34只；完整料号/容差未提供；用户现已确认实际型号CL21B472JBANNNC，先前口头C0G由实际型号纠正为X7R；该款50V/±5%/0805按用户编码图明确。C_VINP_ADC所需的4.7nF/50V/C0G/0805另购状态已获确认；该批C0G库存2只、单板用1只/补购0只；C0G完整料号/容差待归档；CL21B472JBANNNC/X7R库存现已确认50只、单板用4只/补购0只，两类不混计。</t>
+          <t>100nF共16只、4.7nF共5只、默认1nF共2只，另有1只DNP的1nF/100V。</t>
         </is>
       </c>
     </row>
     <row r="15" ht="46" customHeight="1">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>分流器新证据</t>
+          <t>料号纠错</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>RS_IN/OUT：50mΩ P10、图示线径0.8、体高12、标称5A；RS_L：25mΩ P5、图示线径0.7、体高7。电阻体线径不自动证明焊接直脚径，精度/连续功率仍待核。</t>
+          <t>472批次已确认4.7nF；随后用户确认另外买了100nF/0805，两批分开记录。100nF/50V/0805/X7R已购50只，单板需求16只，补购0只，装配一板后余34只；完整料号/容差未提供；用户现已确认实际型号CL21B472JBANNNC，先前口头C0G由实际型号纠正为X7R；该款50V/±5%/0805按用户编码图明确。C_VINP_ADC所需的4.7nF/50V/C0G/0805另购状态已获确认；该批C0G库存2只、单板用1只/补购0只；C0G完整料号/容差待归档；CL21B472JBANNNC/X7R库存现已确认50只、单板用4只/补购0只，两类不混计。</t>
         </is>
       </c>
     </row>
     <row r="16" ht="46" customHeight="1">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>保险夹确认</t>
+          <t>分流器新证据</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>用户明确单夹脚中心距5.66mm；脚宽1.1/材料厚0.5。槽0.9×1.5及双夹中心距15mm是设计选择，装入5×20实物核对端帽接触/止挡后方可冻结；不能使用旧6×30/7.7尺寸。</t>
+          <t>RS_IN/OUT：50mΩ P10、图示线径0.8、体高12、标称5A；RS_L：25mΩ P5、图示线径0.7、体高7。电阻体线径不自动证明焊接直脚径，精度/连续功率仍待核。</t>
         </is>
       </c>
     </row>
     <row r="17" ht="46" customHeight="1">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>二极管确认</t>
+          <t>保险夹确认</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>两只SR560/SMB已由用户明确；沿用现有SMB标准几何，1=K/2=A。DO-201AD图不用于贴片建库，厂家完整电气手册/推荐焊盘最终复核仍需归档。</t>
+          <t>用户明确单夹脚中心距5.66mm；脚宽1.1/材料厚0.5。槽0.9×1.5及双夹中心距15mm是设计选择，装入5×20实物核对端帽接触/止挡后方可冻结；不能使用旧6×30/7.7尺寸。</t>
         </is>
       </c>
     </row>
     <row r="18" ht="46" customHeight="1">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>未确认封装</t>
+          <t>二极管确认</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>C_A3的0805类别已确认；F1组合试装、分流器完整包络及外壳固定仍待核。C_A3完整料号/介质/偏压有效容量、二极管厂家数据待最终复核。</t>
+          <t>两只SR560/SMB已由用户明确；沿用现有SMB标准几何，1=K/2=A。DO-201AD图不用于贴片建库，厂家完整电气手册/推荐焊盘最终复核仍需归档。</t>
         </is>
       </c>
     </row>
     <row r="19" ht="46" customHeight="1">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>电感</t>
+          <t>未确认封装</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>65125图示6A Max不是饱和电流保证；源设计仍要求Isat≥3A、Irms≥1.5A、DCR≤0.15Ω。</t>
+          <t>C_A3的0805类别已确认；F1组合试装、分流器完整包络及外壳固定仍待核。C_A3完整料号/介质/偏压有效容量、二极管厂家数据待最终复核。</t>
         </is>
       </c>
     </row>
     <row r="20" ht="46" customHeight="1">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>当前制造状态</t>
+          <t>电感</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>PCB仍有未布连接，客户端打开、原生ERC/DRC未完成；清单提供采购核对依据，不是制板放行。</t>
+          <t>65125图示6A Max不是饱和电流保证；源设计仍要求Isat≥3A、Irms≥1.5A、DCR≤0.15Ω。</t>
         </is>
       </c>
     </row>
     <row r="21" ht="46" customHeight="1">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>本次原理图影响</t>
+          <t>当前制造状态</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>相对6f26307，原理图和PCB原生文件未改，网络/脚号/设计值/封装与单板用量保持。</t>
+          <t>PCB仍有未布连接，客户端打开、原生ERC/DRC未完成；清单提供采购核对依据，不是制板放行。</t>
         </is>
       </c>
     </row>
     <row r="22" ht="46" customHeight="1">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>本次器件/PCB影响</t>
+          <t>本次原理图影响</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>1nF/50V/C0G/0805登记库存4只，单板用2只/补购0只，预计装一板余2只；1206/X7R款分开。完整料号/容差待归档，46采购行/120位号/104默认有料及既有三类库存保持，无新增或改板要求。</t>
+          <t>相对6f26307，原理图和PCB原生文件未改，网络/脚号/设计值/封装与单板用量保持。</t>
         </is>
       </c>
     </row>
     <row r="23" ht="46" customHeight="1">
       <c r="A23" s="2" t="inlineStr">
         <is>
+          <t>本次器件/PCB影响</t>
+        </is>
+      </c>
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t>1nF/50V/C0G/0805登记库存4只，单板用2只/补购0只，预计装一板余2只；1206/X7R款分开。完整料号/容差待归档，46采购行/120位号/104默认有料及既有三类库存保持，无新增或改板要求。</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="46" customHeight="1">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
           <t>本次仿真/固件影响</t>
         </is>
       </c>
-      <c r="B23" s="2" t="inlineStr">
+      <c r="B24" s="2" t="inlineStr">
         <is>
           <t>未修改或运行Multisim/ngspice/STM32固件，旧器件/功能等效模型未同步为SR560厂家模型，不证明新选型压降、温升、效率或保护实测通过。</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:B23"/>
+  <autoFilter ref="A1:B24"/>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" paperSize="8" fitToHeight="0" fitToWidth="1"/>
@@ -8625,7 +8637,7 @@
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>常开保持型SPST旁路开关，≥30VDC/≥3A</t>
+          <t>NKK MN11SS4W01；SPST ON-OFF保持型，4A/30VDC；面板安装焊片端子</t>
         </is>
       </c>
       <c r="D7" s="2" t="n">
@@ -8638,7 +8650,7 @@
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>与PCB端子分开计数；需明确直流额定，不能仅凭交流额定替代</t>
+          <t>用户提出替代MSS-22D18；本项按J_BYP外接旁路用途选型。两焊片分别接J_BYP.1 FUSED与J_BYP.2 IN_PRE，无极性；面板开孔Ø6.5mm、螺纹M6×0.75。不能直接插原六脚PCB孔，不能替代双刀/换向用途；实际旧开关接线和库存未确认；开关与PCB端子分开计数</t>
         </is>
       </c>
     </row>

</xml_diff>